<commit_message>
Update contacted status for next 5 outreach leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -2836,7 +2836,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C65" t="str">
         <v/>
@@ -2874,7 +2874,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C66" t="str">
         <v/>
@@ -2912,7 +2912,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C67" t="str">
         <v/>
@@ -2950,7 +2950,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C68" t="str">
         <v/>
@@ -2988,7 +2988,7 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C69" t="str">
         <v/>

</xml_diff>

<commit_message>
Mark next 5 WebKreatives leads contacted
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -3026,7 +3026,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C70" t="str">
         <v/>
@@ -3064,7 +3064,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C71" t="str">
         <v/>
@@ -3102,7 +3102,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C72" t="str">
         <v/>
@@ -3140,7 +3140,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C73" t="str">
         <v/>
@@ -3178,7 +3178,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C74" t="str">
         <v/>

</xml_diff>

<commit_message>
WebKreatives: mark next 5 leads contacted
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -3216,7 +3216,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C75" t="str">
         <v/>
@@ -3254,7 +3254,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C76" t="str">
         <v/>
@@ -3292,7 +3292,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C77" t="str">
         <v/>
@@ -3330,7 +3330,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C78" t="str">
         <v/>
@@ -3368,7 +3368,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C79" t="str">
         <v/>

</xml_diff>

<commit_message>
Mark next 5 WebKreatives outreach leads as contacted
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -3406,7 +3406,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C80" t="str">
         <v/>
@@ -3444,7 +3444,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C81" t="str">
         <v/>
@@ -3482,7 +3482,7 @@
         <v>81</v>
       </c>
       <c r="B82" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C82" t="str">
         <v/>
@@ -3520,7 +3520,7 @@
         <v>82</v>
       </c>
       <c r="B83" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C83" t="str">
         <v/>
@@ -3558,7 +3558,7 @@
         <v>83</v>
       </c>
       <c r="B84" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C84" t="str">
         <v/>
@@ -3596,7 +3596,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C85" t="str">
         <v/>
@@ -3634,7 +3634,7 @@
         <v>85</v>
       </c>
       <c r="B86" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C86" t="str">
         <v/>
@@ -3672,7 +3672,7 @@
         <v>86</v>
       </c>
       <c r="B87" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C87" t="str">
         <v/>
@@ -3710,7 +3710,7 @@
         <v>87</v>
       </c>
       <c r="B88" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C88" t="str">
         <v/>
@@ -3748,7 +3748,7 @@
         <v>88</v>
       </c>
       <c r="B89" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C89" t="str">
         <v/>
@@ -3786,7 +3786,7 @@
         <v>89</v>
       </c>
       <c r="B90" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C90" t="str">
         <v/>
@@ -3824,7 +3824,7 @@
         <v>90</v>
       </c>
       <c r="B91" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C91" t="str">
         <v/>
@@ -3862,7 +3862,7 @@
         <v>91</v>
       </c>
       <c r="B92" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C92" t="str">
         <v/>
@@ -3900,7 +3900,7 @@
         <v>92</v>
       </c>
       <c r="B93" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C93" t="str">
         <v/>
@@ -3938,7 +3938,7 @@
         <v>93</v>
       </c>
       <c r="B94" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C94" t="str">
         <v/>

</xml_diff>

<commit_message>
chore(leads): mark next outreach batch contacted
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -3976,7 +3976,7 @@
         <v>94</v>
       </c>
       <c r="B95" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C95" t="str">
         <v/>
@@ -4014,7 +4014,7 @@
         <v>95</v>
       </c>
       <c r="B96" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C96" t="str">
         <v/>
@@ -4052,7 +4052,7 @@
         <v>96</v>
       </c>
       <c r="B97" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C97" t="str">
         <v/>
@@ -4090,7 +4090,7 @@
         <v>97</v>
       </c>
       <c r="B98" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C98" t="str">
         <v/>
@@ -4128,7 +4128,7 @@
         <v>98</v>
       </c>
       <c r="B99" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C99" t="str">
         <v/>

</xml_diff>

<commit_message>
Add 10 kapsalon leads (rows 133-142)
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6575,6 +6575,546 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>fashionhairstylist.nl</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>info@fashionhairstylist.nl</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Lonneke van Dijk Fashion Hairstylist</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Soest</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>06-24555644</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>kapsalon-dehaanenkam.nl</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>info@kapsalon-dehaanenkam.nl</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Kapsalon De Haan &amp; Kam</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Leeuwarden</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>06-18227515</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>hairxclusive.nl</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>info@hairxclusive.nl</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>HairXclusive</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Nijkerk</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>033-2456842</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>ciscashairservice.nl</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>info@ciscashairservice.nl</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Cisca's Hairservice</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Bedum</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>06-49308795</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>haarwereld.nl</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>info@haarwereld.nl</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Haarwereld</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Nieuwleusen</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>0529-480503</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>cutandshine.nl</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>info@cutandshine.nl</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Cut &amp; Shine Professional Hairstyling</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Hillegom</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>0252-751861</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>kappersgevoel.nl</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>info@kappersgevoel.nl</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Kappersgevoel</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Malden</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>024-3881692</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>hair-plaza.nl</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>info@hair-plaza.nl</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Hair Plaza</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Hattem</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>038-4449310</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>glamourhair.nl</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>info@glamourhair.nl</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Glamour Hair</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Assen</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>0592-318585</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Not Yet</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>byyoel.nl</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>info@byyoel.nl</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>By Yoel</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Kapsalon</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Abcoude</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>0294-269452</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Small local salon</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: backup logo, leads update, and linkedin memory
- Add WebKreatives logo asset
- Update Leads.xlsx with latest outreach data
- Add linkedin.md memory file

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -4584,7 +4584,7 @@
         <v>109</v>
       </c>
       <c r="B111" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C111" t="str">
         <v>Yes</v>
@@ -4622,7 +4622,7 @@
         <v>110</v>
       </c>
       <c r="B112" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C112" t="str">
         <v>Yes</v>
@@ -4660,7 +4660,7 @@
         <v>111</v>
       </c>
       <c r="B113" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C113" t="str">
         <v>Yes</v>
@@ -4698,7 +4698,7 @@
         <v>112</v>
       </c>
       <c r="B114" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C114" t="str">
         <v>Yes</v>
@@ -4736,7 +4736,7 @@
         <v>113</v>
       </c>
       <c r="B115" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C115" t="str">
         <v>Yes</v>

</xml_diff>

<commit_message>
Update leads after outreach batch
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -5154,7 +5154,7 @@
         <v>125</v>
       </c>
       <c r="B126" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C126" t="str">
         <v>Yes</v>
@@ -5192,7 +5192,7 @@
         <v>126</v>
       </c>
       <c r="B127" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C127" t="str">
         <v>Yes</v>
@@ -5230,7 +5230,7 @@
         <v>127</v>
       </c>
       <c r="B128" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C128" t="str">
         <v>Yes</v>
@@ -5268,7 +5268,7 @@
         <v>128</v>
       </c>
       <c r="B129" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C129" t="str">
         <v>Yes</v>
@@ -5306,7 +5306,7 @@
         <v>129</v>
       </c>
       <c r="B130" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C130" t="str">
         <v>Yes</v>

</xml_diff>

<commit_message>
chore(leads): mark next 5 webkreatives outreach sends
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -5344,7 +5344,7 @@
         <v>130</v>
       </c>
       <c r="B131" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C131" t="str">
         <v>Yes</v>
@@ -5382,7 +5382,7 @@
         <v>131</v>
       </c>
       <c r="B132" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C132" t="str">
         <v>Yes</v>
@@ -5420,7 +5420,7 @@
         <v>132</v>
       </c>
       <c r="B133" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C133" t="str">
         <v>Yes</v>
@@ -5458,7 +5458,7 @@
         <v>133</v>
       </c>
       <c r="B134" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C134" t="str">
         <v>Yes</v>
@@ -5496,7 +5496,7 @@
         <v>134</v>
       </c>
       <c r="B135" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C135" t="str">
         <v>Yes</v>

</xml_diff>

<commit_message>
Add 20 new WebKreatives leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -1,14 +1,30 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
-  <sheets>
-    <sheet name="leads" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>SheetJS</Application>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>leads</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+</Properties>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance"/>
+</file>
+
+<file path=xl\metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
@@ -30,7 +46,7 @@
 </metadata>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
@@ -75,7 +91,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -395,9 +411,18 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
+  <sheets>
+    <sheet name="leads" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L164"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5853,7 +5878,7 @@
         <v>gladysinternationalhair@gmail.com</v>
       </c>
       <c r="G144" t="str">
-        <v>Gladys Internacional Hair🇩🇴</v>
+        <v>Gladys Internacional HairðŸ‡©ðŸ‡´</v>
       </c>
       <c r="H144" t="str">
         <v>Kapsalon</v>
@@ -5869,6 +5894,766 @@
       </c>
       <c r="L144" t="str">
         <v>Geen website | OSM id:2862569301 | Source: OpenStreetMap</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D145" t="str">
+        <v/>
+      </c>
+      <c r="E145" t="str">
+        <v>dijoschilderwerken.nl</v>
+      </c>
+      <c r="F145" t="str">
+        <v>info@dijoschilderwerken.nl</v>
+      </c>
+      <c r="G145" t="str">
+        <v>DiJo Schilderwerken</v>
+      </c>
+      <c r="H145" t="str">
+        <v>Painter</v>
+      </c>
+      <c r="I145" t="str">
+        <v/>
+      </c>
+      <c r="J145" t="str">
+        <v>Nijmegen, Gelderland</v>
+      </c>
+      <c r="K145" t="str">
+        <v>06-25237179</v>
+      </c>
+      <c r="L145" t="str">
+        <v>Active across Noord-Brabant</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D146" t="str">
+        <v/>
+      </c>
+      <c r="E146" t="str">
+        <v>schildersbedrijf-helmond.nl</v>
+      </c>
+      <c r="F146" t="str">
+        <v>info@anthonyvandinterschilderwerken.nl</v>
+      </c>
+      <c r="G146" t="str">
+        <v>Anthony van Dinter Schilderwerken</v>
+      </c>
+      <c r="H146" t="str">
+        <v>Painter</v>
+      </c>
+      <c r="I146" t="str">
+        <v/>
+      </c>
+      <c r="J146" t="str">
+        <v>Helmond, Noord-Brabant</v>
+      </c>
+      <c r="K146" t="str">
+        <v>0492-514304</v>
+      </c>
+      <c r="L146" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D147" t="str">
+        <v/>
+      </c>
+      <c r="E147" t="str">
+        <v>jaschilderwerken.nl</v>
+      </c>
+      <c r="F147" t="str">
+        <v>info@jaschilderwerken.nl</v>
+      </c>
+      <c r="G147" t="str">
+        <v>J.A. Schilderwerken</v>
+      </c>
+      <c r="H147" t="str">
+        <v>Painter</v>
+      </c>
+      <c r="I147" t="str">
+        <v/>
+      </c>
+      <c r="J147" t="str">
+        <v>Breda, Noord-Brabant</v>
+      </c>
+      <c r="K147" t="str">
+        <v>06-14604288</v>
+      </c>
+      <c r="L147" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C148" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D148" t="str">
+        <v/>
+      </c>
+      <c r="E148" t="str">
+        <v>riegner.nl</v>
+      </c>
+      <c r="F148" t="str">
+        <v>info@riegner.nl</v>
+      </c>
+      <c r="G148" t="str">
+        <v>Riegner Afwerk &amp; Renovatiebedrijf</v>
+      </c>
+      <c r="H148" t="str">
+        <v>Painter / Renovation</v>
+      </c>
+      <c r="I148" t="str">
+        <v/>
+      </c>
+      <c r="J148" t="str">
+        <v>Tilburg, Noord-Brabant</v>
+      </c>
+      <c r="K148" t="str">
+        <v>06-87234582</v>
+      </c>
+      <c r="L148" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C149" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D149" t="str">
+        <v/>
+      </c>
+      <c r="E149" t="str">
+        <v>frankvangameren.nl</v>
+      </c>
+      <c r="F149" t="str">
+        <v>info@frankvangameren.nl</v>
+      </c>
+      <c r="G149" t="str">
+        <v>Hoveniersbedrijf Frank van Gameren</v>
+      </c>
+      <c r="H149" t="str">
+        <v>Landscaper</v>
+      </c>
+      <c r="I149" t="str">
+        <v/>
+      </c>
+      <c r="J149" t="str">
+        <v>Enspijk, Gelderland</v>
+      </c>
+      <c r="K149" t="str">
+        <v>0345-682470</v>
+      </c>
+      <c r="L149" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D150" t="str">
+        <v/>
+      </c>
+      <c r="E150" t="str">
+        <v>hoveniersbedrijfteunaleven.nl</v>
+      </c>
+      <c r="F150" t="str">
+        <v>info@hoveniersbedrijfteunaleven.nl</v>
+      </c>
+      <c r="G150" t="str">
+        <v>Hoveniersbedrijf Teun Aleven</v>
+      </c>
+      <c r="H150" t="str">
+        <v>Landscaper</v>
+      </c>
+      <c r="I150" t="str">
+        <v/>
+      </c>
+      <c r="J150" t="str">
+        <v>Beek Gem. Montferland, Gelderland</v>
+      </c>
+      <c r="K150" t="str">
+        <v>06-30274350</v>
+      </c>
+      <c r="L150" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D151" t="str">
+        <v/>
+      </c>
+      <c r="E151" t="str">
+        <v>hoveniersbedrijfpolman.nl</v>
+      </c>
+      <c r="F151" t="str">
+        <v>info@hoveniersbedrijfpolman.nl</v>
+      </c>
+      <c r="G151" t="str">
+        <v>Hoveniersbedrijf Polman</v>
+      </c>
+      <c r="H151" t="str">
+        <v>Landscaper</v>
+      </c>
+      <c r="I151" t="str">
+        <v/>
+      </c>
+      <c r="J151" t="str">
+        <v>Hengelo, Gelderland</v>
+      </c>
+      <c r="K151" t="str">
+        <v>06-20239881</v>
+      </c>
+      <c r="L151" t="str">
+        <v>Kleinschalig bedrijf</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D152" t="str">
+        <v/>
+      </c>
+      <c r="E152" t="str">
+        <v>mbtimmerbedrijf.nl</v>
+      </c>
+      <c r="F152" t="str">
+        <v>contact@mbtimmerbedrijf.nl</v>
+      </c>
+      <c r="G152" t="str">
+        <v>Mensink &amp; Berends Timmerbedrijf</v>
+      </c>
+      <c r="H152" t="str">
+        <v>Timmerbedrijf</v>
+      </c>
+      <c r="I152" t="str">
+        <v/>
+      </c>
+      <c r="J152" t="str">
+        <v>Wijhe, Overijssel</v>
+      </c>
+      <c r="K152" t="str">
+        <v>06-28545592</v>
+      </c>
+      <c r="L152" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
+      <c r="E153" t="str">
+        <v>bouw-entimmerwerkenscholten.nl</v>
+      </c>
+      <c r="F153" t="str">
+        <v>bouw-entimmerwerkenscholten@outlook.com</v>
+      </c>
+      <c r="G153" t="str">
+        <v>Bouw en Timmerwerken Scholten</v>
+      </c>
+      <c r="H153" t="str">
+        <v>Construction / Carpentry</v>
+      </c>
+      <c r="I153" t="str">
+        <v/>
+      </c>
+      <c r="J153" t="str">
+        <v>Overijssel</v>
+      </c>
+      <c r="K153" t="str">
+        <v>06-17183181</v>
+      </c>
+      <c r="L153" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D154" t="str">
+        <v/>
+      </c>
+      <c r="E154" t="str">
+        <v>timmerfabriekwinters.nl</v>
+      </c>
+      <c r="F154" t="str">
+        <v>tifawinters@planet.nl</v>
+      </c>
+      <c r="G154" t="str">
+        <v>Timmerfabriek Winters</v>
+      </c>
+      <c r="H154" t="str">
+        <v>Timmerfabriek</v>
+      </c>
+      <c r="I154" t="str">
+        <v/>
+      </c>
+      <c r="J154" t="str">
+        <v>Steenwijkerwold, Overijssel</v>
+      </c>
+      <c r="K154" t="str">
+        <v>0521-588217</v>
+      </c>
+      <c r="L154" t="str">
+        <v>Familiebedrijf</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
+      <c r="E155" t="str">
+        <v>tonkerkhoffs.nl</v>
+      </c>
+      <c r="F155" t="str">
+        <v>info@ton-kerkhoffs.nl</v>
+      </c>
+      <c r="G155" t="str">
+        <v>Autobedrijf Ton Kerkhoffs</v>
+      </c>
+      <c r="H155" t="str">
+        <v>Autobedrijf</v>
+      </c>
+      <c r="I155" t="str">
+        <v/>
+      </c>
+      <c r="J155" t="str">
+        <v>Kelpen-Oler, Limburg</v>
+      </c>
+      <c r="K155" t="str">
+        <v>046-4744665</v>
+      </c>
+      <c r="L155" t="str">
+        <v>Familiebedrijf</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D156" t="str">
+        <v/>
+      </c>
+      <c r="E156" t="str">
+        <v>nancyjurgenauto.nl</v>
+      </c>
+      <c r="F156" t="str">
+        <v>info@nancyjurgenauto.nl</v>
+      </c>
+      <c r="G156" t="str">
+        <v>Nancy Jurgen Auto</v>
+      </c>
+      <c r="H156" t="str">
+        <v>Autobedrijf</v>
+      </c>
+      <c r="I156" t="str">
+        <v/>
+      </c>
+      <c r="J156" t="str">
+        <v>Geleen, Limburg</v>
+      </c>
+      <c r="K156" t="str">
+        <v>046-4583120</v>
+      </c>
+      <c r="L156" t="str">
+        <v>Mercedes specialist</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D157" t="str">
+        <v/>
+      </c>
+      <c r="E157" t="str">
+        <v>tdevriesstuc.nl</v>
+      </c>
+      <c r="F157" t="str">
+        <v>info@tdevriesstuc.nl</v>
+      </c>
+      <c r="G157" t="str">
+        <v>Stucadoorbedrijf T. de Vries</v>
+      </c>
+      <c r="H157" t="str">
+        <v>Stukadoor</v>
+      </c>
+      <c r="I157" t="str">
+        <v/>
+      </c>
+      <c r="J157" t="str">
+        <v>Joure, Friesland</v>
+      </c>
+      <c r="K157" t="str">
+        <v>0513-410628</v>
+      </c>
+      <c r="L157" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D158" t="str">
+        <v/>
+      </c>
+      <c r="E158" t="str">
+        <v>a7stukadoor.nl</v>
+      </c>
+      <c r="F158" t="str">
+        <v>info@a7stukadoor.nl</v>
+      </c>
+      <c r="G158" t="str">
+        <v>A7 Stuc- en Spackbedrijf Drachten</v>
+      </c>
+      <c r="H158" t="str">
+        <v>Stukadoor</v>
+      </c>
+      <c r="I158" t="str">
+        <v/>
+      </c>
+      <c r="J158" t="str">
+        <v>Drachten, Friesland</v>
+      </c>
+      <c r="K158" t="str">
+        <v>06-28491516</v>
+      </c>
+      <c r="L158" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C159" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
+      <c r="E159" t="str">
+        <v>kapsalongeorge.nl</v>
+      </c>
+      <c r="F159" t="str">
+        <v>kapsalongeorge@gmail.com</v>
+      </c>
+      <c r="G159" t="str">
+        <v>Kapsalon George</v>
+      </c>
+      <c r="H159" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I159" t="str">
+        <v/>
+      </c>
+      <c r="J159" t="str">
+        <v>Groningen</v>
+      </c>
+      <c r="K159" t="str">
+        <v>050-2304049</v>
+      </c>
+      <c r="L159" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C160" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
+      <c r="E160" t="str">
+        <v>newstyle-kapsalon.nl</v>
+      </c>
+      <c r="F160" t="str">
+        <v>info@newstyle-kapsalon.nl</v>
+      </c>
+      <c r="G160" t="str">
+        <v>New Style Kapsalon</v>
+      </c>
+      <c r="H160" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I160" t="str">
+        <v/>
+      </c>
+      <c r="J160" t="str">
+        <v>Groningen</v>
+      </c>
+      <c r="K160" t="str">
+        <v>0507851524</v>
+      </c>
+      <c r="L160" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
+      <c r="E161" t="str">
+        <v>tonvandenijssel.nl</v>
+      </c>
+      <c r="F161" t="str">
+        <v>info@tonvandenijssel.nl</v>
+      </c>
+      <c r="G161" t="str">
+        <v>Ton van den IJssel Tweewielers</v>
+      </c>
+      <c r="H161" t="str">
+        <v>Fietsenwinkel</v>
+      </c>
+      <c r="I161" t="str">
+        <v/>
+      </c>
+      <c r="J161" t="str">
+        <v>Utrecht</v>
+      </c>
+      <c r="K161" t="str">
+        <v>030-2932679</v>
+      </c>
+      <c r="L161" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D162" t="str">
+        <v/>
+      </c>
+      <c r="E162" t="str">
+        <v>030-fietsen.nl</v>
+      </c>
+      <c r="F162" t="str">
+        <v>info@030-fietsen.nl</v>
+      </c>
+      <c r="G162" t="str">
+        <v>030 Fietsen</v>
+      </c>
+      <c r="H162" t="str">
+        <v>Fietsenwinkel</v>
+      </c>
+      <c r="I162" t="str">
+        <v/>
+      </c>
+      <c r="J162" t="str">
+        <v>Utrecht</v>
+      </c>
+      <c r="K162" t="str">
+        <v>06-43485150</v>
+      </c>
+      <c r="L162" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C163" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
+      <c r="E163" t="str">
+        <v>kokfietsen.nl</v>
+      </c>
+      <c r="F163" t="str">
+        <v>info@kokfietsen.nl</v>
+      </c>
+      <c r="G163" t="str">
+        <v>Kok Fietsen</v>
+      </c>
+      <c r="H163" t="str">
+        <v>Fietsenwinkel</v>
+      </c>
+      <c r="I163" t="str">
+        <v/>
+      </c>
+      <c r="J163" t="str">
+        <v>Utrecht</v>
+      </c>
+      <c r="K163" t="str">
+        <v>030-2315780</v>
+      </c>
+      <c r="L163" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C164" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
+      <c r="E164" t="str">
+        <v>electrotechniekzwaan.nl</v>
+      </c>
+      <c r="F164" t="str">
+        <v>info@electrotechniekzwaan.nl</v>
+      </c>
+      <c r="G164" t="str">
+        <v>Electrotechniek Zwaan</v>
+      </c>
+      <c r="H164" t="str">
+        <v>Elektrotechniek</v>
+      </c>
+      <c r="I164" t="str">
+        <v/>
+      </c>
+      <c r="J164" t="str">
+        <v>Andijk, Noord-Holland</v>
+      </c>
+      <c r="K164" t="str">
+        <v>0228-850209</v>
+      </c>
+      <c r="L164" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Advance outreach leads after sending next 5 contacts
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -1,30 +1,14 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>SheetJS</Application>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>Worksheets</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>leads</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
+  <sheets>
+    <sheet name="leads" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance"/>
-</file>
-
-<file path=xl\metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
@@ -46,7 +30,7 @@
 </metadata>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
@@ -91,7 +75,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -411,16 +395,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
-  <sheets>
-    <sheet name="leads" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L164"/>
   <sheetData>
@@ -5559,7 +5534,7 @@
         <v>135</v>
       </c>
       <c r="B136" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C136" t="str">
         <v>Yes</v>
@@ -5597,7 +5572,7 @@
         <v>136</v>
       </c>
       <c r="B137" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C137" t="str">
         <v>Yes</v>
@@ -5635,7 +5610,7 @@
         <v>137</v>
       </c>
       <c r="B138" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C138" t="str">
         <v>Yes</v>
@@ -5673,7 +5648,7 @@
         <v>138</v>
       </c>
       <c r="B139" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C139" t="str">
         <v>Yes</v>
@@ -5711,7 +5686,7 @@
         <v>139</v>
       </c>
       <c r="B140" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C140" t="str">
         <v>Yes</v>
@@ -6658,7 +6633,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L144"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L164"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 new leads to Leads.xlsx
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L184"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6631,9 +6631,769 @@
         <v/>
       </c>
     </row>
+    <row r="165">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
+      <c r="E165" t="str">
+        <v>hoveniersbedrijfkoops.nl</v>
+      </c>
+      <c r="F165" t="str">
+        <v>info@hoveniersbedrijfkoops.nl</v>
+      </c>
+      <c r="G165" t="str">
+        <v>Hoveniersbedrijf Koops</v>
+      </c>
+      <c r="H165" t="str">
+        <v>Hovenier</v>
+      </c>
+      <c r="I165" t="str">
+        <v/>
+      </c>
+      <c r="J165" t="str">
+        <v>Oosterwolde, Friesland</v>
+      </c>
+      <c r="K165" t="str">
+        <v>0516-764766</v>
+      </c>
+      <c r="L165" t="str">
+        <v>Local hovenier; contact page surfaced via Tavily snippet</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
+      <c r="E166" t="str">
+        <v>hoveniersbedrijfstevens.nl</v>
+      </c>
+      <c r="F166" t="str">
+        <v>info@hoveniersbedrijfstevens.nl</v>
+      </c>
+      <c r="G166" t="str">
+        <v>Hoveniersbedrijf Stevens</v>
+      </c>
+      <c r="H166" t="str">
+        <v>Hovenier</v>
+      </c>
+      <c r="I166" t="str">
+        <v/>
+      </c>
+      <c r="J166" t="str">
+        <v>Tiendeveen, Drenthe</v>
+      </c>
+      <c r="K166" t="str">
+        <v>0528-741040</v>
+      </c>
+      <c r="L166" t="str">
+        <v>Local hovenier; dated/simple contact-page style</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C167" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D167" t="str">
+        <v/>
+      </c>
+      <c r="E167" t="str">
+        <v>hoveniersbedrijfhendrickx.nl</v>
+      </c>
+      <c r="F167" t="str">
+        <v>info@hoveniersbedrijfhendrickx.nl</v>
+      </c>
+      <c r="G167" t="str">
+        <v>Hoveniersbedrijf Hendrickx</v>
+      </c>
+      <c r="H167" t="str">
+        <v>Hovenier</v>
+      </c>
+      <c r="I167" t="str">
+        <v/>
+      </c>
+      <c r="J167" t="str">
+        <v>Espel, Flevoland</v>
+      </c>
+      <c r="K167" t="str">
+        <v>0527-271088</v>
+      </c>
+      <c r="L167" t="str">
+        <v>Small regional hovenier</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D168" t="str">
+        <v/>
+      </c>
+      <c r="E168" t="str">
+        <v>hoveniersbedrijfeikenhorst.nl</v>
+      </c>
+      <c r="F168" t="str">
+        <v>info@hoveniersbedrijfeikenhorst.nl</v>
+      </c>
+      <c r="G168" t="str">
+        <v>Hoveniersbedrijf Eikenhorst</v>
+      </c>
+      <c r="H168" t="str">
+        <v>Hovenier</v>
+      </c>
+      <c r="I168" t="str">
+        <v/>
+      </c>
+      <c r="J168" t="str">
+        <v>Bleiswijk, Zuid-Holland</v>
+      </c>
+      <c r="K168" t="str">
+        <v>06-27485601</v>
+      </c>
+      <c r="L168" t="str">
+        <v>Small regional hovenier</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D169" t="str">
+        <v/>
+      </c>
+      <c r="E169" t="str">
+        <v>hoveniersbedrijfgoes.nl</v>
+      </c>
+      <c r="F169" t="str">
+        <v>info@hoveniersbedrijfgoes.nl</v>
+      </c>
+      <c r="G169" t="str">
+        <v>Hoveniersbedrijf Goes</v>
+      </c>
+      <c r="H169" t="str">
+        <v>Hovenier</v>
+      </c>
+      <c r="I169" t="str">
+        <v/>
+      </c>
+      <c r="J169" t="str">
+        <v>Haarlem region, Noord-Holland</v>
+      </c>
+      <c r="K169" t="str">
+        <v>06-15836080</v>
+      </c>
+      <c r="L169" t="str">
+        <v>Local hovenier active around Haarlem/Heemstede/Bloemendaal</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D170" t="str">
+        <v/>
+      </c>
+      <c r="E170" t="str">
+        <v>hoveniersbedrijfderooij.nl</v>
+      </c>
+      <c r="F170" t="str">
+        <v>info@hoveniersbedrijfderooij.nl</v>
+      </c>
+      <c r="G170" t="str">
+        <v>Hoveniersbedrijf de Rooij</v>
+      </c>
+      <c r="H170" t="str">
+        <v>Hovenier</v>
+      </c>
+      <c r="I170" t="str">
+        <v/>
+      </c>
+      <c r="J170" t="str">
+        <v>Hillegom, Zuid-Holland</v>
+      </c>
+      <c r="K170" t="str">
+        <v>0252-684923</v>
+      </c>
+      <c r="L170" t="str">
+        <v>Local hovenier; contact page mentions Bollenstreek coverage</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D171" t="str">
+        <v/>
+      </c>
+      <c r="E171" t="str">
+        <v>kapsalonprinsheerlijk.nl</v>
+      </c>
+      <c r="F171" t="str">
+        <v>info@kapsalonprinsheerlijk.nl</v>
+      </c>
+      <c r="G171" t="str">
+        <v>Kapsalon Prinsheerlijk</v>
+      </c>
+      <c r="H171" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I171" t="str">
+        <v/>
+      </c>
+      <c r="J171" t="str">
+        <v>Amsterdam, Noord-Holland</v>
+      </c>
+      <c r="K171" t="str">
+        <v>0206251666</v>
+      </c>
+      <c r="L171" t="str">
+        <v>Salon; email/address on contact page</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
+      <c r="E172" t="str">
+        <v>kapsalondeniz.nl</v>
+      </c>
+      <c r="F172" t="str">
+        <v>info@kapsalondeniz.nl</v>
+      </c>
+      <c r="G172" t="str">
+        <v>Kapsalon Deniz</v>
+      </c>
+      <c r="H172" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I172" t="str">
+        <v/>
+      </c>
+      <c r="J172" t="str">
+        <v>Ermelo, Gelderland</v>
+      </c>
+      <c r="K172" t="str">
+        <v>0341-795122</v>
+      </c>
+      <c r="L172" t="str">
+        <v>Local kapsalon</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D173" t="str">
+        <v/>
+      </c>
+      <c r="E173" t="str">
+        <v>mariaskapsalon.nl</v>
+      </c>
+      <c r="F173" t="str">
+        <v>info@mariaskapsalon.nl</v>
+      </c>
+      <c r="G173" t="str">
+        <v>Maria's Kapsalon</v>
+      </c>
+      <c r="H173" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I173" t="str">
+        <v/>
+      </c>
+      <c r="J173" t="str">
+        <v>Maastricht, Limburg</v>
+      </c>
+      <c r="K173" t="str">
+        <v>06-48218493</v>
+      </c>
+      <c r="L173" t="str">
+        <v>Local salon in Maastricht</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D174" t="str">
+        <v/>
+      </c>
+      <c r="E174" t="str">
+        <v>de-kapsalon.nl</v>
+      </c>
+      <c r="F174" t="str">
+        <v>info@de-kapsalon.nl</v>
+      </c>
+      <c r="G174" t="str">
+        <v>De Kapsalon</v>
+      </c>
+      <c r="H174" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I174" t="str">
+        <v/>
+      </c>
+      <c r="J174" t="str">
+        <v>Udenhout, Noord-Brabant</v>
+      </c>
+      <c r="K174" t="str">
+        <v>06-86654941</v>
+      </c>
+      <c r="L174" t="str">
+        <v>Simple Hostnet site</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D175" t="str">
+        <v/>
+      </c>
+      <c r="E175" t="str">
+        <v>kapsalonswitch.nl</v>
+      </c>
+      <c r="F175" t="str">
+        <v>info@kapsalonswitch.nl</v>
+      </c>
+      <c r="G175" t="str">
+        <v>Kapsalon Switch</v>
+      </c>
+      <c r="H175" t="str">
+        <v>Kapsalon</v>
+      </c>
+      <c r="I175" t="str">
+        <v/>
+      </c>
+      <c r="J175" t="str">
+        <v>Nederweert, Limburg</v>
+      </c>
+      <c r="K175" t="str">
+        <v>0495-632903</v>
+      </c>
+      <c r="L175" t="str">
+        <v>Local kapsalon</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D176" t="str">
+        <v/>
+      </c>
+      <c r="E176" t="str">
+        <v>de-bloemenwinkel.nl</v>
+      </c>
+      <c r="F176" t="str">
+        <v>info@de-bloemenwinkel.nl</v>
+      </c>
+      <c r="G176" t="str">
+        <v>De Bloemenwinkel</v>
+      </c>
+      <c r="H176" t="str">
+        <v>Bloemist</v>
+      </c>
+      <c r="I176" t="str">
+        <v/>
+      </c>
+      <c r="J176" t="str">
+        <v>Rijen, Noord-Brabant</v>
+      </c>
+      <c r="K176" t="str">
+        <v>0161-778593</v>
+      </c>
+      <c r="L176" t="str">
+        <v>Small bloemenwinkel; contact page very lightweight</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
+      <c r="E177" t="str">
+        <v>bloemist-apeldoorn.nl</v>
+      </c>
+      <c r="F177" t="str">
+        <v>info@bloemist-apeldoorn.nl</v>
+      </c>
+      <c r="G177" t="str">
+        <v>De Bloemenwinkel by Marilene</v>
+      </c>
+      <c r="H177" t="str">
+        <v>Bloemist</v>
+      </c>
+      <c r="I177" t="str">
+        <v/>
+      </c>
+      <c r="J177" t="str">
+        <v>Apeldoorn, Gelderland</v>
+      </c>
+      <c r="K177" t="str">
+        <v>055-5768012</v>
+      </c>
+      <c r="L177" t="str">
+        <v>Independent florist with Ugchelen location too</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D178" t="str">
+        <v/>
+      </c>
+      <c r="E178" t="str">
+        <v>bloemenhuispietersen.nl</v>
+      </c>
+      <c r="F178" t="str">
+        <v>info@bloemenhuispietersen.nl</v>
+      </c>
+      <c r="G178" t="str">
+        <v>Bloemenhuis Pietersen</v>
+      </c>
+      <c r="H178" t="str">
+        <v>Bloemist</v>
+      </c>
+      <c r="I178" t="str">
+        <v/>
+      </c>
+      <c r="J178" t="str">
+        <v>Noorden, Zuid-Holland</v>
+      </c>
+      <c r="K178" t="str">
+        <v>0172-408530</v>
+      </c>
+      <c r="L178" t="str">
+        <v>Independent florist</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D179" t="str">
+        <v/>
+      </c>
+      <c r="E179" t="str">
+        <v>myosotisbloemen.nl</v>
+      </c>
+      <c r="F179" t="str">
+        <v>info@myosotisbloemen.nl</v>
+      </c>
+      <c r="G179" t="str">
+        <v>Myosotis Bloemen</v>
+      </c>
+      <c r="H179" t="str">
+        <v>Bloemist</v>
+      </c>
+      <c r="I179" t="str">
+        <v/>
+      </c>
+      <c r="J179" t="str">
+        <v>Rhoon, Zuid-Holland</v>
+      </c>
+      <c r="K179" t="str">
+        <v>010-5015969</v>
+      </c>
+      <c r="L179" t="str">
+        <v>Local florist</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D180" t="str">
+        <v/>
+      </c>
+      <c r="E180" t="str">
+        <v>garageremko.nl</v>
+      </c>
+      <c r="F180" t="str">
+        <v>info@garageremko.nl</v>
+      </c>
+      <c r="G180" t="str">
+        <v>Garage Remko</v>
+      </c>
+      <c r="H180" t="str">
+        <v>Autobedrijf / Garage</v>
+      </c>
+      <c r="I180" t="str">
+        <v/>
+      </c>
+      <c r="J180" t="str">
+        <v>Eindhoven, Noord-Brabant</v>
+      </c>
+      <c r="K180" t="str">
+        <v>040-2904494</v>
+      </c>
+      <c r="L180" t="str">
+        <v>Independent garage; simple older-style site</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D181" t="str">
+        <v/>
+      </c>
+      <c r="E181" t="str">
+        <v>autobedrijfsips.nl</v>
+      </c>
+      <c r="F181" t="str">
+        <v>info@autobedrijfsips.nl</v>
+      </c>
+      <c r="G181" t="str">
+        <v>Autobedrijf Sips</v>
+      </c>
+      <c r="H181" t="str">
+        <v>Autobedrijf</v>
+      </c>
+      <c r="I181" t="str">
+        <v/>
+      </c>
+      <c r="J181" t="str">
+        <v>Rijen, Noord-Brabant</v>
+      </c>
+      <c r="K181" t="str">
+        <v>0657537131</v>
+      </c>
+      <c r="L181" t="str">
+        <v>Independent autobedrijf since 2011</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D182" t="str">
+        <v/>
+      </c>
+      <c r="E182" t="str">
+        <v>autobedrijfsnelbv.nl</v>
+      </c>
+      <c r="F182" t="str">
+        <v>info@autobedrijfsnelbv.nl</v>
+      </c>
+      <c r="G182" t="str">
+        <v>Autobedrijf Snel B.V.</v>
+      </c>
+      <c r="H182" t="str">
+        <v>Autobedrijf</v>
+      </c>
+      <c r="I182" t="str">
+        <v/>
+      </c>
+      <c r="J182" t="str">
+        <v>Nederhorst den Berg, Noord-Holland</v>
+      </c>
+      <c r="K182" t="str">
+        <v>0294-251600</v>
+      </c>
+      <c r="L182" t="str">
+        <v>Independent autobedrijf</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D183" t="str">
+        <v/>
+      </c>
+      <c r="E183" t="str">
+        <v>autobedrijf-debruin.nl</v>
+      </c>
+      <c r="F183" t="str">
+        <v>info@autobedrijf-debruin.nl</v>
+      </c>
+      <c r="G183" t="str">
+        <v>Autobedrijf de Bruin</v>
+      </c>
+      <c r="H183" t="str">
+        <v>Autobedrijf</v>
+      </c>
+      <c r="I183" t="str">
+        <v/>
+      </c>
+      <c r="J183" t="str">
+        <v>Dordrecht, Zuid-Holland</v>
+      </c>
+      <c r="K183" t="str">
+        <v>0786160211</v>
+      </c>
+      <c r="L183" t="str">
+        <v>Independent autobedrijf</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="str">
+        <v>Not Yet</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Weak</v>
+      </c>
+      <c r="D184" t="str">
+        <v/>
+      </c>
+      <c r="E184" t="str">
+        <v>apvanbeek.nl</v>
+      </c>
+      <c r="F184" t="str">
+        <v>info@apvanbeek.nl</v>
+      </c>
+      <c r="G184" t="str">
+        <v>Autobedrijf Ap van Beek</v>
+      </c>
+      <c r="H184" t="str">
+        <v>Autobedrijf</v>
+      </c>
+      <c r="I184" t="str">
+        <v/>
+      </c>
+      <c r="J184" t="str">
+        <v>Apeldoorn, Gelderland</v>
+      </c>
+      <c r="K184" t="str">
+        <v>055-3034272</v>
+      </c>
+      <c r="L184" t="str">
+        <v>Independent autobedrijf</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L164"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L184"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(leads): advance webkreatives outreach batch
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -5724,7 +5724,7 @@
         <v>140</v>
       </c>
       <c r="B141" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C141" t="str">
         <v>Yes</v>
@@ -5762,7 +5762,7 @@
         <v>141</v>
       </c>
       <c r="B142" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C142" t="str">
         <v>Yes</v>
@@ -5800,7 +5800,7 @@
         <v>142</v>
       </c>
       <c r="B143" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C143" t="str">
         <v>Yes</v>
@@ -5838,7 +5838,7 @@
         <v>143</v>
       </c>
       <c r="B144" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C144" t="str">
         <v>No</v>
@@ -5876,7 +5876,7 @@
         <v>144</v>
       </c>
       <c r="B145" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C145" t="str">
         <v>Weak</v>

</xml_diff>

<commit_message>
Add 40 new WebKreatives OSM leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3711" uniqueCount="2212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4239" uniqueCount="2400">
   <si>
     <t>#</t>
   </si>
@@ -6647,6 +6647,570 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:11034305313 | Source: OpenStreetMap | klussenbedrijf | Utrecht | Website: https://deschrijn.nl</t>
+  </si>
+  <si>
+    <t>info@catalados.nl</t>
+  </si>
+  <si>
+    <t>Catalados</t>
+  </si>
+  <si>
+    <t>Smedestraat 2011RE</t>
+  </si>
+  <si>
+    <t>+31 23 551 74 60</t>
+  </si>
+  <si>
+    <t>Geen website | Email from OSM | OSM id:2709744387 | Source: OpenStreetMap | kapsalon | Haarlem</t>
+  </si>
+  <si>
+    <t>info@stomerijapeldoorn.nl</t>
+  </si>
+  <si>
+    <t>Mondial Express</t>
+  </si>
+  <si>
+    <t>Koninginnelaan 7315BP</t>
+  </si>
+  <si>
+    <t>+31 55 521 7461</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2686309210 | Source: OpenStreetMap | stomerij | Apeldoorn | Website: http://www.mondialexpress.nl</t>
+  </si>
+  <si>
+    <t>info@stomerij-hofstraat.nl</t>
+  </si>
+  <si>
+    <t>Stomerij Hofstraat</t>
+  </si>
+  <si>
+    <t>Hofstraat 7311KV</t>
+  </si>
+  <si>
+    <t>+31 55 521 2875</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2687033800 | Source: OpenStreetMap | stomerij | Apeldoorn | Website: https://www.stomerij-hofstraat.nl</t>
+  </si>
+  <si>
+    <t>info@animodierenspeciaalzaak.nl</t>
+  </si>
+  <si>
+    <t>Discus Animo</t>
+  </si>
+  <si>
+    <t>Gasthuisring 5041DT</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2850941568 | Source: OpenStreetMap | dierenwinkel | Tilburg | Website: https://www.discus.nl/dierenwinkel/tilburg</t>
+  </si>
+  <si>
+    <t>tilburg@animalcenter.nl</t>
+  </si>
+  <si>
+    <t>Animal Center</t>
+  </si>
+  <si>
+    <t>Rugdijk 5011XA</t>
+  </si>
+  <si>
+    <t>+31 13 782 0921</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:11125558356 | Source: OpenStreetMap | dierenwinkel | Tilburg | Website: https://www.animalcenter.nl/animal-center-tilburg</t>
+  </si>
+  <si>
+    <t>info@sohokappers.nl</t>
+  </si>
+  <si>
+    <t>Soho</t>
+  </si>
+  <si>
+    <t>Kleine Houtstraat 2011DH</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:528922626 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://sohokappers.nl</t>
+  </si>
+  <si>
+    <t>haarlem@kinki.nl</t>
+  </si>
+  <si>
+    <t>Kinki</t>
+  </si>
+  <si>
+    <t>Kleine Houtstraat 2011DD</t>
+  </si>
+  <si>
+    <t>+31 23 551 3221</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:528922660 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.kinki.nl/salons/haarlem</t>
+  </si>
+  <si>
+    <t>info@conforzakappers.nl</t>
+  </si>
+  <si>
+    <t>Conforza</t>
+  </si>
+  <si>
+    <t>Schouwtjeslaan 2012KG</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1154644552 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.conforzakappers.nl</t>
+  </si>
+  <si>
+    <t>info@pierot.nl</t>
+  </si>
+  <si>
+    <t>Pierôt</t>
+  </si>
+  <si>
+    <t>Houtplein</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1213144323 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.pierot.nl</t>
+  </si>
+  <si>
+    <t>info@hairlemkappers.nl</t>
+  </si>
+  <si>
+    <t>Hairlem Kappers</t>
+  </si>
+  <si>
+    <t>Zijlweg 2013DJ</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1222784209 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://hairlemkappers.nl</t>
+  </si>
+  <si>
+    <t>jan@meesterbarbier.nl</t>
+  </si>
+  <si>
+    <t>Barbier</t>
+  </si>
+  <si>
+    <t>Spaarnwouderstraat 2011AE</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1413730866 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://janheidemanmeesterbarbier.nl</t>
+  </si>
+  <si>
+    <t>haarlem@toniandguy.nl</t>
+  </si>
+  <si>
+    <t>Toni &amp; Guy</t>
+  </si>
+  <si>
+    <t>Anegang 2011HS</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2272308048 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.toniandguy.nl/salon/haarlem</t>
+  </si>
+  <si>
+    <t>info@stylisimo.nl</t>
+  </si>
+  <si>
+    <t>Stylisimo</t>
+  </si>
+  <si>
+    <t>Spaarnwouderstraat 2011AH</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2708485436 | Source: OpenStreetMap | kapsalon | Haarlem | Website: http://www.stylisimo.nl</t>
+  </si>
+  <si>
+    <t>info@barbershophaarlem.nl</t>
+  </si>
+  <si>
+    <t>Barbershop Haarlem</t>
+  </si>
+  <si>
+    <t>Amsterdamstraat 2032PS</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2708555572 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://barbershophaarlem.nl</t>
+  </si>
+  <si>
+    <t>info@avangihair.nl</t>
+  </si>
+  <si>
+    <t>Avangi</t>
+  </si>
+  <si>
+    <t>Kleine Houtstraat 2011DE</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2708637045 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.avangihair.nl</t>
+  </si>
+  <si>
+    <t>info@addicthaarlem.nl</t>
+  </si>
+  <si>
+    <t>Addict Haarlem</t>
+  </si>
+  <si>
+    <t>Gedempte Oude Gracht 2011GN</t>
+  </si>
+  <si>
+    <t>+31 6 14 55 60 51</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2708637501 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.addicthaarlem.nl</t>
+  </si>
+  <si>
+    <t>info@nardihairdesign.nl</t>
+  </si>
+  <si>
+    <t>Nardi Hairdesign</t>
+  </si>
+  <si>
+    <t>+31 23 200 27 44</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2708637507 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://nardihairdesign.nl</t>
+  </si>
+  <si>
+    <t>thewayhaarlem@outlook.com</t>
+  </si>
+  <si>
+    <t>The Way Beauty Center</t>
+  </si>
+  <si>
+    <t>Kleine Houtstraat 2011DS</t>
+  </si>
+  <si>
+    <t>+31 23 532 13 32</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2709387048 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.thewaycurlsandcoils.com</t>
+  </si>
+  <si>
+    <t>info@thehairatelier.nl</t>
+  </si>
+  <si>
+    <t>The Hair Atelier</t>
+  </si>
+  <si>
+    <t>Gasthuisvest 2011ET</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2709387144 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://thehairatelier.nl</t>
+  </si>
+  <si>
+    <t>info@kapsalon-papillotte.nl</t>
+  </si>
+  <si>
+    <t>Papillotte</t>
+  </si>
+  <si>
+    <t>Klein Heiligland 2011ED</t>
+  </si>
+  <si>
+    <t>+31 23 534 17 17</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2709387645 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://kapsalon-papillotte.nl</t>
+  </si>
+  <si>
+    <t>alkmaar@robpeetoom.nl</t>
+  </si>
+  <si>
+    <t>Rob Peetoom</t>
+  </si>
+  <si>
+    <t>Zijlstraat 2011TR</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2709466457 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.robpeetoom.nl</t>
+  </si>
+  <si>
+    <t>info@salon54.nl</t>
+  </si>
+  <si>
+    <t>Salon 45</t>
+  </si>
+  <si>
+    <t>Pieter Kiesstraat 2013BJ</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2710737677 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.salon54.nl</t>
+  </si>
+  <si>
+    <t>info@billyholliday.nl</t>
+  </si>
+  <si>
+    <t>Billy Holliday</t>
+  </si>
+  <si>
+    <t>Botermarkt 2011XM</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2711299303 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.billyholliday.nl</t>
+  </si>
+  <si>
+    <t>info@schultheis.nl</t>
+  </si>
+  <si>
+    <t>Schultheis Coiffures</t>
+  </si>
+  <si>
+    <t>+31 23 531 2461</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2711299320 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://schultheis.nl</t>
+  </si>
+  <si>
+    <t>barbershop@maddaddys.nl</t>
+  </si>
+  <si>
+    <t>Mad Daddy's Barbershop</t>
+  </si>
+  <si>
+    <t>Doelstraat 2011XB</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2711301274 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://www.maddaddys.nl</t>
+  </si>
+  <si>
+    <t>wilsonsbarbershopinhaarlem@gmail.com</t>
+  </si>
+  <si>
+    <t>Wilson's Barbershop</t>
+  </si>
+  <si>
+    <t>Rustenburgerlaan 2012AL</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2711716793 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://wilsonsbarbershop.nl</t>
+  </si>
+  <si>
+    <t>info@centrumschalkwijk.nl</t>
+  </si>
+  <si>
+    <t>HairSalon SixtyOne</t>
+  </si>
+  <si>
+    <t>Mentonpassage 2037AB</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2714756526 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://centrumschalkwijk.nl/ondernemers/hairsalon-sixtyone</t>
+  </si>
+  <si>
+    <t>dortmundt@planet.nl</t>
+  </si>
+  <si>
+    <t>Hart en Ziel Kappers</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2714805678 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://hartenzielkappers.nl</t>
+  </si>
+  <si>
+    <t>info@patriciahairfashion.nl</t>
+  </si>
+  <si>
+    <t>Patricia's Hairfashion</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2714806304 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://patriciahairfashion.nl</t>
+  </si>
+  <si>
+    <t>adm@haarlemsebarbier.nl</t>
+  </si>
+  <si>
+    <t>Haarlemse Barbier</t>
+  </si>
+  <si>
+    <t>Generaal Cronjéstraat 2021JM</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2715764370 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://haarlemse-barbier.mytreatwell.nl</t>
+  </si>
+  <si>
+    <t>zalaszalon@gmail.com</t>
+  </si>
+  <si>
+    <t>Zzalon</t>
+  </si>
+  <si>
+    <t>Schoterweg 2021HM</t>
+  </si>
+  <si>
+    <t>+31 23 525 2265</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2715836091 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://zzalon.com</t>
+  </si>
+  <si>
+    <t>knipinnhaarlem@hotmail.com</t>
+  </si>
+  <si>
+    <t>Knip Inn</t>
+  </si>
+  <si>
+    <t>Rijksstraatweg 2024DD</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2715963295 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://knipinn-haarlem.weebly.com</t>
+  </si>
+  <si>
+    <t>kapsalonmegastar@gmail.com</t>
+  </si>
+  <si>
+    <t>Megastar</t>
+  </si>
+  <si>
+    <t>Rijksstraatweg 2024DA</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2715964620 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://kapsalonmegastar.nl</t>
+  </si>
+  <si>
+    <t>info@barberara.nl</t>
+  </si>
+  <si>
+    <t>Barber Ara</t>
+  </si>
+  <si>
+    <t>Rijksstraatweg 2022DG</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2716162585 | Source: OpenStreetMap | kapsalon | Haarlem | Website: https://barberara.nl</t>
+  </si>
+  <si>
+    <t>info@salubriousbeautysalon.nl</t>
+  </si>
+  <si>
+    <t>Salubrious</t>
+  </si>
+  <si>
+    <t>Johan Huizingalaan 1065JM</t>
+  </si>
+  <si>
+    <t>+31 6 52632229</t>
+  </si>
+  <si>
+    <t>Geen website | Email from OSM | OSM id:1768618445 | Source: OpenStreetMap | schoonheidssalon | Amsterdam</t>
+  </si>
+  <si>
+    <t>crystalnails.nl@gmail.com</t>
+  </si>
+  <si>
+    <t>Crystal Nails</t>
+  </si>
+  <si>
+    <t>Ceintuurbaan 1072ES</t>
+  </si>
+  <si>
+    <t>+31 20 6752588</t>
+  </si>
+  <si>
+    <t>Geen website | Email from OSM | OSM id:2817611754 | Source: OpenStreetMap | schoonheidssalon | Amsterdam</t>
+  </si>
+  <si>
+    <t>info@artistlab.nl</t>
+  </si>
+  <si>
+    <t>Artist Lab</t>
+  </si>
+  <si>
+    <t>Sarphatipark 1072PB</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:257518672 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://artistlab.nl</t>
+  </si>
+  <si>
+    <t>info@asepsis.nl</t>
+  </si>
+  <si>
+    <t>Asepsis</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:332692571 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://asepsis.nl</t>
+  </si>
+  <si>
+    <t>mail@thebrowbarber.com</t>
+  </si>
+  <si>
+    <t>The Browbarber</t>
+  </si>
+  <si>
+    <t>Westerstraat 1015ML</t>
+  </si>
+  <si>
+    <t>+31 6 41270047</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1497842621 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://www.thebrowbarber.com</t>
+  </si>
+  <si>
+    <t>info@beauty-me.nl</t>
+  </si>
+  <si>
+    <t>Beauty-ME</t>
+  </si>
+  <si>
+    <t>Koningsstraat 1011ES</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2725746969 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://beauty-me.nl</t>
+  </si>
+  <si>
+    <t>info@americanfitness.nl</t>
+  </si>
+  <si>
+    <t>American Fitness</t>
+  </si>
+  <si>
+    <t>Blasiusstraat 1091CZ</t>
+  </si>
+  <si>
+    <t>+31 20 694 1358;+31 6 51905823</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2522585265 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://americanfitness.nl</t>
+  </si>
+  <si>
+    <t>service@rituals.com</t>
+  </si>
+  <si>
+    <t>House of Rituals</t>
+  </si>
+  <si>
+    <t>Spui 1012WZ</t>
+  </si>
+  <si>
+    <t>+31 20 705 5180</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2724000369 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://www.rituals.com/en-nl/house-of-rituals.html</t>
+  </si>
+  <si>
+    <t>sophie-vlaming-@wwmodels.nl</t>
+  </si>
+  <si>
+    <t>Mogeen</t>
+  </si>
+  <si>
+    <t>Vijzelgracht 1017HN</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2737956995 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://mogeen.nl</t>
+  </si>
+  <si>
+    <t>smile@deninie.nl</t>
+  </si>
+  <si>
+    <t>Deninie</t>
+  </si>
+  <si>
+    <t>Vijzelgracht 1017HP</t>
+  </si>
+  <si>
+    <t>+31 6 45024568</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2737962124 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://deninie.nl</t>
   </si>
 </sst>
 </file>
@@ -7023,7 +7587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L413"/>
+  <dimension ref="A1:L461"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -20199,6 +20763,1830 @@
         <v>2211</v>
       </c>
     </row>
+    <row r="414" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A414">
+        <v>408</v>
+      </c>
+      <c r="B414" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C414" t="s">
+        <v>14</v>
+      </c>
+      <c r="D414" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E414" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F414" t="s">
+        <v>2212</v>
+      </c>
+      <c r="G414" t="s">
+        <v>2213</v>
+      </c>
+      <c r="H414" t="s">
+        <v>428</v>
+      </c>
+      <c r="I414" t="s">
+        <v>2214</v>
+      </c>
+      <c r="J414" t="s">
+        <v>308</v>
+      </c>
+      <c r="K414" t="s">
+        <v>2215</v>
+      </c>
+      <c r="L414" t="s">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="415" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A415">
+        <v>409</v>
+      </c>
+      <c r="B415" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C415" t="s">
+        <v>14</v>
+      </c>
+      <c r="D415" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E415" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F415" t="s">
+        <v>2217</v>
+      </c>
+      <c r="G415" t="s">
+        <v>2218</v>
+      </c>
+      <c r="H415" t="s">
+        <v>2041</v>
+      </c>
+      <c r="I415" t="s">
+        <v>2219</v>
+      </c>
+      <c r="J415" t="s">
+        <v>419</v>
+      </c>
+      <c r="K415" t="s">
+        <v>2220</v>
+      </c>
+      <c r="L415" t="s">
+        <v>2221</v>
+      </c>
+    </row>
+    <row r="416" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A416">
+        <v>410</v>
+      </c>
+      <c r="B416" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C416" t="s">
+        <v>14</v>
+      </c>
+      <c r="D416" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E416" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F416" t="s">
+        <v>2222</v>
+      </c>
+      <c r="G416" t="s">
+        <v>2223</v>
+      </c>
+      <c r="H416" t="s">
+        <v>2041</v>
+      </c>
+      <c r="I416" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J416" t="s">
+        <v>419</v>
+      </c>
+      <c r="K416" t="s">
+        <v>2225</v>
+      </c>
+      <c r="L416" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="417" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A417">
+        <v>411</v>
+      </c>
+      <c r="B417" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C417" t="s">
+        <v>14</v>
+      </c>
+      <c r="D417" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E417" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F417" t="s">
+        <v>2227</v>
+      </c>
+      <c r="G417" t="s">
+        <v>2228</v>
+      </c>
+      <c r="H417" t="s">
+        <v>2055</v>
+      </c>
+      <c r="I417" t="s">
+        <v>2229</v>
+      </c>
+      <c r="J417" t="s">
+        <v>345</v>
+      </c>
+      <c r="K417" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L417" t="s">
+        <v>2230</v>
+      </c>
+    </row>
+    <row r="418" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A418">
+        <v>412</v>
+      </c>
+      <c r="B418" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C418" t="s">
+        <v>14</v>
+      </c>
+      <c r="D418" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E418" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F418" t="s">
+        <v>2231</v>
+      </c>
+      <c r="G418" t="s">
+        <v>2232</v>
+      </c>
+      <c r="H418" t="s">
+        <v>2055</v>
+      </c>
+      <c r="I418" t="s">
+        <v>2233</v>
+      </c>
+      <c r="J418" t="s">
+        <v>345</v>
+      </c>
+      <c r="K418" t="s">
+        <v>2234</v>
+      </c>
+      <c r="L418" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="419" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A419">
+        <v>413</v>
+      </c>
+      <c r="B419" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C419" t="s">
+        <v>14</v>
+      </c>
+      <c r="D419" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E419" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F419" t="s">
+        <v>2236</v>
+      </c>
+      <c r="G419" t="s">
+        <v>2237</v>
+      </c>
+      <c r="H419" t="s">
+        <v>428</v>
+      </c>
+      <c r="I419" t="s">
+        <v>2238</v>
+      </c>
+      <c r="J419" t="s">
+        <v>308</v>
+      </c>
+      <c r="K419" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L419" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="420" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A420">
+        <v>414</v>
+      </c>
+      <c r="B420" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C420" t="s">
+        <v>14</v>
+      </c>
+      <c r="D420" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E420" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F420" t="s">
+        <v>2240</v>
+      </c>
+      <c r="G420" t="s">
+        <v>2241</v>
+      </c>
+      <c r="H420" t="s">
+        <v>428</v>
+      </c>
+      <c r="I420" t="s">
+        <v>2242</v>
+      </c>
+      <c r="J420" t="s">
+        <v>308</v>
+      </c>
+      <c r="K420" t="s">
+        <v>2243</v>
+      </c>
+      <c r="L420" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="421" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A421">
+        <v>415</v>
+      </c>
+      <c r="B421" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C421" t="s">
+        <v>14</v>
+      </c>
+      <c r="D421" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E421" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F421" t="s">
+        <v>2245</v>
+      </c>
+      <c r="G421" t="s">
+        <v>2246</v>
+      </c>
+      <c r="H421" t="s">
+        <v>428</v>
+      </c>
+      <c r="I421" t="s">
+        <v>2247</v>
+      </c>
+      <c r="J421" t="s">
+        <v>308</v>
+      </c>
+      <c r="K421" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L421" t="s">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="422" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A422">
+        <v>416</v>
+      </c>
+      <c r="B422" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C422" t="s">
+        <v>14</v>
+      </c>
+      <c r="D422" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E422" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F422" t="s">
+        <v>2249</v>
+      </c>
+      <c r="G422" t="s">
+        <v>2250</v>
+      </c>
+      <c r="H422" t="s">
+        <v>428</v>
+      </c>
+      <c r="I422" t="s">
+        <v>2251</v>
+      </c>
+      <c r="J422" t="s">
+        <v>308</v>
+      </c>
+      <c r="K422" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L422" t="s">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="423" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A423">
+        <v>417</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C423" t="s">
+        <v>14</v>
+      </c>
+      <c r="D423" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E423" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F423" t="s">
+        <v>2253</v>
+      </c>
+      <c r="G423" t="s">
+        <v>2254</v>
+      </c>
+      <c r="H423" t="s">
+        <v>428</v>
+      </c>
+      <c r="I423" t="s">
+        <v>2255</v>
+      </c>
+      <c r="J423" t="s">
+        <v>308</v>
+      </c>
+      <c r="K423" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L423" t="s">
+        <v>2256</v>
+      </c>
+    </row>
+    <row r="424" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A424">
+        <v>418</v>
+      </c>
+      <c r="B424" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C424" t="s">
+        <v>14</v>
+      </c>
+      <c r="D424" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E424" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F424" t="s">
+        <v>2257</v>
+      </c>
+      <c r="G424" t="s">
+        <v>2258</v>
+      </c>
+      <c r="H424" t="s">
+        <v>428</v>
+      </c>
+      <c r="I424" t="s">
+        <v>2259</v>
+      </c>
+      <c r="J424" t="s">
+        <v>308</v>
+      </c>
+      <c r="K424" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L424" t="s">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="425" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A425">
+        <v>419</v>
+      </c>
+      <c r="B425" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C425" t="s">
+        <v>14</v>
+      </c>
+      <c r="D425" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E425" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F425" t="s">
+        <v>2261</v>
+      </c>
+      <c r="G425" t="s">
+        <v>2262</v>
+      </c>
+      <c r="H425" t="s">
+        <v>428</v>
+      </c>
+      <c r="I425" t="s">
+        <v>2263</v>
+      </c>
+      <c r="J425" t="s">
+        <v>308</v>
+      </c>
+      <c r="K425" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L425" t="s">
+        <v>2264</v>
+      </c>
+    </row>
+    <row r="426" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A426">
+        <v>420</v>
+      </c>
+      <c r="B426" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C426" t="s">
+        <v>14</v>
+      </c>
+      <c r="D426" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E426" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F426" t="s">
+        <v>2265</v>
+      </c>
+      <c r="G426" t="s">
+        <v>2266</v>
+      </c>
+      <c r="H426" t="s">
+        <v>428</v>
+      </c>
+      <c r="I426" t="s">
+        <v>2267</v>
+      </c>
+      <c r="J426" t="s">
+        <v>308</v>
+      </c>
+      <c r="K426" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L426" t="s">
+        <v>2268</v>
+      </c>
+    </row>
+    <row r="427" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A427">
+        <v>421</v>
+      </c>
+      <c r="B427" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C427" t="s">
+        <v>14</v>
+      </c>
+      <c r="D427" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E427" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F427" t="s">
+        <v>2269</v>
+      </c>
+      <c r="G427" t="s">
+        <v>2270</v>
+      </c>
+      <c r="H427" t="s">
+        <v>428</v>
+      </c>
+      <c r="I427" t="s">
+        <v>2271</v>
+      </c>
+      <c r="J427" t="s">
+        <v>308</v>
+      </c>
+      <c r="K427" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L427" t="s">
+        <v>2272</v>
+      </c>
+    </row>
+    <row r="428" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A428">
+        <v>422</v>
+      </c>
+      <c r="B428" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C428" t="s">
+        <v>14</v>
+      </c>
+      <c r="D428" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E428" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F428" t="s">
+        <v>2273</v>
+      </c>
+      <c r="G428" t="s">
+        <v>2274</v>
+      </c>
+      <c r="H428" t="s">
+        <v>428</v>
+      </c>
+      <c r="I428" t="s">
+        <v>2275</v>
+      </c>
+      <c r="J428" t="s">
+        <v>308</v>
+      </c>
+      <c r="K428" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L428" t="s">
+        <v>2276</v>
+      </c>
+    </row>
+    <row r="429" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A429">
+        <v>423</v>
+      </c>
+      <c r="B429" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C429" t="s">
+        <v>14</v>
+      </c>
+      <c r="D429" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E429" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F429" t="s">
+        <v>2277</v>
+      </c>
+      <c r="G429" t="s">
+        <v>2278</v>
+      </c>
+      <c r="H429" t="s">
+        <v>428</v>
+      </c>
+      <c r="I429" t="s">
+        <v>2279</v>
+      </c>
+      <c r="J429" t="s">
+        <v>308</v>
+      </c>
+      <c r="K429" t="s">
+        <v>2280</v>
+      </c>
+      <c r="L429" t="s">
+        <v>2281</v>
+      </c>
+    </row>
+    <row r="430" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A430">
+        <v>424</v>
+      </c>
+      <c r="B430" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C430" t="s">
+        <v>14</v>
+      </c>
+      <c r="D430" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E430" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F430" t="s">
+        <v>2282</v>
+      </c>
+      <c r="G430" t="s">
+        <v>2283</v>
+      </c>
+      <c r="H430" t="s">
+        <v>428</v>
+      </c>
+      <c r="I430" t="s">
+        <v>2279</v>
+      </c>
+      <c r="J430" t="s">
+        <v>308</v>
+      </c>
+      <c r="K430" t="s">
+        <v>2284</v>
+      </c>
+      <c r="L430" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="431" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A431">
+        <v>425</v>
+      </c>
+      <c r="B431" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C431" t="s">
+        <v>14</v>
+      </c>
+      <c r="D431" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E431" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F431" t="s">
+        <v>2286</v>
+      </c>
+      <c r="G431" t="s">
+        <v>2287</v>
+      </c>
+      <c r="H431" t="s">
+        <v>428</v>
+      </c>
+      <c r="I431" t="s">
+        <v>2288</v>
+      </c>
+      <c r="J431" t="s">
+        <v>308</v>
+      </c>
+      <c r="K431" t="s">
+        <v>2289</v>
+      </c>
+      <c r="L431" t="s">
+        <v>2290</v>
+      </c>
+    </row>
+    <row r="432" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A432">
+        <v>426</v>
+      </c>
+      <c r="B432" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C432" t="s">
+        <v>14</v>
+      </c>
+      <c r="D432" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E432" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F432" t="s">
+        <v>2291</v>
+      </c>
+      <c r="G432" t="s">
+        <v>2292</v>
+      </c>
+      <c r="H432" t="s">
+        <v>428</v>
+      </c>
+      <c r="I432" t="s">
+        <v>2293</v>
+      </c>
+      <c r="J432" t="s">
+        <v>308</v>
+      </c>
+      <c r="K432" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L432" t="s">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="433" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A433">
+        <v>427</v>
+      </c>
+      <c r="B433" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C433" t="s">
+        <v>14</v>
+      </c>
+      <c r="D433" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E433" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F433" t="s">
+        <v>2295</v>
+      </c>
+      <c r="G433" t="s">
+        <v>2296</v>
+      </c>
+      <c r="H433" t="s">
+        <v>428</v>
+      </c>
+      <c r="I433" t="s">
+        <v>2297</v>
+      </c>
+      <c r="J433" t="s">
+        <v>308</v>
+      </c>
+      <c r="K433" t="s">
+        <v>2298</v>
+      </c>
+      <c r="L433" t="s">
+        <v>2299</v>
+      </c>
+    </row>
+    <row r="434" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A434">
+        <v>428</v>
+      </c>
+      <c r="B434" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C434" t="s">
+        <v>14</v>
+      </c>
+      <c r="D434" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E434" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F434" t="s">
+        <v>2300</v>
+      </c>
+      <c r="G434" t="s">
+        <v>2301</v>
+      </c>
+      <c r="H434" t="s">
+        <v>428</v>
+      </c>
+      <c r="I434" t="s">
+        <v>2302</v>
+      </c>
+      <c r="J434" t="s">
+        <v>308</v>
+      </c>
+      <c r="K434" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L434" t="s">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="435" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A435">
+        <v>429</v>
+      </c>
+      <c r="B435" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C435" t="s">
+        <v>14</v>
+      </c>
+      <c r="D435" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E435" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F435" t="s">
+        <v>2304</v>
+      </c>
+      <c r="G435" t="s">
+        <v>2305</v>
+      </c>
+      <c r="H435" t="s">
+        <v>428</v>
+      </c>
+      <c r="I435" t="s">
+        <v>2306</v>
+      </c>
+      <c r="J435" t="s">
+        <v>308</v>
+      </c>
+      <c r="K435" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L435" t="s">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="436" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A436">
+        <v>430</v>
+      </c>
+      <c r="B436" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C436" t="s">
+        <v>14</v>
+      </c>
+      <c r="D436" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E436" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F436" t="s">
+        <v>2308</v>
+      </c>
+      <c r="G436" t="s">
+        <v>2309</v>
+      </c>
+      <c r="H436" t="s">
+        <v>428</v>
+      </c>
+      <c r="I436" t="s">
+        <v>2310</v>
+      </c>
+      <c r="J436" t="s">
+        <v>308</v>
+      </c>
+      <c r="K436" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L436" t="s">
+        <v>2311</v>
+      </c>
+    </row>
+    <row r="437" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A437">
+        <v>431</v>
+      </c>
+      <c r="B437" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C437" t="s">
+        <v>14</v>
+      </c>
+      <c r="D437" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E437" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F437" t="s">
+        <v>2312</v>
+      </c>
+      <c r="G437" t="s">
+        <v>2313</v>
+      </c>
+      <c r="H437" t="s">
+        <v>428</v>
+      </c>
+      <c r="I437" t="s">
+        <v>1642</v>
+      </c>
+      <c r="J437" t="s">
+        <v>308</v>
+      </c>
+      <c r="K437" t="s">
+        <v>2314</v>
+      </c>
+      <c r="L437" t="s">
+        <v>2315</v>
+      </c>
+    </row>
+    <row r="438" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A438">
+        <v>432</v>
+      </c>
+      <c r="B438" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C438" t="s">
+        <v>14</v>
+      </c>
+      <c r="D438" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E438" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F438" t="s">
+        <v>2316</v>
+      </c>
+      <c r="G438" t="s">
+        <v>2317</v>
+      </c>
+      <c r="H438" t="s">
+        <v>428</v>
+      </c>
+      <c r="I438" t="s">
+        <v>2318</v>
+      </c>
+      <c r="J438" t="s">
+        <v>308</v>
+      </c>
+      <c r="K438" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L438" t="s">
+        <v>2319</v>
+      </c>
+    </row>
+    <row r="439" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A439">
+        <v>433</v>
+      </c>
+      <c r="B439" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C439" t="s">
+        <v>14</v>
+      </c>
+      <c r="D439" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E439" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F439" t="s">
+        <v>2320</v>
+      </c>
+      <c r="G439" t="s">
+        <v>2321</v>
+      </c>
+      <c r="H439" t="s">
+        <v>428</v>
+      </c>
+      <c r="I439" t="s">
+        <v>2322</v>
+      </c>
+      <c r="J439" t="s">
+        <v>308</v>
+      </c>
+      <c r="K439" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L439" t="s">
+        <v>2323</v>
+      </c>
+    </row>
+    <row r="440" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A440">
+        <v>434</v>
+      </c>
+      <c r="B440" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C440" t="s">
+        <v>14</v>
+      </c>
+      <c r="D440" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E440" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F440" t="s">
+        <v>2324</v>
+      </c>
+      <c r="G440" t="s">
+        <v>2325</v>
+      </c>
+      <c r="H440" t="s">
+        <v>428</v>
+      </c>
+      <c r="I440" t="s">
+        <v>2326</v>
+      </c>
+      <c r="J440" t="s">
+        <v>308</v>
+      </c>
+      <c r="K440" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L440" t="s">
+        <v>2327</v>
+      </c>
+    </row>
+    <row r="441" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A441">
+        <v>435</v>
+      </c>
+      <c r="B441" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C441" t="s">
+        <v>14</v>
+      </c>
+      <c r="D441" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E441" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F441" t="s">
+        <v>2328</v>
+      </c>
+      <c r="G441" t="s">
+        <v>2329</v>
+      </c>
+      <c r="H441" t="s">
+        <v>428</v>
+      </c>
+      <c r="I441" t="s">
+        <v>1650</v>
+      </c>
+      <c r="J441" t="s">
+        <v>308</v>
+      </c>
+      <c r="K441" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L441" t="s">
+        <v>2330</v>
+      </c>
+    </row>
+    <row r="442" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A442">
+        <v>436</v>
+      </c>
+      <c r="B442" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C442" t="s">
+        <v>14</v>
+      </c>
+      <c r="D442" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E442" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F442" t="s">
+        <v>2331</v>
+      </c>
+      <c r="G442" t="s">
+        <v>2332</v>
+      </c>
+      <c r="H442" t="s">
+        <v>428</v>
+      </c>
+      <c r="I442" t="s">
+        <v>1650</v>
+      </c>
+      <c r="J442" t="s">
+        <v>308</v>
+      </c>
+      <c r="K442" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L442" t="s">
+        <v>2333</v>
+      </c>
+    </row>
+    <row r="443" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A443">
+        <v>437</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C443" t="s">
+        <v>14</v>
+      </c>
+      <c r="D443" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E443" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F443" t="s">
+        <v>2334</v>
+      </c>
+      <c r="G443" t="s">
+        <v>2335</v>
+      </c>
+      <c r="H443" t="s">
+        <v>428</v>
+      </c>
+      <c r="I443" t="s">
+        <v>2336</v>
+      </c>
+      <c r="J443" t="s">
+        <v>308</v>
+      </c>
+      <c r="K443" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L443" t="s">
+        <v>2337</v>
+      </c>
+    </row>
+    <row r="444" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A444">
+        <v>438</v>
+      </c>
+      <c r="B444" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C444" t="s">
+        <v>14</v>
+      </c>
+      <c r="D444" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E444" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F444" t="s">
+        <v>2338</v>
+      </c>
+      <c r="G444" t="s">
+        <v>2339</v>
+      </c>
+      <c r="H444" t="s">
+        <v>428</v>
+      </c>
+      <c r="I444" t="s">
+        <v>2340</v>
+      </c>
+      <c r="J444" t="s">
+        <v>308</v>
+      </c>
+      <c r="K444" t="s">
+        <v>2341</v>
+      </c>
+      <c r="L444" t="s">
+        <v>2342</v>
+      </c>
+    </row>
+    <row r="445" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A445">
+        <v>439</v>
+      </c>
+      <c r="B445" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C445" t="s">
+        <v>14</v>
+      </c>
+      <c r="D445" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E445" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F445" t="s">
+        <v>2343</v>
+      </c>
+      <c r="G445" t="s">
+        <v>2344</v>
+      </c>
+      <c r="H445" t="s">
+        <v>428</v>
+      </c>
+      <c r="I445" t="s">
+        <v>2345</v>
+      </c>
+      <c r="J445" t="s">
+        <v>308</v>
+      </c>
+      <c r="K445" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L445" t="s">
+        <v>2346</v>
+      </c>
+    </row>
+    <row r="446" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A446">
+        <v>440</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C446" t="s">
+        <v>14</v>
+      </c>
+      <c r="D446" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E446" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F446" t="s">
+        <v>2347</v>
+      </c>
+      <c r="G446" t="s">
+        <v>2348</v>
+      </c>
+      <c r="H446" t="s">
+        <v>428</v>
+      </c>
+      <c r="I446" t="s">
+        <v>2349</v>
+      </c>
+      <c r="J446" t="s">
+        <v>308</v>
+      </c>
+      <c r="K446" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L446" t="s">
+        <v>2350</v>
+      </c>
+    </row>
+    <row r="447" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A447">
+        <v>441</v>
+      </c>
+      <c r="B447" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C447" t="s">
+        <v>14</v>
+      </c>
+      <c r="D447" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E447" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F447" t="s">
+        <v>2351</v>
+      </c>
+      <c r="G447" t="s">
+        <v>2352</v>
+      </c>
+      <c r="H447" t="s">
+        <v>428</v>
+      </c>
+      <c r="I447" t="s">
+        <v>2353</v>
+      </c>
+      <c r="J447" t="s">
+        <v>308</v>
+      </c>
+      <c r="K447" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L447" t="s">
+        <v>2354</v>
+      </c>
+    </row>
+    <row r="448" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A448">
+        <v>442</v>
+      </c>
+      <c r="B448" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C448" t="s">
+        <v>14</v>
+      </c>
+      <c r="D448" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E448" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F448" t="s">
+        <v>2355</v>
+      </c>
+      <c r="G448" t="s">
+        <v>2356</v>
+      </c>
+      <c r="H448" t="s">
+        <v>343</v>
+      </c>
+      <c r="I448" t="s">
+        <v>2357</v>
+      </c>
+      <c r="J448" t="s">
+        <v>460</v>
+      </c>
+      <c r="K448" t="s">
+        <v>2358</v>
+      </c>
+      <c r="L448" t="s">
+        <v>2359</v>
+      </c>
+    </row>
+    <row r="449" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A449">
+        <v>443</v>
+      </c>
+      <c r="B449" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C449" t="s">
+        <v>14</v>
+      </c>
+      <c r="D449" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E449" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F449" t="s">
+        <v>2360</v>
+      </c>
+      <c r="G449" t="s">
+        <v>2361</v>
+      </c>
+      <c r="H449" t="s">
+        <v>343</v>
+      </c>
+      <c r="I449" t="s">
+        <v>2362</v>
+      </c>
+      <c r="J449" t="s">
+        <v>460</v>
+      </c>
+      <c r="K449" t="s">
+        <v>2363</v>
+      </c>
+      <c r="L449" t="s">
+        <v>2364</v>
+      </c>
+    </row>
+    <row r="450" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A450">
+        <v>444</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C450" t="s">
+        <v>14</v>
+      </c>
+      <c r="D450" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E450" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F450" t="s">
+        <v>2365</v>
+      </c>
+      <c r="G450" t="s">
+        <v>2366</v>
+      </c>
+      <c r="H450" t="s">
+        <v>343</v>
+      </c>
+      <c r="I450" t="s">
+        <v>2367</v>
+      </c>
+      <c r="J450" t="s">
+        <v>460</v>
+      </c>
+      <c r="K450" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L450" t="s">
+        <v>2368</v>
+      </c>
+    </row>
+    <row r="451" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A451">
+        <v>445</v>
+      </c>
+      <c r="B451" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C451" t="s">
+        <v>14</v>
+      </c>
+      <c r="D451" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E451" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F451" t="s">
+        <v>2369</v>
+      </c>
+      <c r="G451" t="s">
+        <v>2370</v>
+      </c>
+      <c r="H451" t="s">
+        <v>343</v>
+      </c>
+      <c r="I451" t="s">
+        <v>2362</v>
+      </c>
+      <c r="J451" t="s">
+        <v>460</v>
+      </c>
+      <c r="K451" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L451" t="s">
+        <v>2371</v>
+      </c>
+    </row>
+    <row r="452" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A452">
+        <v>446</v>
+      </c>
+      <c r="B452" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C452" t="s">
+        <v>14</v>
+      </c>
+      <c r="D452" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E452" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F452" t="s">
+        <v>2372</v>
+      </c>
+      <c r="G452" t="s">
+        <v>2373</v>
+      </c>
+      <c r="H452" t="s">
+        <v>343</v>
+      </c>
+      <c r="I452" t="s">
+        <v>2374</v>
+      </c>
+      <c r="J452" t="s">
+        <v>460</v>
+      </c>
+      <c r="K452" t="s">
+        <v>2375</v>
+      </c>
+      <c r="L452" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="453" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A453">
+        <v>447</v>
+      </c>
+      <c r="B453" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C453" t="s">
+        <v>14</v>
+      </c>
+      <c r="D453" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E453" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F453" t="s">
+        <v>2377</v>
+      </c>
+      <c r="G453" t="s">
+        <v>2378</v>
+      </c>
+      <c r="H453" t="s">
+        <v>343</v>
+      </c>
+      <c r="I453" t="s">
+        <v>2379</v>
+      </c>
+      <c r="J453" t="s">
+        <v>460</v>
+      </c>
+      <c r="K453" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L453" t="s">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="454" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A454">
+        <v>448</v>
+      </c>
+      <c r="B454" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C454" t="s">
+        <v>14</v>
+      </c>
+      <c r="D454" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E454" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F454" t="s">
+        <v>2365</v>
+      </c>
+      <c r="G454" t="s">
+        <v>2366</v>
+      </c>
+      <c r="H454" t="s">
+        <v>343</v>
+      </c>
+      <c r="I454" t="s">
+        <v>2367</v>
+      </c>
+      <c r="J454" t="s">
+        <v>460</v>
+      </c>
+      <c r="K454" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L454" t="s">
+        <v>2368</v>
+      </c>
+    </row>
+    <row r="455" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A455">
+        <v>449</v>
+      </c>
+      <c r="B455" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C455" t="s">
+        <v>14</v>
+      </c>
+      <c r="D455" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E455" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F455" t="s">
+        <v>2369</v>
+      </c>
+      <c r="G455" t="s">
+        <v>2370</v>
+      </c>
+      <c r="H455" t="s">
+        <v>343</v>
+      </c>
+      <c r="I455" t="s">
+        <v>2362</v>
+      </c>
+      <c r="J455" t="s">
+        <v>460</v>
+      </c>
+      <c r="K455" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L455" t="s">
+        <v>2371</v>
+      </c>
+    </row>
+    <row r="456" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A456">
+        <v>450</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C456" t="s">
+        <v>14</v>
+      </c>
+      <c r="D456" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E456" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F456" t="s">
+        <v>2372</v>
+      </c>
+      <c r="G456" t="s">
+        <v>2373</v>
+      </c>
+      <c r="H456" t="s">
+        <v>343</v>
+      </c>
+      <c r="I456" t="s">
+        <v>2374</v>
+      </c>
+      <c r="J456" t="s">
+        <v>460</v>
+      </c>
+      <c r="K456" t="s">
+        <v>2375</v>
+      </c>
+      <c r="L456" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="457" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A457">
+        <v>451</v>
+      </c>
+      <c r="B457" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C457" t="s">
+        <v>14</v>
+      </c>
+      <c r="D457" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E457" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F457" t="s">
+        <v>2381</v>
+      </c>
+      <c r="G457" t="s">
+        <v>2382</v>
+      </c>
+      <c r="H457" t="s">
+        <v>343</v>
+      </c>
+      <c r="I457" t="s">
+        <v>2383</v>
+      </c>
+      <c r="J457" t="s">
+        <v>460</v>
+      </c>
+      <c r="K457" t="s">
+        <v>2384</v>
+      </c>
+      <c r="L457" t="s">
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="458" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A458">
+        <v>452</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C458" t="s">
+        <v>14</v>
+      </c>
+      <c r="D458" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E458" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F458" t="s">
+        <v>2386</v>
+      </c>
+      <c r="G458" t="s">
+        <v>2387</v>
+      </c>
+      <c r="H458" t="s">
+        <v>343</v>
+      </c>
+      <c r="I458" t="s">
+        <v>2388</v>
+      </c>
+      <c r="J458" t="s">
+        <v>460</v>
+      </c>
+      <c r="K458" t="s">
+        <v>2389</v>
+      </c>
+      <c r="L458" t="s">
+        <v>2390</v>
+      </c>
+    </row>
+    <row r="459" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A459">
+        <v>453</v>
+      </c>
+      <c r="B459" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C459" t="s">
+        <v>14</v>
+      </c>
+      <c r="D459" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E459" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F459" t="s">
+        <v>2377</v>
+      </c>
+      <c r="G459" t="s">
+        <v>2378</v>
+      </c>
+      <c r="H459" t="s">
+        <v>343</v>
+      </c>
+      <c r="I459" t="s">
+        <v>2379</v>
+      </c>
+      <c r="J459" t="s">
+        <v>460</v>
+      </c>
+      <c r="K459" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L459" t="s">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="460" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A460">
+        <v>454</v>
+      </c>
+      <c r="B460" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C460" t="s">
+        <v>14</v>
+      </c>
+      <c r="D460" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E460" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F460" t="s">
+        <v>2391</v>
+      </c>
+      <c r="G460" t="s">
+        <v>2392</v>
+      </c>
+      <c r="H460" t="s">
+        <v>343</v>
+      </c>
+      <c r="I460" t="s">
+        <v>2393</v>
+      </c>
+      <c r="J460" t="s">
+        <v>460</v>
+      </c>
+      <c r="K460" t="s">
+        <v>1848</v>
+      </c>
+      <c r="L460" t="s">
+        <v>2394</v>
+      </c>
+    </row>
+    <row r="461" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A461">
+        <v>455</v>
+      </c>
+      <c r="B461" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C461" t="s">
+        <v>14</v>
+      </c>
+      <c r="D461" t="s">
+        <v>1848</v>
+      </c>
+      <c r="E461" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F461" t="s">
+        <v>2395</v>
+      </c>
+      <c r="G461" t="s">
+        <v>2396</v>
+      </c>
+      <c r="H461" t="s">
+        <v>343</v>
+      </c>
+      <c r="I461" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J461" t="s">
+        <v>460</v>
+      </c>
+      <c r="K461" t="s">
+        <v>2398</v>
+      </c>
+      <c r="L461" t="s">
+        <v>2399</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 3 WebKreatives OSM leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4589" uniqueCount="2714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="2729">
   <si>
     <t>#</t>
   </si>
@@ -8153,6 +8153,51 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:2860110797 | Source: OpenStreetMap | schoonheidssalon | Amsterdam | Website: https://www.amarylishuidverzorging.nl</t>
+  </si>
+  <si>
+    <t>johnsdierenwereld@gmail.com</t>
+  </si>
+  <si>
+    <t>John's Dierenwereld</t>
+  </si>
+  <si>
+    <t>Geitenkamp 6823HE</t>
+  </si>
+  <si>
+    <t>Arnhem</t>
+  </si>
+  <si>
+    <t>+31 26 379 3347</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2721234060 | Source: OpenStreetMap | dierenwinkel | Arnhem | Website: http://www.johnsdierenwereld.nl</t>
+  </si>
+  <si>
+    <t>arnhempietercalandweg@maxizoo.nl</t>
+  </si>
+  <si>
+    <t>Maxi Zoo XXL</t>
+  </si>
+  <si>
+    <t>P. Calandweg 6827BK</t>
+  </si>
+  <si>
+    <t>+31 26 3648811</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2722374735 | Source: OpenStreetMap | dierenwinkel | Arnhem | Website: https://www.maxizoo.nl/winkels/maxi-zoo-arnhem-xxl</t>
+  </si>
+  <si>
+    <t>info@animalsandmore.nl</t>
+  </si>
+  <si>
+    <t>Animals &amp; More</t>
+  </si>
+  <si>
+    <t>Elderveldplein 6843JA</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2725541777 | Source: OpenStreetMap | dierenwinkel | Arnhem | Website: https://animalsandmore.nl</t>
   </si>
 </sst>
 </file>
@@ -8529,8 +8574,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L526"/>
-  <sheetFormatPr customHeight="1"/>
+  <dimension ref="A1:L529"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -24929,6 +24974,120 @@
         <v>2713</v>
       </c>
     </row>
+    <row r="527" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A527">
+        <v>526</v>
+      </c>
+      <c r="B527" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C527" t="s">
+        <v>14</v>
+      </c>
+      <c r="D527" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E527" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F527" t="s">
+        <v>2714</v>
+      </c>
+      <c r="G527" t="s">
+        <v>2715</v>
+      </c>
+      <c r="H527" t="s">
+        <v>2054</v>
+      </c>
+      <c r="I527" t="s">
+        <v>2716</v>
+      </c>
+      <c r="J527" t="s">
+        <v>2717</v>
+      </c>
+      <c r="K527" t="s">
+        <v>2718</v>
+      </c>
+      <c r="L527" t="s">
+        <v>2719</v>
+      </c>
+    </row>
+    <row r="528" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A528">
+        <v>527</v>
+      </c>
+      <c r="B528" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C528" t="s">
+        <v>14</v>
+      </c>
+      <c r="D528" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E528" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F528" t="s">
+        <v>2720</v>
+      </c>
+      <c r="G528" t="s">
+        <v>2721</v>
+      </c>
+      <c r="H528" t="s">
+        <v>2054</v>
+      </c>
+      <c r="I528" t="s">
+        <v>2722</v>
+      </c>
+      <c r="J528" t="s">
+        <v>2717</v>
+      </c>
+      <c r="K528" t="s">
+        <v>2723</v>
+      </c>
+      <c r="L528" t="s">
+        <v>2724</v>
+      </c>
+    </row>
+    <row r="529" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A529">
+        <v>528</v>
+      </c>
+      <c r="B529" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C529" t="s">
+        <v>14</v>
+      </c>
+      <c r="D529" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E529" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F529" t="s">
+        <v>2725</v>
+      </c>
+      <c r="G529" t="s">
+        <v>2726</v>
+      </c>
+      <c r="H529" t="s">
+        <v>2054</v>
+      </c>
+      <c r="I529" t="s">
+        <v>2727</v>
+      </c>
+      <c r="J529" t="s">
+        <v>2717</v>
+      </c>
+      <c r="K529" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L529" t="s">
+        <v>2728</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 40 new OSM leads to Leads workbook
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="2729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5146" uniqueCount="2916">
   <si>
     <t>#</t>
   </si>
@@ -8198,6 +8198,567 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:2725541777 | Source: OpenStreetMap | dierenwinkel | Arnhem | Website: https://animalsandmore.nl</t>
+  </si>
+  <si>
+    <t>info@cristalcleaning.nl</t>
+  </si>
+  <si>
+    <t>Cristal Cleaning</t>
+  </si>
+  <si>
+    <t>Geldropseweg 5611SJ</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2759420023 | Source: OpenStreetMap | stomerij | Eindhoven | Website: https://cristalcleaning.nl</t>
+  </si>
+  <si>
+    <t>info@cococlinics.nl</t>
+  </si>
+  <si>
+    <t>Coco Clinics</t>
+  </si>
+  <si>
+    <t>Amsterdamsestraatweg 3551CM</t>
+  </si>
+  <si>
+    <t>+31 30 202 3470</t>
+  </si>
+  <si>
+    <t>Geen website | Email from OSM | OSM id:2632906720 | Source: OpenStreetMap | schoonheidssalon | Utrecht</t>
+  </si>
+  <si>
+    <t>info@stomerijverhagen.com</t>
+  </si>
+  <si>
+    <t>Stomerij Verhagen</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:12222992565 | Source: OpenStreetMap | stomerij | Eindhoven | Website: https://www.stomerijverhagen.com</t>
+  </si>
+  <si>
+    <t>info@wasserettesoapclub.nl</t>
+  </si>
+  <si>
+    <t>Soapclub</t>
+  </si>
+  <si>
+    <t>Sumatraweg 1335JM</t>
+  </si>
+  <si>
+    <t>+31 6 16 367 216</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2844873864 | Source: OpenStreetMap | wasserette | Almere | Website: https://www.wasserettesoapclub.nl</t>
+  </si>
+  <si>
+    <t>keesdeegitaren@gmail.com</t>
+  </si>
+  <si>
+    <t>Kees Dee</t>
+  </si>
+  <si>
+    <t>Leusderweg 3817KB</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2638642143 | Source: OpenStreetMap | muziekwinkel | Amersfoort | Website: https://www.keesdee.nl</t>
+  </si>
+  <si>
+    <t>info@voerman.nl</t>
+  </si>
+  <si>
+    <t>Voerman</t>
+  </si>
+  <si>
+    <t>Vanadiumweg 3812PX</t>
+  </si>
+  <si>
+    <t>+31 33 461 2908</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2684746104 | Source: OpenStreetMap | muziekwinkel | Amersfoort | Website: https://www.voerman.nl</t>
+  </si>
+  <si>
+    <t>info@koekenreinders.nl</t>
+  </si>
+  <si>
+    <t>Koek &amp; Reinders</t>
+  </si>
+  <si>
+    <t>Tauber 2491DB</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2608637861 | Source: OpenStreetMap | schildersbedrijf | Den Haag | Website: https://koekenreinders.nl</t>
+  </si>
+  <si>
+    <t>info@tib.nl</t>
+  </si>
+  <si>
+    <t>TIB Totaal-Installateurs</t>
+  </si>
+  <si>
+    <t>Felland-Noord 9753TB</t>
+  </si>
+  <si>
+    <t>Haren Gn</t>
+  </si>
+  <si>
+    <t>+31 50 534 9902</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2813734790 | Source: OpenStreetMap | loodgieter | Groningen | Website: https://www.tib.nl</t>
+  </si>
+  <si>
+    <t>breda@hoppenbrouwers.nl</t>
+  </si>
+  <si>
+    <t>Hoppenbrouwers</t>
+  </si>
+  <si>
+    <t>Mijkenbroek 4824AA</t>
+  </si>
+  <si>
+    <t>+31 76 201 3200</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:8416043461 | Source: OpenStreetMap | elektricien | Breda | Website: https://www.hoppenbrouwerstechniek.nl/vestiging/breda</t>
+  </si>
+  <si>
+    <t>info@jacobselektro.nl</t>
+  </si>
+  <si>
+    <t>Jacobs Elektro</t>
+  </si>
+  <si>
+    <t>Minervum 4817ZL</t>
+  </si>
+  <si>
+    <t>+31 76 560 70 80</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:9386441204 | Source: OpenStreetMap | elektricien | Breda | Website: https://jacobselektro.nl</t>
+  </si>
+  <si>
+    <t>candelabeautyclinic@gmail.com</t>
+  </si>
+  <si>
+    <t>Candela Beauty Clinic</t>
+  </si>
+  <si>
+    <t>Aquamarijnlaan 3523EK</t>
+  </si>
+  <si>
+    <t>+31 6 28856394</t>
+  </si>
+  <si>
+    <t>Geen website | Email from OSM | OSM id:3035791722 | Source: OpenStreetMap | schoonheidssalon | Utrecht</t>
+  </si>
+  <si>
+    <t>info@apeldoorn-bloemzaad.nl</t>
+  </si>
+  <si>
+    <t>Apeldoorn &amp; Bloemzaad</t>
+  </si>
+  <si>
+    <t>Wilmersdorf 7327AC</t>
+  </si>
+  <si>
+    <t>+31 55 366 6610</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2685596439 | Source: OpenStreetMap | rijschool | Apeldoorn | Website: https://www.apeldoornenbloemzaad.nl</t>
+  </si>
+  <si>
+    <t>info@frankschuurman.nl</t>
+  </si>
+  <si>
+    <t>Frank Schuurman</t>
+  </si>
+  <si>
+    <t>Ovenbouwershoek 7328JH</t>
+  </si>
+  <si>
+    <t>+31 55 366 4363</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2685902825 | Source: OpenStreetMap | rijschool | Apeldoorn | Website: https://frankschuurman.nl</t>
+  </si>
+  <si>
+    <t>info@lesismoreapeldoorn.nl</t>
+  </si>
+  <si>
+    <t>Les is More</t>
+  </si>
+  <si>
+    <t>Kraaienweg 7331HZ</t>
+  </si>
+  <si>
+    <t>+31 6 43185597</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2686859278 | Source: OpenStreetMap | rijschool | Apeldoorn | Website: https://lesismoreapeldoorn.nl</t>
+  </si>
+  <si>
+    <t>info@verkeersschool-develuwe.nl</t>
+  </si>
+  <si>
+    <t>De Veluwe</t>
+  </si>
+  <si>
+    <t>+31 55 533 5333</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:5175999870 | Source: OpenStreetMap | rijschool | Apeldoorn | Website: https://www.verkeersschool-develuwe.nl</t>
+  </si>
+  <si>
+    <t>info@deweerd.net</t>
+  </si>
+  <si>
+    <t>De Weerd</t>
+  </si>
+  <si>
+    <t>Kayersdijk 7332AP</t>
+  </si>
+  <si>
+    <t>+31 85 073 2400</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:8730846983 | Source: OpenStreetMap | rijschool | Apeldoorn | Website: https://deweerd.net</t>
+  </si>
+  <si>
+    <t>bestel@lesalonard.shop</t>
+  </si>
+  <si>
+    <t>Le Salonard</t>
+  </si>
+  <si>
+    <t>Witmakersstraat 6211HV</t>
+  </si>
+  <si>
+    <t>+31 6 50741662</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2804897354 | Source: OpenStreetMap | traiteur | Maastricht | Website: https://lesalonard.shop</t>
+  </si>
+  <si>
+    <t>info@adriaandesmaakmaker.nl</t>
+  </si>
+  <si>
+    <t>Adriaan De Smaakmaker</t>
+  </si>
+  <si>
+    <t>Sint Pieterstraat 6211JN</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:6799165677 | Source: OpenStreetMap | traiteur | Maastricht | Website: https://adriaandesmaakmaker.nl</t>
+  </si>
+  <si>
+    <t>raymon@sessions-hair.nl</t>
+  </si>
+  <si>
+    <t>Sessions</t>
+  </si>
+  <si>
+    <t>Ferdinand Bolstraat 1072LG</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:257518629 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://sessions-hair.nl</t>
+  </si>
+  <si>
+    <t>leonard@reyez.nl</t>
+  </si>
+  <si>
+    <t>CFH Care For Hair</t>
+  </si>
+  <si>
+    <t>Kempenlaan 1066RB</t>
+  </si>
+  <si>
+    <t>+31 20 615 1215</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:746906773 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://careforhair.nl</t>
+  </si>
+  <si>
+    <t>info@barbershopjordaan.nl</t>
+  </si>
+  <si>
+    <t>Barbershop Jordaan</t>
+  </si>
+  <si>
+    <t>Eerste Looiersdwarsstraat 1016VM</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:859922189 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://barbershopjordaan.com</t>
+  </si>
+  <si>
+    <t>xandrashairstyling@ziggo.nl</t>
+  </si>
+  <si>
+    <t>Xandra's hairstyling</t>
+  </si>
+  <si>
+    <t>Bos en Lommerweg 1055EJ</t>
+  </si>
+  <si>
+    <t>+31 20 682 5333</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1044711285 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://xandras-hairstyling.nl</t>
+  </si>
+  <si>
+    <t>info@ossi-hairstyling.com</t>
+  </si>
+  <si>
+    <t>Ossi</t>
+  </si>
+  <si>
+    <t>Jan Pieter Heijestraat 1054MH</t>
+  </si>
+  <si>
+    <t>+31 20 618 3462</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:1686808203 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: http://ossi-hairstyling.com</t>
+  </si>
+  <si>
+    <t>info@thehairdoctor.nl</t>
+  </si>
+  <si>
+    <t>The Hair Doctor</t>
+  </si>
+  <si>
+    <t>Beukenweg 1091KE</t>
+  </si>
+  <si>
+    <t>+31 20 663 3139;+31 6 30105598</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2363285234 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.thehairdoctor.nl</t>
+  </si>
+  <si>
+    <t>info@gentleman.nl</t>
+  </si>
+  <si>
+    <t>Gentleman</t>
+  </si>
+  <si>
+    <t>Levantplein 1019MB</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2382672981 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.gentleman.nl</t>
+  </si>
+  <si>
+    <t>hello@atsoap.com</t>
+  </si>
+  <si>
+    <t>Soap Treatment Store</t>
+  </si>
+  <si>
+    <t>Oudkerkhof 3512GL</t>
+  </si>
+  <si>
+    <t>+31 30 341 0050</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:874363744 | Source: OpenStreetMap | schoonheidssalon | Utrecht | Website: https://soaptreatmentstore.com</t>
+  </si>
+  <si>
+    <t>hello@haaremajes.nl</t>
+  </si>
+  <si>
+    <t>Haare Majes</t>
+  </si>
+  <si>
+    <t>Czaar Peterstraat 1018PV</t>
+  </si>
+  <si>
+    <t>+31 20 620 60 70</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2415190892 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://haaremajes.nl</t>
+  </si>
+  <si>
+    <t>info@parlour.amsterdam</t>
+  </si>
+  <si>
+    <t>Parlour Amsterdam</t>
+  </si>
+  <si>
+    <t>Eerste Van der Helststraat 1072NZ</t>
+  </si>
+  <si>
+    <t>+31 6 15020269</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2510438388 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://parlour.amsterdam</t>
+  </si>
+  <si>
+    <t>hallo@potionhairdesign.nl</t>
+  </si>
+  <si>
+    <t>Potion Hairdesign</t>
+  </si>
+  <si>
+    <t>Sarphatipark 1073CX</t>
+  </si>
+  <si>
+    <t>+31 20 4700085</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2511420731 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.potionhairdesign.nl</t>
+  </si>
+  <si>
+    <t>info@menspire.nl</t>
+  </si>
+  <si>
+    <t>Menspire</t>
+  </si>
+  <si>
+    <t>Gerard Douplein 1072VE</t>
+  </si>
+  <si>
+    <t>+31 20 2213948</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2641085731 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://menspire.nl</t>
+  </si>
+  <si>
+    <t>info@mo-hair.nl</t>
+  </si>
+  <si>
+    <t>Mohair</t>
+  </si>
+  <si>
+    <t>Noordermarkt 1015MX</t>
+  </si>
+  <si>
+    <t>+31 20 428 4939</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2720871690 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://mo-hair.nl</t>
+  </si>
+  <si>
+    <t>heath@ohyouprettythings.nl</t>
+  </si>
+  <si>
+    <t>Oh You Pretty Things</t>
+  </si>
+  <si>
+    <t>Spuistraat 1012ST</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2721522278 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.ohyouprettythings.nl</t>
+  </si>
+  <si>
+    <t>barbernadir@hotmail.com</t>
+  </si>
+  <si>
+    <t>Barbershop Stardam</t>
+  </si>
+  <si>
+    <t>Nieuwezijds Voorburgwal 1012RD</t>
+  </si>
+  <si>
+    <t>+31 6 48 39 40 06</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2721772897 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://barbershopstardam.com</t>
+  </si>
+  <si>
+    <t>info@theatredecoiffure.nl</t>
+  </si>
+  <si>
+    <t>Theatre de Coiffure</t>
+  </si>
+  <si>
+    <t>Rozengracht 1016LP</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2721817199 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: http://www.theatredecoiffure.nl</t>
+  </si>
+  <si>
+    <t>elencantohairsalon@hotmail.com</t>
+  </si>
+  <si>
+    <t>El Encanto</t>
+  </si>
+  <si>
+    <t>Reguliersdwarsstraat 1017BK</t>
+  </si>
+  <si>
+    <t>+31 20 331 9142</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2725914014 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.elencantohairsalon.com</t>
+  </si>
+  <si>
+    <t>info@whocaressalon.com</t>
+  </si>
+  <si>
+    <t>Who Cares</t>
+  </si>
+  <si>
+    <t>Reguliersdwarsstraat 1017BM</t>
+  </si>
+  <si>
+    <t>+31 20 625 8224</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2725914333 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.whocaressalon.com</t>
+  </si>
+  <si>
+    <t>admin@redefinedbarbers.nl</t>
+  </si>
+  <si>
+    <t>Redefined Barbers</t>
+  </si>
+  <si>
+    <t>Vijzelstraat 1017HG</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2736378803 | Source: OpenStreetMap | kapsalon | Amsterdam | Website: https://www.redefinedbarbers.nl</t>
+  </si>
+  <si>
+    <t>info@nailsbyhuong.nl</t>
+  </si>
+  <si>
+    <t>Nails by Huong</t>
+  </si>
+  <si>
+    <t>Steenweg 3511JL</t>
+  </si>
+  <si>
+    <t>+31 6 4926 0372</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:874368484 | Source: OpenStreetMap | schoonheidssalon | Utrecht | Website: https://nailsbyhuong.nl</t>
+  </si>
+  <si>
+    <t>info@perfectlaserbeauty.nl</t>
+  </si>
+  <si>
+    <t>Perfect Laser &amp; Beauty</t>
+  </si>
+  <si>
+    <t>Spitsenhagen 3078BM</t>
+  </si>
+  <si>
+    <t>Geen website | Email from OSM | OSM id:2791459423 | Source: OpenStreetMap | schoonheidssalon | Rotterdam</t>
+  </si>
+  <si>
+    <t>info@aquariuscare.nl</t>
+  </si>
+  <si>
+    <t>Aquarius huidverzorgingsinstituut</t>
+  </si>
+  <si>
+    <t>Kreekplein 3079AB</t>
+  </si>
+  <si>
+    <t>+31 10 482 6912</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:1709201934 | Source: OpenStreetMap | schoonheidssalon | Rotterdam | Website: http://www.aquariuscare.nl</t>
   </si>
 </sst>
 </file>
@@ -8574,7 +9135,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L529"/>
+  <dimension ref="A1:L576"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -11478,7 +12039,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -25088,6 +25649,1792 @@
         <v>2728</v>
       </c>
     </row>
+    <row r="530" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A530">
+        <v>529</v>
+      </c>
+      <c r="B530" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C530" t="s">
+        <v>14</v>
+      </c>
+      <c r="D530" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E530" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F530" t="s">
+        <v>2729</v>
+      </c>
+      <c r="G530" t="s">
+        <v>2730</v>
+      </c>
+      <c r="H530" t="s">
+        <v>2040</v>
+      </c>
+      <c r="I530" t="s">
+        <v>2731</v>
+      </c>
+      <c r="J530" t="s">
+        <v>291</v>
+      </c>
+      <c r="K530" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L530" t="s">
+        <v>2732</v>
+      </c>
+    </row>
+    <row r="531" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A531">
+        <v>530</v>
+      </c>
+      <c r="B531" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C531" t="s">
+        <v>14</v>
+      </c>
+      <c r="D531" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E531" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F531" t="s">
+        <v>2733</v>
+      </c>
+      <c r="G531" t="s">
+        <v>2734</v>
+      </c>
+      <c r="H531" t="s">
+        <v>343</v>
+      </c>
+      <c r="I531" t="s">
+        <v>2735</v>
+      </c>
+      <c r="J531" t="s">
+        <v>103</v>
+      </c>
+      <c r="K531" t="s">
+        <v>2736</v>
+      </c>
+      <c r="L531" t="s">
+        <v>2737</v>
+      </c>
+    </row>
+    <row r="532" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A532">
+        <v>531</v>
+      </c>
+      <c r="B532" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C532" t="s">
+        <v>14</v>
+      </c>
+      <c r="D532" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E532" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F532" t="s">
+        <v>2738</v>
+      </c>
+      <c r="G532" t="s">
+        <v>2739</v>
+      </c>
+      <c r="H532" t="s">
+        <v>2040</v>
+      </c>
+      <c r="I532" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J532" t="s">
+        <v>291</v>
+      </c>
+      <c r="K532" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L532" t="s">
+        <v>2740</v>
+      </c>
+    </row>
+    <row r="533" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A533">
+        <v>532</v>
+      </c>
+      <c r="B533" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C533" t="s">
+        <v>14</v>
+      </c>
+      <c r="D533" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E533" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F533" t="s">
+        <v>2741</v>
+      </c>
+      <c r="G533" t="s">
+        <v>2742</v>
+      </c>
+      <c r="H533" t="s">
+        <v>1895</v>
+      </c>
+      <c r="I533" t="s">
+        <v>2743</v>
+      </c>
+      <c r="J533" t="s">
+        <v>2002</v>
+      </c>
+      <c r="K533" t="s">
+        <v>2744</v>
+      </c>
+      <c r="L533" t="s">
+        <v>2745</v>
+      </c>
+    </row>
+    <row r="534" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A534">
+        <v>533</v>
+      </c>
+      <c r="B534" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C534" t="s">
+        <v>14</v>
+      </c>
+      <c r="D534" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E534" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F534" t="s">
+        <v>2746</v>
+      </c>
+      <c r="G534" t="s">
+        <v>2747</v>
+      </c>
+      <c r="H534" t="s">
+        <v>716</v>
+      </c>
+      <c r="I534" t="s">
+        <v>2748</v>
+      </c>
+      <c r="J534" t="s">
+        <v>484</v>
+      </c>
+      <c r="K534" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L534" t="s">
+        <v>2749</v>
+      </c>
+    </row>
+    <row r="535" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A535">
+        <v>534</v>
+      </c>
+      <c r="B535" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C535" t="s">
+        <v>14</v>
+      </c>
+      <c r="D535" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E535" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F535" t="s">
+        <v>2750</v>
+      </c>
+      <c r="G535" t="s">
+        <v>2751</v>
+      </c>
+      <c r="H535" t="s">
+        <v>716</v>
+      </c>
+      <c r="I535" t="s">
+        <v>2752</v>
+      </c>
+      <c r="J535" t="s">
+        <v>484</v>
+      </c>
+      <c r="K535" t="s">
+        <v>2753</v>
+      </c>
+      <c r="L535" t="s">
+        <v>2754</v>
+      </c>
+    </row>
+    <row r="536" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A536">
+        <v>535</v>
+      </c>
+      <c r="B536" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C536" t="s">
+        <v>14</v>
+      </c>
+      <c r="D536" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E536" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F536" t="s">
+        <v>2755</v>
+      </c>
+      <c r="G536" t="s">
+        <v>2756</v>
+      </c>
+      <c r="H536" t="s">
+        <v>290</v>
+      </c>
+      <c r="I536" t="s">
+        <v>2757</v>
+      </c>
+      <c r="J536" t="s">
+        <v>1897</v>
+      </c>
+      <c r="K536" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L536" t="s">
+        <v>2758</v>
+      </c>
+    </row>
+    <row r="537" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A537">
+        <v>536</v>
+      </c>
+      <c r="B537" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C537" t="s">
+        <v>14</v>
+      </c>
+      <c r="D537" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E537" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F537" t="s">
+        <v>2759</v>
+      </c>
+      <c r="G537" t="s">
+        <v>2760</v>
+      </c>
+      <c r="H537" t="s">
+        <v>273</v>
+      </c>
+      <c r="I537" t="s">
+        <v>2761</v>
+      </c>
+      <c r="J537" t="s">
+        <v>2762</v>
+      </c>
+      <c r="K537" t="s">
+        <v>2763</v>
+      </c>
+      <c r="L537" t="s">
+        <v>2764</v>
+      </c>
+    </row>
+    <row r="538" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A538">
+        <v>537</v>
+      </c>
+      <c r="B538" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C538" t="s">
+        <v>14</v>
+      </c>
+      <c r="D538" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E538" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F538" t="s">
+        <v>2765</v>
+      </c>
+      <c r="G538" t="s">
+        <v>2766</v>
+      </c>
+      <c r="H538" t="s">
+        <v>380</v>
+      </c>
+      <c r="I538" t="s">
+        <v>2767</v>
+      </c>
+      <c r="J538" t="s">
+        <v>356</v>
+      </c>
+      <c r="K538" t="s">
+        <v>2768</v>
+      </c>
+      <c r="L538" t="s">
+        <v>2769</v>
+      </c>
+    </row>
+    <row r="539" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A539">
+        <v>538</v>
+      </c>
+      <c r="B539" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C539" t="s">
+        <v>14</v>
+      </c>
+      <c r="D539" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E539" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F539" t="s">
+        <v>2770</v>
+      </c>
+      <c r="G539" t="s">
+        <v>2771</v>
+      </c>
+      <c r="H539" t="s">
+        <v>380</v>
+      </c>
+      <c r="I539" t="s">
+        <v>2772</v>
+      </c>
+      <c r="J539" t="s">
+        <v>356</v>
+      </c>
+      <c r="K539" t="s">
+        <v>2773</v>
+      </c>
+      <c r="L539" t="s">
+        <v>2774</v>
+      </c>
+    </row>
+    <row r="540" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A540">
+        <v>539</v>
+      </c>
+      <c r="B540" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C540" t="s">
+        <v>14</v>
+      </c>
+      <c r="D540" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E540" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F540" t="s">
+        <v>2775</v>
+      </c>
+      <c r="G540" t="s">
+        <v>2776</v>
+      </c>
+      <c r="H540" t="s">
+        <v>343</v>
+      </c>
+      <c r="I540" t="s">
+        <v>2777</v>
+      </c>
+      <c r="J540" t="s">
+        <v>103</v>
+      </c>
+      <c r="K540" t="s">
+        <v>2778</v>
+      </c>
+      <c r="L540" t="s">
+        <v>2779</v>
+      </c>
+    </row>
+    <row r="541" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A541">
+        <v>540</v>
+      </c>
+      <c r="B541" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C541" t="s">
+        <v>14</v>
+      </c>
+      <c r="D541" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E541" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F541" t="s">
+        <v>2780</v>
+      </c>
+      <c r="G541" t="s">
+        <v>2781</v>
+      </c>
+      <c r="H541" t="s">
+        <v>370</v>
+      </c>
+      <c r="I541" t="s">
+        <v>2782</v>
+      </c>
+      <c r="J541" t="s">
+        <v>419</v>
+      </c>
+      <c r="K541" t="s">
+        <v>2783</v>
+      </c>
+      <c r="L541" t="s">
+        <v>2784</v>
+      </c>
+    </row>
+    <row r="542" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A542">
+        <v>541</v>
+      </c>
+      <c r="B542" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C542" t="s">
+        <v>14</v>
+      </c>
+      <c r="D542" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E542" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F542" t="s">
+        <v>2785</v>
+      </c>
+      <c r="G542" t="s">
+        <v>2786</v>
+      </c>
+      <c r="H542" t="s">
+        <v>370</v>
+      </c>
+      <c r="I542" t="s">
+        <v>2787</v>
+      </c>
+      <c r="J542" t="s">
+        <v>419</v>
+      </c>
+      <c r="K542" t="s">
+        <v>2788</v>
+      </c>
+      <c r="L542" t="s">
+        <v>2789</v>
+      </c>
+    </row>
+    <row r="543" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A543">
+        <v>542</v>
+      </c>
+      <c r="B543" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C543" t="s">
+        <v>14</v>
+      </c>
+      <c r="D543" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E543" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F543" t="s">
+        <v>2790</v>
+      </c>
+      <c r="G543" t="s">
+        <v>2791</v>
+      </c>
+      <c r="H543" t="s">
+        <v>370</v>
+      </c>
+      <c r="I543" t="s">
+        <v>2792</v>
+      </c>
+      <c r="J543" t="s">
+        <v>419</v>
+      </c>
+      <c r="K543" t="s">
+        <v>2793</v>
+      </c>
+      <c r="L543" t="s">
+        <v>2794</v>
+      </c>
+    </row>
+    <row r="544" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A544">
+        <v>543</v>
+      </c>
+      <c r="B544" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C544" t="s">
+        <v>14</v>
+      </c>
+      <c r="D544" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E544" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F544" t="s">
+        <v>2795</v>
+      </c>
+      <c r="G544" t="s">
+        <v>2796</v>
+      </c>
+      <c r="H544" t="s">
+        <v>370</v>
+      </c>
+      <c r="I544" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J544" t="s">
+        <v>419</v>
+      </c>
+      <c r="K544" t="s">
+        <v>2797</v>
+      </c>
+      <c r="L544" t="s">
+        <v>2798</v>
+      </c>
+    </row>
+    <row r="545" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A545">
+        <v>544</v>
+      </c>
+      <c r="B545" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C545" t="s">
+        <v>14</v>
+      </c>
+      <c r="D545" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E545" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F545" t="s">
+        <v>2799</v>
+      </c>
+      <c r="G545" t="s">
+        <v>2800</v>
+      </c>
+      <c r="H545" t="s">
+        <v>370</v>
+      </c>
+      <c r="I545" t="s">
+        <v>2801</v>
+      </c>
+      <c r="J545" t="s">
+        <v>419</v>
+      </c>
+      <c r="K545" t="s">
+        <v>2802</v>
+      </c>
+      <c r="L545" t="s">
+        <v>2803</v>
+      </c>
+    </row>
+    <row r="546" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A546">
+        <v>545</v>
+      </c>
+      <c r="B546" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C546" t="s">
+        <v>14</v>
+      </c>
+      <c r="D546" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E546" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F546" t="s">
+        <v>2804</v>
+      </c>
+      <c r="G546" t="s">
+        <v>2805</v>
+      </c>
+      <c r="H546" t="s">
+        <v>2443</v>
+      </c>
+      <c r="I546" t="s">
+        <v>2806</v>
+      </c>
+      <c r="J546" t="s">
+        <v>333</v>
+      </c>
+      <c r="K546" t="s">
+        <v>2807</v>
+      </c>
+      <c r="L546" t="s">
+        <v>2808</v>
+      </c>
+    </row>
+    <row r="547" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A547">
+        <v>546</v>
+      </c>
+      <c r="B547" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C547" t="s">
+        <v>14</v>
+      </c>
+      <c r="D547" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E547" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F547" t="s">
+        <v>2809</v>
+      </c>
+      <c r="G547" t="s">
+        <v>2810</v>
+      </c>
+      <c r="H547" t="s">
+        <v>2443</v>
+      </c>
+      <c r="I547" t="s">
+        <v>2811</v>
+      </c>
+      <c r="J547" t="s">
+        <v>333</v>
+      </c>
+      <c r="K547" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L547" t="s">
+        <v>2812</v>
+      </c>
+    </row>
+    <row r="548" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A548">
+        <v>547</v>
+      </c>
+      <c r="B548" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C548" t="s">
+        <v>14</v>
+      </c>
+      <c r="D548" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E548" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F548" t="s">
+        <v>2813</v>
+      </c>
+      <c r="G548" t="s">
+        <v>2814</v>
+      </c>
+      <c r="H548" t="s">
+        <v>428</v>
+      </c>
+      <c r="I548" t="s">
+        <v>2815</v>
+      </c>
+      <c r="J548" t="s">
+        <v>460</v>
+      </c>
+      <c r="K548" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L548" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="549" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A549">
+        <v>548</v>
+      </c>
+      <c r="B549" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C549" t="s">
+        <v>14</v>
+      </c>
+      <c r="D549" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E549" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F549" t="s">
+        <v>2817</v>
+      </c>
+      <c r="G549" t="s">
+        <v>2818</v>
+      </c>
+      <c r="H549" t="s">
+        <v>428</v>
+      </c>
+      <c r="I549" t="s">
+        <v>2819</v>
+      </c>
+      <c r="J549" t="s">
+        <v>460</v>
+      </c>
+      <c r="K549" t="s">
+        <v>2820</v>
+      </c>
+      <c r="L549" t="s">
+        <v>2821</v>
+      </c>
+    </row>
+    <row r="550" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A550">
+        <v>549</v>
+      </c>
+      <c r="B550" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C550" t="s">
+        <v>14</v>
+      </c>
+      <c r="D550" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E550" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F550" t="s">
+        <v>2822</v>
+      </c>
+      <c r="G550" t="s">
+        <v>2823</v>
+      </c>
+      <c r="H550" t="s">
+        <v>428</v>
+      </c>
+      <c r="I550" t="s">
+        <v>2824</v>
+      </c>
+      <c r="J550" t="s">
+        <v>460</v>
+      </c>
+      <c r="K550" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L550" t="s">
+        <v>2825</v>
+      </c>
+    </row>
+    <row r="551" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A551">
+        <v>550</v>
+      </c>
+      <c r="B551" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C551" t="s">
+        <v>14</v>
+      </c>
+      <c r="D551" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E551" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F551" t="s">
+        <v>2826</v>
+      </c>
+      <c r="G551" t="s">
+        <v>2827</v>
+      </c>
+      <c r="H551" t="s">
+        <v>428</v>
+      </c>
+      <c r="I551" t="s">
+        <v>2828</v>
+      </c>
+      <c r="J551" t="s">
+        <v>460</v>
+      </c>
+      <c r="K551" t="s">
+        <v>2829</v>
+      </c>
+      <c r="L551" t="s">
+        <v>2830</v>
+      </c>
+    </row>
+    <row r="552" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A552">
+        <v>551</v>
+      </c>
+      <c r="B552" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C552" t="s">
+        <v>14</v>
+      </c>
+      <c r="D552" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E552" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F552" t="s">
+        <v>2831</v>
+      </c>
+      <c r="G552" t="s">
+        <v>2832</v>
+      </c>
+      <c r="H552" t="s">
+        <v>428</v>
+      </c>
+      <c r="I552" t="s">
+        <v>2833</v>
+      </c>
+      <c r="J552" t="s">
+        <v>460</v>
+      </c>
+      <c r="K552" t="s">
+        <v>2834</v>
+      </c>
+      <c r="L552" t="s">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="553" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A553">
+        <v>552</v>
+      </c>
+      <c r="B553" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C553" t="s">
+        <v>14</v>
+      </c>
+      <c r="D553" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E553" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F553" t="s">
+        <v>2836</v>
+      </c>
+      <c r="G553" t="s">
+        <v>2837</v>
+      </c>
+      <c r="H553" t="s">
+        <v>428</v>
+      </c>
+      <c r="I553" t="s">
+        <v>2838</v>
+      </c>
+      <c r="J553" t="s">
+        <v>460</v>
+      </c>
+      <c r="K553" t="s">
+        <v>2839</v>
+      </c>
+      <c r="L553" t="s">
+        <v>2840</v>
+      </c>
+    </row>
+    <row r="554" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A554">
+        <v>553</v>
+      </c>
+      <c r="B554" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C554" t="s">
+        <v>14</v>
+      </c>
+      <c r="D554" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E554" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F554" t="s">
+        <v>2841</v>
+      </c>
+      <c r="G554" t="s">
+        <v>2842</v>
+      </c>
+      <c r="H554" t="s">
+        <v>428</v>
+      </c>
+      <c r="I554" t="s">
+        <v>2843</v>
+      </c>
+      <c r="J554" t="s">
+        <v>460</v>
+      </c>
+      <c r="K554" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L554" t="s">
+        <v>2844</v>
+      </c>
+    </row>
+    <row r="555" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A555">
+        <v>554</v>
+      </c>
+      <c r="B555" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C555" t="s">
+        <v>14</v>
+      </c>
+      <c r="D555" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E555" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F555" t="s">
+        <v>2845</v>
+      </c>
+      <c r="G555" t="s">
+        <v>2846</v>
+      </c>
+      <c r="H555" t="s">
+        <v>343</v>
+      </c>
+      <c r="I555" t="s">
+        <v>2847</v>
+      </c>
+      <c r="J555" t="s">
+        <v>103</v>
+      </c>
+      <c r="K555" t="s">
+        <v>2848</v>
+      </c>
+      <c r="L555" t="s">
+        <v>2849</v>
+      </c>
+    </row>
+    <row r="556" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A556">
+        <v>555</v>
+      </c>
+      <c r="B556" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C556" t="s">
+        <v>14</v>
+      </c>
+      <c r="D556" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E556" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F556" t="s">
+        <v>2850</v>
+      </c>
+      <c r="G556" t="s">
+        <v>2851</v>
+      </c>
+      <c r="H556" t="s">
+        <v>428</v>
+      </c>
+      <c r="I556" t="s">
+        <v>2852</v>
+      </c>
+      <c r="J556" t="s">
+        <v>460</v>
+      </c>
+      <c r="K556" t="s">
+        <v>2853</v>
+      </c>
+      <c r="L556" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="557" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A557">
+        <v>556</v>
+      </c>
+      <c r="B557" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C557" t="s">
+        <v>14</v>
+      </c>
+      <c r="D557" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E557" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F557" t="s">
+        <v>2855</v>
+      </c>
+      <c r="G557" t="s">
+        <v>2856</v>
+      </c>
+      <c r="H557" t="s">
+        <v>428</v>
+      </c>
+      <c r="I557" t="s">
+        <v>2857</v>
+      </c>
+      <c r="J557" t="s">
+        <v>460</v>
+      </c>
+      <c r="K557" t="s">
+        <v>2858</v>
+      </c>
+      <c r="L557" t="s">
+        <v>2859</v>
+      </c>
+    </row>
+    <row r="558" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A558">
+        <v>557</v>
+      </c>
+      <c r="B558" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C558" t="s">
+        <v>14</v>
+      </c>
+      <c r="D558" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E558" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F558" t="s">
+        <v>2860</v>
+      </c>
+      <c r="G558" t="s">
+        <v>2861</v>
+      </c>
+      <c r="H558" t="s">
+        <v>428</v>
+      </c>
+      <c r="I558" t="s">
+        <v>2862</v>
+      </c>
+      <c r="J558" t="s">
+        <v>460</v>
+      </c>
+      <c r="K558" t="s">
+        <v>2863</v>
+      </c>
+      <c r="L558" t="s">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="559" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A559">
+        <v>558</v>
+      </c>
+      <c r="B559" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C559" t="s">
+        <v>14</v>
+      </c>
+      <c r="D559" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E559" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F559" t="s">
+        <v>2865</v>
+      </c>
+      <c r="G559" t="s">
+        <v>2866</v>
+      </c>
+      <c r="H559" t="s">
+        <v>428</v>
+      </c>
+      <c r="I559" t="s">
+        <v>2867</v>
+      </c>
+      <c r="J559" t="s">
+        <v>460</v>
+      </c>
+      <c r="K559" t="s">
+        <v>2868</v>
+      </c>
+      <c r="L559" t="s">
+        <v>2869</v>
+      </c>
+    </row>
+    <row r="560" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A560">
+        <v>559</v>
+      </c>
+      <c r="B560" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C560" t="s">
+        <v>14</v>
+      </c>
+      <c r="D560" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E560" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F560" t="s">
+        <v>2870</v>
+      </c>
+      <c r="G560" t="s">
+        <v>2871</v>
+      </c>
+      <c r="H560" t="s">
+        <v>428</v>
+      </c>
+      <c r="I560" t="s">
+        <v>2872</v>
+      </c>
+      <c r="J560" t="s">
+        <v>460</v>
+      </c>
+      <c r="K560" t="s">
+        <v>2873</v>
+      </c>
+      <c r="L560" t="s">
+        <v>2874</v>
+      </c>
+    </row>
+    <row r="561" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A561">
+        <v>560</v>
+      </c>
+      <c r="B561" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C561" t="s">
+        <v>14</v>
+      </c>
+      <c r="D561" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E561" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F561" t="s">
+        <v>2875</v>
+      </c>
+      <c r="G561" t="s">
+        <v>2876</v>
+      </c>
+      <c r="H561" t="s">
+        <v>428</v>
+      </c>
+      <c r="I561" t="s">
+        <v>2877</v>
+      </c>
+      <c r="J561" t="s">
+        <v>460</v>
+      </c>
+      <c r="K561" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L561" t="s">
+        <v>2878</v>
+      </c>
+    </row>
+    <row r="562" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A562">
+        <v>561</v>
+      </c>
+      <c r="B562" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C562" t="s">
+        <v>14</v>
+      </c>
+      <c r="D562" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E562" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F562" t="s">
+        <v>2879</v>
+      </c>
+      <c r="G562" t="s">
+        <v>2880</v>
+      </c>
+      <c r="H562" t="s">
+        <v>428</v>
+      </c>
+      <c r="I562" t="s">
+        <v>2881</v>
+      </c>
+      <c r="J562" t="s">
+        <v>460</v>
+      </c>
+      <c r="K562" t="s">
+        <v>2882</v>
+      </c>
+      <c r="L562" t="s">
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="563" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A563">
+        <v>562</v>
+      </c>
+      <c r="B563" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C563" t="s">
+        <v>14</v>
+      </c>
+      <c r="D563" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E563" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F563" t="s">
+        <v>2884</v>
+      </c>
+      <c r="G563" t="s">
+        <v>2885</v>
+      </c>
+      <c r="H563" t="s">
+        <v>428</v>
+      </c>
+      <c r="I563" t="s">
+        <v>2886</v>
+      </c>
+      <c r="J563" t="s">
+        <v>460</v>
+      </c>
+      <c r="K563" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L563" t="s">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="564" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A564">
+        <v>563</v>
+      </c>
+      <c r="B564" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C564" t="s">
+        <v>14</v>
+      </c>
+      <c r="D564" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E564" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F564" t="s">
+        <v>2888</v>
+      </c>
+      <c r="G564" t="s">
+        <v>2889</v>
+      </c>
+      <c r="H564" t="s">
+        <v>428</v>
+      </c>
+      <c r="I564" t="s">
+        <v>2890</v>
+      </c>
+      <c r="J564" t="s">
+        <v>460</v>
+      </c>
+      <c r="K564" t="s">
+        <v>2891</v>
+      </c>
+      <c r="L564" t="s">
+        <v>2892</v>
+      </c>
+    </row>
+    <row r="565" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A565">
+        <v>564</v>
+      </c>
+      <c r="B565" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C565" t="s">
+        <v>14</v>
+      </c>
+      <c r="D565" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E565" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F565" t="s">
+        <v>2893</v>
+      </c>
+      <c r="G565" t="s">
+        <v>2894</v>
+      </c>
+      <c r="H565" t="s">
+        <v>428</v>
+      </c>
+      <c r="I565" t="s">
+        <v>2895</v>
+      </c>
+      <c r="J565" t="s">
+        <v>460</v>
+      </c>
+      <c r="K565" t="s">
+        <v>2896</v>
+      </c>
+      <c r="L565" t="s">
+        <v>2897</v>
+      </c>
+    </row>
+    <row r="566" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A566">
+        <v>565</v>
+      </c>
+      <c r="B566" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C566" t="s">
+        <v>14</v>
+      </c>
+      <c r="D566" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E566" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F566" t="s">
+        <v>2898</v>
+      </c>
+      <c r="G566" t="s">
+        <v>2899</v>
+      </c>
+      <c r="H566" t="s">
+        <v>428</v>
+      </c>
+      <c r="I566" t="s">
+        <v>2900</v>
+      </c>
+      <c r="J566" t="s">
+        <v>460</v>
+      </c>
+      <c r="K566" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L566" t="s">
+        <v>2901</v>
+      </c>
+    </row>
+    <row r="567" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A567">
+        <v>566</v>
+      </c>
+      <c r="B567" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C567" t="s">
+        <v>14</v>
+      </c>
+      <c r="D567" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E567" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F567" t="s">
+        <v>2902</v>
+      </c>
+      <c r="G567" t="s">
+        <v>2903</v>
+      </c>
+      <c r="H567" t="s">
+        <v>343</v>
+      </c>
+      <c r="I567" t="s">
+        <v>2904</v>
+      </c>
+      <c r="J567" t="s">
+        <v>103</v>
+      </c>
+      <c r="K567" t="s">
+        <v>2905</v>
+      </c>
+      <c r="L567" t="s">
+        <v>2906</v>
+      </c>
+    </row>
+    <row r="568" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A568">
+        <v>567</v>
+      </c>
+      <c r="B568" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C568" t="s">
+        <v>14</v>
+      </c>
+      <c r="D568" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E568" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F568" t="s">
+        <v>2907</v>
+      </c>
+      <c r="G568" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H568" t="s">
+        <v>343</v>
+      </c>
+      <c r="I568" t="s">
+        <v>2909</v>
+      </c>
+      <c r="J568" t="s">
+        <v>268</v>
+      </c>
+      <c r="K568" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L568" t="s">
+        <v>2910</v>
+      </c>
+    </row>
+    <row r="569" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A569">
+        <v>568</v>
+      </c>
+      <c r="B569" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C569" t="s">
+        <v>14</v>
+      </c>
+      <c r="D569" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E569" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F569" t="s">
+        <v>2911</v>
+      </c>
+      <c r="G569" t="s">
+        <v>2912</v>
+      </c>
+      <c r="H569" t="s">
+        <v>343</v>
+      </c>
+      <c r="I569" t="s">
+        <v>2913</v>
+      </c>
+      <c r="J569" t="s">
+        <v>268</v>
+      </c>
+      <c r="K569" t="s">
+        <v>2914</v>
+      </c>
+      <c r="L569" t="s">
+        <v>2915</v>
+      </c>
+    </row>
+    <row r="570" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K570" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L570" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="571" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K571" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L571" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="572" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K572" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L572" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="573" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K573" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L573" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="574" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K574" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L574" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="575" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K575" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L575" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="576" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="E576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="F576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="J576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="K576" t="s">
+        <v>2577</v>
+      </c>
+      <c r="L576" t="s">
+        <v>2577</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(leads): mark next 10 outreach sends contacted
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -9980,7 +9980,7 @@
         <v>252</v>
       </c>
       <c r="B253" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C253" t="str">
         <v>Weak</v>
@@ -10018,7 +10018,7 @@
         <v>253</v>
       </c>
       <c r="B254" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C254" t="str">
         <v>Weak</v>
@@ -10056,7 +10056,7 @@
         <v>254</v>
       </c>
       <c r="B255" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C255" t="str">
         <v>Weak</v>
@@ -10094,7 +10094,7 @@
         <v>255</v>
       </c>
       <c r="B256" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C256" t="str">
         <v>Weak</v>
@@ -10132,7 +10132,7 @@
         <v>256</v>
       </c>
       <c r="B257" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C257" t="str">
         <v>Weak</v>
@@ -10170,7 +10170,7 @@
         <v>257</v>
       </c>
       <c r="B258" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C258" t="str">
         <v>Weak</v>
@@ -10208,7 +10208,7 @@
         <v>258</v>
       </c>
       <c r="B259" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C259" t="str">
         <v>Weak</v>
@@ -10246,7 +10246,7 @@
         <v>259</v>
       </c>
       <c r="B260" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C260" t="str">
         <v>Weak</v>
@@ -10284,7 +10284,7 @@
         <v>260</v>
       </c>
       <c r="B261" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C261" t="str">
         <v>Weak</v>
@@ -10322,7 +10322,7 @@
         <v>261</v>
       </c>
       <c r="B262" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C262" t="str">
         <v>Weak</v>

</xml_diff>

<commit_message>
Add 39 OSM leads to WebKreatives workbook
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7365" uniqueCount="4142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7794" uniqueCount="4322">
   <si>
     <t>#</t>
   </si>
@@ -12437,6 +12437,546 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:2239473797 | Source: OpenStreetMap | bakkerij | Breda | Website: https://trumpitime.foodticket.nl</t>
+  </si>
+  <si>
+    <t>info@bakkerijlips.nl</t>
+  </si>
+  <si>
+    <t>Brood- en Banket bakkerij Lips</t>
+  </si>
+  <si>
+    <t>Dreef 4813ED</t>
+  </si>
+  <si>
+    <t>+31 76 521 1415</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2728029858 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.bakkerijlips.nl</t>
+  </si>
+  <si>
+    <t>p.bogaert@ziggo.nl</t>
+  </si>
+  <si>
+    <t>Pol van den Bogaert</t>
+  </si>
+  <si>
+    <t>+31 76 521 1340</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2728035608 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.bakkervandenbogaert.nl</t>
+  </si>
+  <si>
+    <t>info@fogobakehouse.nl</t>
+  </si>
+  <si>
+    <t>FOGO Bakehouse</t>
+  </si>
+  <si>
+    <t>Heuvelstraat 4812PH</t>
+  </si>
+  <si>
+    <t>+31 6 45116878</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2728037308 | Source: OpenStreetMap | bakkerij | Breda | Website: https://fogobakehouse.nl</t>
+  </si>
+  <si>
+    <t>info@asyabakkerij.nl</t>
+  </si>
+  <si>
+    <t>ASYA Bakkerij</t>
+  </si>
+  <si>
+    <t>Epelenberg 4817CM</t>
+  </si>
+  <si>
+    <t>+31 76 515 4048</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2730848943 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.asyabakkerij.nl</t>
+  </si>
+  <si>
+    <t>info@bakkerwim.com</t>
+  </si>
+  <si>
+    <t>Bakker Wim</t>
+  </si>
+  <si>
+    <t>Oranjeboomstraat 4814EG</t>
+  </si>
+  <si>
+    <t>+31 76 522 2866</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2730882514 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.bakkerwim.com</t>
+  </si>
+  <si>
+    <t>teteringen@dejongdeli.nl</t>
+  </si>
+  <si>
+    <t>De Jong Deli</t>
+  </si>
+  <si>
+    <t>Nieuwe Boschstraat 4811CW</t>
+  </si>
+  <si>
+    <t>+31 76 521 7467</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2731463509 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.dejongdeli.nl</t>
+  </si>
+  <si>
+    <t>info@back-werk.nl</t>
+  </si>
+  <si>
+    <t>Backwerk</t>
+  </si>
+  <si>
+    <t>Ridderstraat 4811JA</t>
+  </si>
+  <si>
+    <t>+31 35 221 0001</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2731476211 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.back-werk.nl</t>
+  </si>
+  <si>
+    <t>info@bakkertjebol.nl</t>
+  </si>
+  <si>
+    <t>Bakkertje Bol</t>
+  </si>
+  <si>
+    <t>Karrestraat 4811WT</t>
+  </si>
+  <si>
+    <t>+31 76 303 6250</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2731485460 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.bakkertjebol.nl</t>
+  </si>
+  <si>
+    <t>info@echt-brood.nl</t>
+  </si>
+  <si>
+    <t>Echt Brood</t>
+  </si>
+  <si>
+    <t>Boschstraat 4811GH</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2731486700 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.echt-brood.com</t>
+  </si>
+  <si>
+    <t>van.disseldorp@echtebakker.nl</t>
+  </si>
+  <si>
+    <t>van Disseldorp</t>
+  </si>
+  <si>
+    <t>Kloosterstraat 4854CM</t>
+  </si>
+  <si>
+    <t>Bavel</t>
+  </si>
+  <si>
+    <t>+31 161 437 036</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2731990145 | Source: OpenStreetMap | bakkerij | Breda | Website: https://bakkerijvandisseldorp.nl</t>
+  </si>
+  <si>
+    <t>info@bakkerijmenke.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij Menke</t>
+  </si>
+  <si>
+    <t>Valkeniersplein 4835RB</t>
+  </si>
+  <si>
+    <t>+31 76 561 1884</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2738788881 | Source: OpenStreetMap | bakkerij | Breda | Website: https://bakkerijmenke.nl</t>
+  </si>
+  <si>
+    <t>verkoop@vromansbakkers.nl</t>
+  </si>
+  <si>
+    <t>Vromans Bakkers</t>
+  </si>
+  <si>
+    <t>+31 76 303 0043</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2738791105 | Source: OpenStreetMap | bakkerij | Breda | Website: https://vromansbakkers.nl</t>
+  </si>
+  <si>
+    <t>ebrord@bakkershuys.info</t>
+  </si>
+  <si>
+    <t>Bakkershuys</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:4261393604 | Source: OpenStreetMap | bakkerij | Breda | Website: https://bakkershuys.info</t>
+  </si>
+  <si>
+    <t>bakkerijvromans@planet.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij Vromans</t>
+  </si>
+  <si>
+    <t>Lunenburgstraat 4834HG</t>
+  </si>
+  <si>
+    <t>+31 76 565 3682</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:4494103501 | Source: OpenStreetMap | bakkerij | Breda | Website: https://bakkerijvromans.nl</t>
+  </si>
+  <si>
+    <t>rijngoos@live.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij Rijngoos</t>
+  </si>
+  <si>
+    <t>+31 76 565 4464</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:4494103575 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.bakkerrijngoos.nl/nl-nl</t>
+  </si>
+  <si>
+    <t>ginnekenweg@supersandwich.nl</t>
+  </si>
+  <si>
+    <t>Super Sandwich Broodjeswinkel</t>
+  </si>
+  <si>
+    <t>+31 76 514 0031</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:5490940566 | Source: OpenStreetMap | bakkerij | Breda | Website: https://www.supersandwich.nl</t>
+  </si>
+  <si>
+    <t>bakkerijelsevier@hetnet.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij Elsevier</t>
+  </si>
+  <si>
+    <t>+31 76 514 2845</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:5494083283 | Source: OpenStreetMap | bakkerij | Breda | Website: https://bakkerijelsevier.nl</t>
+  </si>
+  <si>
+    <t>info@violien.nl</t>
+  </si>
+  <si>
+    <t>Violien</t>
+  </si>
+  <si>
+    <t>Haagweg 4813XG</t>
+  </si>
+  <si>
+    <t>+31 76 522 6722</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2727961268 | Source: OpenStreetMap | bloemist | Breda | Website: https://www.violien.nl</t>
+  </si>
+  <si>
+    <t>support@thegreensubmarine.nl</t>
+  </si>
+  <si>
+    <t>The Green Submarine Plantenwinkel</t>
+  </si>
+  <si>
+    <t>+31 6 50 87 23 67</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2731554071 | Source: OpenStreetMap | bloemist | Breda | Website: https://www.thegreensubmarine.nl</t>
+  </si>
+  <si>
+    <t>info@bloembinderijoxalis.nl</t>
+  </si>
+  <si>
+    <t>Bloembinderij Oxalis</t>
+  </si>
+  <si>
+    <t>Pastoor Doensstraat 4854CP</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2731973535 | Source: OpenStreetMap | bloemist | Breda | Website: https://bloembinderijoxalis.nl</t>
+  </si>
+  <si>
+    <t>juffertje_in_t_groen@hotmail.com</t>
+  </si>
+  <si>
+    <t>Juffertje in 't Groen</t>
+  </si>
+  <si>
+    <t>+31 76 5413297</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2732468853 | Source: OpenStreetMap | bloemist | Breda | Website: https://www.juffertjeintgroen.com</t>
+  </si>
+  <si>
+    <t>info@ceesvaneijck.nl</t>
+  </si>
+  <si>
+    <t>Cees van Eijck</t>
+  </si>
+  <si>
+    <t>Generaal Maczekstraat 4818BV</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2738693586 | Source: OpenStreetMap | bloemist | Breda | Website: https://ceesvaneijck.nl</t>
+  </si>
+  <si>
+    <t>info@rosario-bloemen.nl</t>
+  </si>
+  <si>
+    <t>Rosario</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2738788069 | Source: OpenStreetMap | bloemist | Breda | Website: https://rosario-bloemen.nl</t>
+  </si>
+  <si>
+    <t>info@venvwonen.nl</t>
+  </si>
+  <si>
+    <t>V&amp;V Bloemen en Wonen</t>
+  </si>
+  <si>
+    <t>Ginnekenweg 4818JB</t>
+  </si>
+  <si>
+    <t>+31 76 521 6759</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2738794329 | Source: OpenStreetMap | bloemist | Breda | Website: https://www.venvbloemenenwonen.nl</t>
+  </si>
+  <si>
+    <t>info@loekinette.nl</t>
+  </si>
+  <si>
+    <t>Stomerij Loekinette</t>
+  </si>
+  <si>
+    <t>Nieuwe Ginnekenstraat 4811NS</t>
+  </si>
+  <si>
+    <t>+31 76 522 8184</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2731477449 | Source: OpenStreetMap | stomerij | Breda | Website: https://www.stomerijbreda.nl</t>
+  </si>
+  <si>
+    <t>kolibrie-stomerijen@planet.nl</t>
+  </si>
+  <si>
+    <t>Stomerij Kolibrie</t>
+  </si>
+  <si>
+    <t>+31 76 565 3143</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2735593226 | Source: OpenStreetMap | stomerij | Breda | Website: https://www.stomerijkolibrie.nl</t>
+  </si>
+  <si>
+    <t>charlotte@kapperdekrul.nl</t>
+  </si>
+  <si>
+    <t>Kapper de Krul</t>
+  </si>
+  <si>
+    <t>Laauwikstraat 6663CJ</t>
+  </si>
+  <si>
+    <t>Lent</t>
+  </si>
+  <si>
+    <t>+31 24 324 0903</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:417037326 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.kapperdekrul.nl</t>
+  </si>
+  <si>
+    <t>info@storadokappers.nl</t>
+  </si>
+  <si>
+    <t>Storado Kappers</t>
+  </si>
+  <si>
+    <t>Stijn Buysstraat 6512CR</t>
+  </si>
+  <si>
+    <t>+31 24 324 1989</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2093534152 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://storadokappers.nl</t>
+  </si>
+  <si>
+    <t>robinteunissen@hotmail.nl</t>
+  </si>
+  <si>
+    <t>Robin's Hair &amp; Beauty Salon</t>
+  </si>
+  <si>
+    <t>Laauwikstraat 6663CK</t>
+  </si>
+  <si>
+    <t>+31 24 322 0215</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2528510830 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://robinshairenbeautysalon.nl</t>
+  </si>
+  <si>
+    <t>info@alsaifbarber.nl</t>
+  </si>
+  <si>
+    <t>Alsaif Barber</t>
+  </si>
+  <si>
+    <t>Kanunnik Boenenstraat 6525WJ</t>
+  </si>
+  <si>
+    <t>+31 24 350 3126</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2826353634 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://alsaifbarber.nl</t>
+  </si>
+  <si>
+    <t>info@larosadecubakappers.nl</t>
+  </si>
+  <si>
+    <t>La Rosa de Cuba</t>
+  </si>
+  <si>
+    <t>Koolemans Beynenstraat 6521EX</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2829308862 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.larosadecubakappers.nl</t>
+  </si>
+  <si>
+    <t>info@djikappers.nl</t>
+  </si>
+  <si>
+    <t>Haarstudio Sara</t>
+  </si>
+  <si>
+    <t>Burghardt van den Berghstraat 6512DH</t>
+  </si>
+  <si>
+    <t>+31 24 324 3924</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2847291456 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.haarstudiosara.nl</t>
+  </si>
+  <si>
+    <t>nijmegen@salonflor.nl</t>
+  </si>
+  <si>
+    <t>Salon Flor</t>
+  </si>
+  <si>
+    <t>In de Betouwstraat 6511GC</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2847379019 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.salonflor.nl</t>
+  </si>
+  <si>
+    <t>info@noahkappers.nl</t>
+  </si>
+  <si>
+    <t>Noah Kappers</t>
+  </si>
+  <si>
+    <t>Willemsweg 6531DM</t>
+  </si>
+  <si>
+    <t>+31 6 34024487</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2848105276 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.noahkappers.nl</t>
+  </si>
+  <si>
+    <t>tkshairdresser@gmail.com</t>
+  </si>
+  <si>
+    <t>Zegt u het maar!</t>
+  </si>
+  <si>
+    <t>Hatertseweg 6533AD</t>
+  </si>
+  <si>
+    <t>+31 24 355 9044</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2848277361 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: http://zegtuhetmaar.info</t>
+  </si>
+  <si>
+    <t>info@mariobarbershop.nl</t>
+  </si>
+  <si>
+    <t>Mario Barbershop</t>
+  </si>
+  <si>
+    <t>Sint Jacobslaan 6533BS</t>
+  </si>
+  <si>
+    <t>+31 6 37623237</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2848283544 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.mariobarbershop.nl</t>
+  </si>
+  <si>
+    <t>info@rootzhairandcare.nl</t>
+  </si>
+  <si>
+    <t>Rootz Hair &amp; Care</t>
+  </si>
+  <si>
+    <t>Gemsstraat 6531TC</t>
+  </si>
+  <si>
+    <t>+31 24 355 4156</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2848314473 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.rootzhairandcare.nl</t>
+  </si>
+  <si>
+    <t>info@kapsalonxing.nl</t>
+  </si>
+  <si>
+    <t>Kapsalon Xing</t>
+  </si>
+  <si>
+    <t>Poemastraat 6531MH</t>
+  </si>
+  <si>
+    <t>+31 24 355 3836</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2848698381 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: http://www.kapsalonxing.nl</t>
+  </si>
+  <si>
+    <t>koopmankappers@ziggo.nl</t>
+  </si>
+  <si>
+    <t>Koopman Kappers</t>
+  </si>
+  <si>
+    <t>Oude Molenweg 6533WK</t>
+  </si>
+  <si>
+    <t>+31 24 377 2408</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2851803165 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.koopmankappers.nl</t>
   </si>
 </sst>
 </file>
@@ -12813,8 +13353,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L849"/>
-  <sheetFormatPr customHeight="1"/>
+  <dimension ref="A1:L888"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -39156,6 +39696,1488 @@
         <v>4141</v>
       </c>
     </row>
+    <row r="850" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A850">
+        <v>849</v>
+      </c>
+      <c r="B850" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C850" t="s">
+        <v>14</v>
+      </c>
+      <c r="D850" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E850" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F850" t="s">
+        <v>4142</v>
+      </c>
+      <c r="G850" t="s">
+        <v>4143</v>
+      </c>
+      <c r="H850" t="s">
+        <v>390</v>
+      </c>
+      <c r="I850" t="s">
+        <v>4144</v>
+      </c>
+      <c r="J850" t="s">
+        <v>356</v>
+      </c>
+      <c r="K850" t="s">
+        <v>4145</v>
+      </c>
+      <c r="L850" t="s">
+        <v>4146</v>
+      </c>
+    </row>
+    <row r="851" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A851">
+        <v>850</v>
+      </c>
+      <c r="B851" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C851" t="s">
+        <v>14</v>
+      </c>
+      <c r="D851" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E851" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F851" t="s">
+        <v>4147</v>
+      </c>
+      <c r="G851" t="s">
+        <v>4148</v>
+      </c>
+      <c r="H851" t="s">
+        <v>390</v>
+      </c>
+      <c r="I851" t="s">
+        <v>3885</v>
+      </c>
+      <c r="J851" t="s">
+        <v>356</v>
+      </c>
+      <c r="K851" t="s">
+        <v>4149</v>
+      </c>
+      <c r="L851" t="s">
+        <v>4150</v>
+      </c>
+    </row>
+    <row r="852" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A852">
+        <v>851</v>
+      </c>
+      <c r="B852" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C852" t="s">
+        <v>14</v>
+      </c>
+      <c r="D852" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E852" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F852" t="s">
+        <v>4151</v>
+      </c>
+      <c r="G852" t="s">
+        <v>4152</v>
+      </c>
+      <c r="H852" t="s">
+        <v>390</v>
+      </c>
+      <c r="I852" t="s">
+        <v>4153</v>
+      </c>
+      <c r="J852" t="s">
+        <v>356</v>
+      </c>
+      <c r="K852" t="s">
+        <v>4154</v>
+      </c>
+      <c r="L852" t="s">
+        <v>4155</v>
+      </c>
+    </row>
+    <row r="853" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A853">
+        <v>852</v>
+      </c>
+      <c r="B853" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C853" t="s">
+        <v>14</v>
+      </c>
+      <c r="D853" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E853" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F853" t="s">
+        <v>4156</v>
+      </c>
+      <c r="G853" t="s">
+        <v>4157</v>
+      </c>
+      <c r="H853" t="s">
+        <v>390</v>
+      </c>
+      <c r="I853" t="s">
+        <v>4158</v>
+      </c>
+      <c r="J853" t="s">
+        <v>356</v>
+      </c>
+      <c r="K853" t="s">
+        <v>4159</v>
+      </c>
+      <c r="L853" t="s">
+        <v>4160</v>
+      </c>
+    </row>
+    <row r="854" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A854">
+        <v>853</v>
+      </c>
+      <c r="B854" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C854" t="s">
+        <v>14</v>
+      </c>
+      <c r="D854" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E854" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F854" t="s">
+        <v>4161</v>
+      </c>
+      <c r="G854" t="s">
+        <v>4162</v>
+      </c>
+      <c r="H854" t="s">
+        <v>390</v>
+      </c>
+      <c r="I854" t="s">
+        <v>4163</v>
+      </c>
+      <c r="J854" t="s">
+        <v>356</v>
+      </c>
+      <c r="K854" t="s">
+        <v>4164</v>
+      </c>
+      <c r="L854" t="s">
+        <v>4165</v>
+      </c>
+    </row>
+    <row r="855" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A855">
+        <v>854</v>
+      </c>
+      <c r="B855" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C855" t="s">
+        <v>14</v>
+      </c>
+      <c r="D855" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E855" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F855" t="s">
+        <v>4166</v>
+      </c>
+      <c r="G855" t="s">
+        <v>4167</v>
+      </c>
+      <c r="H855" t="s">
+        <v>390</v>
+      </c>
+      <c r="I855" t="s">
+        <v>4168</v>
+      </c>
+      <c r="J855" t="s">
+        <v>356</v>
+      </c>
+      <c r="K855" t="s">
+        <v>4169</v>
+      </c>
+      <c r="L855" t="s">
+        <v>4170</v>
+      </c>
+    </row>
+    <row r="856" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A856">
+        <v>855</v>
+      </c>
+      <c r="B856" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C856" t="s">
+        <v>14</v>
+      </c>
+      <c r="D856" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E856" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F856" t="s">
+        <v>4171</v>
+      </c>
+      <c r="G856" t="s">
+        <v>4172</v>
+      </c>
+      <c r="H856" t="s">
+        <v>390</v>
+      </c>
+      <c r="I856" t="s">
+        <v>4173</v>
+      </c>
+      <c r="J856" t="s">
+        <v>356</v>
+      </c>
+      <c r="K856" t="s">
+        <v>4174</v>
+      </c>
+      <c r="L856" t="s">
+        <v>4175</v>
+      </c>
+    </row>
+    <row r="857" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A857">
+        <v>856</v>
+      </c>
+      <c r="B857" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C857" t="s">
+        <v>14</v>
+      </c>
+      <c r="D857" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E857" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F857" t="s">
+        <v>4176</v>
+      </c>
+      <c r="G857" t="s">
+        <v>4177</v>
+      </c>
+      <c r="H857" t="s">
+        <v>390</v>
+      </c>
+      <c r="I857" t="s">
+        <v>4178</v>
+      </c>
+      <c r="J857" t="s">
+        <v>356</v>
+      </c>
+      <c r="K857" t="s">
+        <v>4179</v>
+      </c>
+      <c r="L857" t="s">
+        <v>4180</v>
+      </c>
+    </row>
+    <row r="858" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A858">
+        <v>857</v>
+      </c>
+      <c r="B858" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C858" t="s">
+        <v>14</v>
+      </c>
+      <c r="D858" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E858" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F858" t="s">
+        <v>4181</v>
+      </c>
+      <c r="G858" t="s">
+        <v>4182</v>
+      </c>
+      <c r="H858" t="s">
+        <v>390</v>
+      </c>
+      <c r="I858" t="s">
+        <v>4183</v>
+      </c>
+      <c r="J858" t="s">
+        <v>356</v>
+      </c>
+      <c r="K858" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L858" t="s">
+        <v>4184</v>
+      </c>
+    </row>
+    <row r="859" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A859">
+        <v>858</v>
+      </c>
+      <c r="B859" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C859" t="s">
+        <v>14</v>
+      </c>
+      <c r="D859" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E859" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F859" t="s">
+        <v>4185</v>
+      </c>
+      <c r="G859" t="s">
+        <v>4186</v>
+      </c>
+      <c r="H859" t="s">
+        <v>390</v>
+      </c>
+      <c r="I859" t="s">
+        <v>4187</v>
+      </c>
+      <c r="J859" t="s">
+        <v>4188</v>
+      </c>
+      <c r="K859" t="s">
+        <v>4189</v>
+      </c>
+      <c r="L859" t="s">
+        <v>4190</v>
+      </c>
+    </row>
+    <row r="860" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A860">
+        <v>859</v>
+      </c>
+      <c r="B860" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C860" t="s">
+        <v>14</v>
+      </c>
+      <c r="D860" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E860" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F860" t="s">
+        <v>4191</v>
+      </c>
+      <c r="G860" t="s">
+        <v>4192</v>
+      </c>
+      <c r="H860" t="s">
+        <v>390</v>
+      </c>
+      <c r="I860" t="s">
+        <v>4193</v>
+      </c>
+      <c r="J860" t="s">
+        <v>356</v>
+      </c>
+      <c r="K860" t="s">
+        <v>4194</v>
+      </c>
+      <c r="L860" t="s">
+        <v>4195</v>
+      </c>
+    </row>
+    <row r="861" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A861">
+        <v>860</v>
+      </c>
+      <c r="B861" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C861" t="s">
+        <v>14</v>
+      </c>
+      <c r="D861" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E861" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F861" t="s">
+        <v>4196</v>
+      </c>
+      <c r="G861" t="s">
+        <v>4197</v>
+      </c>
+      <c r="H861" t="s">
+        <v>390</v>
+      </c>
+      <c r="I861" t="s">
+        <v>3970</v>
+      </c>
+      <c r="J861" t="s">
+        <v>356</v>
+      </c>
+      <c r="K861" t="s">
+        <v>4198</v>
+      </c>
+      <c r="L861" t="s">
+        <v>4199</v>
+      </c>
+    </row>
+    <row r="862" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A862">
+        <v>861</v>
+      </c>
+      <c r="B862" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C862" t="s">
+        <v>14</v>
+      </c>
+      <c r="D862" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E862" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F862" t="s">
+        <v>4200</v>
+      </c>
+      <c r="G862" t="s">
+        <v>4201</v>
+      </c>
+      <c r="H862" t="s">
+        <v>390</v>
+      </c>
+      <c r="I862" t="s">
+        <v>3847</v>
+      </c>
+      <c r="J862" t="s">
+        <v>356</v>
+      </c>
+      <c r="K862" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L862" t="s">
+        <v>4202</v>
+      </c>
+    </row>
+    <row r="863" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A863">
+        <v>862</v>
+      </c>
+      <c r="B863" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C863" t="s">
+        <v>14</v>
+      </c>
+      <c r="D863" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E863" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F863" t="s">
+        <v>4203</v>
+      </c>
+      <c r="G863" t="s">
+        <v>4204</v>
+      </c>
+      <c r="H863" t="s">
+        <v>390</v>
+      </c>
+      <c r="I863" t="s">
+        <v>4205</v>
+      </c>
+      <c r="J863" t="s">
+        <v>356</v>
+      </c>
+      <c r="K863" t="s">
+        <v>4206</v>
+      </c>
+      <c r="L863" t="s">
+        <v>4207</v>
+      </c>
+    </row>
+    <row r="864" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A864">
+        <v>863</v>
+      </c>
+      <c r="B864" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C864" t="s">
+        <v>14</v>
+      </c>
+      <c r="D864" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E864" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F864" t="s">
+        <v>4208</v>
+      </c>
+      <c r="G864" t="s">
+        <v>4209</v>
+      </c>
+      <c r="H864" t="s">
+        <v>390</v>
+      </c>
+      <c r="I864" t="s">
+        <v>2069</v>
+      </c>
+      <c r="J864" t="s">
+        <v>356</v>
+      </c>
+      <c r="K864" t="s">
+        <v>4210</v>
+      </c>
+      <c r="L864" t="s">
+        <v>4211</v>
+      </c>
+    </row>
+    <row r="865" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A865">
+        <v>864</v>
+      </c>
+      <c r="B865" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C865" t="s">
+        <v>14</v>
+      </c>
+      <c r="D865" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E865" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F865" t="s">
+        <v>4212</v>
+      </c>
+      <c r="G865" t="s">
+        <v>4213</v>
+      </c>
+      <c r="H865" t="s">
+        <v>390</v>
+      </c>
+      <c r="I865" t="s">
+        <v>3970</v>
+      </c>
+      <c r="J865" t="s">
+        <v>356</v>
+      </c>
+      <c r="K865" t="s">
+        <v>4214</v>
+      </c>
+      <c r="L865" t="s">
+        <v>4215</v>
+      </c>
+    </row>
+    <row r="866" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A866">
+        <v>865</v>
+      </c>
+      <c r="B866" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C866" t="s">
+        <v>14</v>
+      </c>
+      <c r="D866" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E866" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F866" t="s">
+        <v>4216</v>
+      </c>
+      <c r="G866" t="s">
+        <v>4217</v>
+      </c>
+      <c r="H866" t="s">
+        <v>390</v>
+      </c>
+      <c r="I866" t="s">
+        <v>4130</v>
+      </c>
+      <c r="J866" t="s">
+        <v>356</v>
+      </c>
+      <c r="K866" t="s">
+        <v>4218</v>
+      </c>
+      <c r="L866" t="s">
+        <v>4219</v>
+      </c>
+    </row>
+    <row r="867" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A867">
+        <v>866</v>
+      </c>
+      <c r="B867" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C867" t="s">
+        <v>14</v>
+      </c>
+      <c r="D867" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E867" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F867" t="s">
+        <v>4220</v>
+      </c>
+      <c r="G867" t="s">
+        <v>4221</v>
+      </c>
+      <c r="H867" t="s">
+        <v>300</v>
+      </c>
+      <c r="I867" t="s">
+        <v>4222</v>
+      </c>
+      <c r="J867" t="s">
+        <v>356</v>
+      </c>
+      <c r="K867" t="s">
+        <v>4223</v>
+      </c>
+      <c r="L867" t="s">
+        <v>4224</v>
+      </c>
+    </row>
+    <row r="868" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A868">
+        <v>867</v>
+      </c>
+      <c r="B868" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C868" t="s">
+        <v>14</v>
+      </c>
+      <c r="D868" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E868" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F868" t="s">
+        <v>4225</v>
+      </c>
+      <c r="G868" t="s">
+        <v>4226</v>
+      </c>
+      <c r="H868" t="s">
+        <v>300</v>
+      </c>
+      <c r="I868" t="s">
+        <v>3927</v>
+      </c>
+      <c r="J868" t="s">
+        <v>356</v>
+      </c>
+      <c r="K868" t="s">
+        <v>4227</v>
+      </c>
+      <c r="L868" t="s">
+        <v>4228</v>
+      </c>
+    </row>
+    <row r="869" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A869">
+        <v>868</v>
+      </c>
+      <c r="B869" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C869" t="s">
+        <v>14</v>
+      </c>
+      <c r="D869" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E869" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F869" t="s">
+        <v>4229</v>
+      </c>
+      <c r="G869" t="s">
+        <v>4230</v>
+      </c>
+      <c r="H869" t="s">
+        <v>300</v>
+      </c>
+      <c r="I869" t="s">
+        <v>4231</v>
+      </c>
+      <c r="J869" t="s">
+        <v>4188</v>
+      </c>
+      <c r="K869" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L869" t="s">
+        <v>4232</v>
+      </c>
+    </row>
+    <row r="870" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A870">
+        <v>869</v>
+      </c>
+      <c r="B870" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C870" t="s">
+        <v>14</v>
+      </c>
+      <c r="D870" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E870" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F870" t="s">
+        <v>4233</v>
+      </c>
+      <c r="G870" t="s">
+        <v>4234</v>
+      </c>
+      <c r="H870" t="s">
+        <v>300</v>
+      </c>
+      <c r="I870" t="s">
+        <v>3956</v>
+      </c>
+      <c r="J870" t="s">
+        <v>3951</v>
+      </c>
+      <c r="K870" t="s">
+        <v>4235</v>
+      </c>
+      <c r="L870" t="s">
+        <v>4236</v>
+      </c>
+    </row>
+    <row r="871" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A871">
+        <v>870</v>
+      </c>
+      <c r="B871" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C871" t="s">
+        <v>14</v>
+      </c>
+      <c r="D871" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E871" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F871" t="s">
+        <v>4237</v>
+      </c>
+      <c r="G871" t="s">
+        <v>4238</v>
+      </c>
+      <c r="H871" t="s">
+        <v>300</v>
+      </c>
+      <c r="I871" t="s">
+        <v>4239</v>
+      </c>
+      <c r="J871" t="s">
+        <v>356</v>
+      </c>
+      <c r="K871" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L871" t="s">
+        <v>4240</v>
+      </c>
+    </row>
+    <row r="872" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A872">
+        <v>871</v>
+      </c>
+      <c r="B872" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C872" t="s">
+        <v>14</v>
+      </c>
+      <c r="D872" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E872" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F872" t="s">
+        <v>4241</v>
+      </c>
+      <c r="G872" t="s">
+        <v>4242</v>
+      </c>
+      <c r="H872" t="s">
+        <v>300</v>
+      </c>
+      <c r="I872" t="s">
+        <v>4193</v>
+      </c>
+      <c r="J872" t="s">
+        <v>356</v>
+      </c>
+      <c r="K872" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L872" t="s">
+        <v>4243</v>
+      </c>
+    </row>
+    <row r="873" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A873">
+        <v>872</v>
+      </c>
+      <c r="B873" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C873" t="s">
+        <v>14</v>
+      </c>
+      <c r="D873" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E873" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F873" t="s">
+        <v>4244</v>
+      </c>
+      <c r="G873" t="s">
+        <v>4245</v>
+      </c>
+      <c r="H873" t="s">
+        <v>300</v>
+      </c>
+      <c r="I873" t="s">
+        <v>4246</v>
+      </c>
+      <c r="J873" t="s">
+        <v>356</v>
+      </c>
+      <c r="K873" t="s">
+        <v>4247</v>
+      </c>
+      <c r="L873" t="s">
+        <v>4248</v>
+      </c>
+    </row>
+    <row r="874" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A874">
+        <v>873</v>
+      </c>
+      <c r="B874" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C874" t="s">
+        <v>14</v>
+      </c>
+      <c r="D874" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E874" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F874" t="s">
+        <v>4249</v>
+      </c>
+      <c r="G874" t="s">
+        <v>4250</v>
+      </c>
+      <c r="H874" t="s">
+        <v>2040</v>
+      </c>
+      <c r="I874" t="s">
+        <v>4251</v>
+      </c>
+      <c r="J874" t="s">
+        <v>356</v>
+      </c>
+      <c r="K874" t="s">
+        <v>4252</v>
+      </c>
+      <c r="L874" t="s">
+        <v>4253</v>
+      </c>
+    </row>
+    <row r="875" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A875">
+        <v>874</v>
+      </c>
+      <c r="B875" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C875" t="s">
+        <v>14</v>
+      </c>
+      <c r="D875" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E875" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F875" t="s">
+        <v>4254</v>
+      </c>
+      <c r="G875" t="s">
+        <v>4255</v>
+      </c>
+      <c r="H875" t="s">
+        <v>2040</v>
+      </c>
+      <c r="I875" t="s">
+        <v>2069</v>
+      </c>
+      <c r="J875" t="s">
+        <v>356</v>
+      </c>
+      <c r="K875" t="s">
+        <v>4256</v>
+      </c>
+      <c r="L875" t="s">
+        <v>4257</v>
+      </c>
+    </row>
+    <row r="876" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A876">
+        <v>875</v>
+      </c>
+      <c r="B876" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C876" t="s">
+        <v>14</v>
+      </c>
+      <c r="D876" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E876" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F876" t="s">
+        <v>4258</v>
+      </c>
+      <c r="G876" t="s">
+        <v>4259</v>
+      </c>
+      <c r="H876" t="s">
+        <v>428</v>
+      </c>
+      <c r="I876" t="s">
+        <v>4260</v>
+      </c>
+      <c r="J876" t="s">
+        <v>4261</v>
+      </c>
+      <c r="K876" t="s">
+        <v>4262</v>
+      </c>
+      <c r="L876" t="s">
+        <v>4263</v>
+      </c>
+    </row>
+    <row r="877" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A877">
+        <v>876</v>
+      </c>
+      <c r="B877" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C877" t="s">
+        <v>14</v>
+      </c>
+      <c r="D877" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E877" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F877" t="s">
+        <v>4264</v>
+      </c>
+      <c r="G877" t="s">
+        <v>4265</v>
+      </c>
+      <c r="H877" t="s">
+        <v>428</v>
+      </c>
+      <c r="I877" t="s">
+        <v>4266</v>
+      </c>
+      <c r="J877" t="s">
+        <v>366</v>
+      </c>
+      <c r="K877" t="s">
+        <v>4267</v>
+      </c>
+      <c r="L877" t="s">
+        <v>4268</v>
+      </c>
+    </row>
+    <row r="878" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A878">
+        <v>877</v>
+      </c>
+      <c r="B878" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C878" t="s">
+        <v>14</v>
+      </c>
+      <c r="D878" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E878" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F878" t="s">
+        <v>4269</v>
+      </c>
+      <c r="G878" t="s">
+        <v>4270</v>
+      </c>
+      <c r="H878" t="s">
+        <v>428</v>
+      </c>
+      <c r="I878" t="s">
+        <v>4271</v>
+      </c>
+      <c r="J878" t="s">
+        <v>4261</v>
+      </c>
+      <c r="K878" t="s">
+        <v>4272</v>
+      </c>
+      <c r="L878" t="s">
+        <v>4273</v>
+      </c>
+    </row>
+    <row r="879" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A879">
+        <v>878</v>
+      </c>
+      <c r="B879" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C879" t="s">
+        <v>14</v>
+      </c>
+      <c r="D879" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E879" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F879" t="s">
+        <v>4274</v>
+      </c>
+      <c r="G879" t="s">
+        <v>4275</v>
+      </c>
+      <c r="H879" t="s">
+        <v>428</v>
+      </c>
+      <c r="I879" t="s">
+        <v>4276</v>
+      </c>
+      <c r="J879" t="s">
+        <v>366</v>
+      </c>
+      <c r="K879" t="s">
+        <v>4277</v>
+      </c>
+      <c r="L879" t="s">
+        <v>4278</v>
+      </c>
+    </row>
+    <row r="880" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A880">
+        <v>879</v>
+      </c>
+      <c r="B880" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C880" t="s">
+        <v>14</v>
+      </c>
+      <c r="D880" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E880" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F880" t="s">
+        <v>4279</v>
+      </c>
+      <c r="G880" t="s">
+        <v>4280</v>
+      </c>
+      <c r="H880" t="s">
+        <v>428</v>
+      </c>
+      <c r="I880" t="s">
+        <v>4281</v>
+      </c>
+      <c r="J880" t="s">
+        <v>366</v>
+      </c>
+      <c r="K880" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L880" t="s">
+        <v>4282</v>
+      </c>
+    </row>
+    <row r="881" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A881">
+        <v>880</v>
+      </c>
+      <c r="B881" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C881" t="s">
+        <v>14</v>
+      </c>
+      <c r="D881" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E881" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F881" t="s">
+        <v>4283</v>
+      </c>
+      <c r="G881" t="s">
+        <v>4284</v>
+      </c>
+      <c r="H881" t="s">
+        <v>428</v>
+      </c>
+      <c r="I881" t="s">
+        <v>4285</v>
+      </c>
+      <c r="J881" t="s">
+        <v>366</v>
+      </c>
+      <c r="K881" t="s">
+        <v>4286</v>
+      </c>
+      <c r="L881" t="s">
+        <v>4287</v>
+      </c>
+    </row>
+    <row r="882" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A882">
+        <v>881</v>
+      </c>
+      <c r="B882" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C882" t="s">
+        <v>14</v>
+      </c>
+      <c r="D882" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E882" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F882" t="s">
+        <v>4288</v>
+      </c>
+      <c r="G882" t="s">
+        <v>4289</v>
+      </c>
+      <c r="H882" t="s">
+        <v>428</v>
+      </c>
+      <c r="I882" t="s">
+        <v>4290</v>
+      </c>
+      <c r="J882" t="s">
+        <v>366</v>
+      </c>
+      <c r="K882" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L882" t="s">
+        <v>4291</v>
+      </c>
+    </row>
+    <row r="883" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A883">
+        <v>882</v>
+      </c>
+      <c r="B883" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C883" t="s">
+        <v>14</v>
+      </c>
+      <c r="D883" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E883" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F883" t="s">
+        <v>4292</v>
+      </c>
+      <c r="G883" t="s">
+        <v>4293</v>
+      </c>
+      <c r="H883" t="s">
+        <v>428</v>
+      </c>
+      <c r="I883" t="s">
+        <v>4294</v>
+      </c>
+      <c r="J883" t="s">
+        <v>366</v>
+      </c>
+      <c r="K883" t="s">
+        <v>4295</v>
+      </c>
+      <c r="L883" t="s">
+        <v>4296</v>
+      </c>
+    </row>
+    <row r="884" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A884">
+        <v>883</v>
+      </c>
+      <c r="B884" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C884" t="s">
+        <v>14</v>
+      </c>
+      <c r="D884" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E884" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F884" t="s">
+        <v>4297</v>
+      </c>
+      <c r="G884" t="s">
+        <v>4298</v>
+      </c>
+      <c r="H884" t="s">
+        <v>428</v>
+      </c>
+      <c r="I884" t="s">
+        <v>4299</v>
+      </c>
+      <c r="J884" t="s">
+        <v>366</v>
+      </c>
+      <c r="K884" t="s">
+        <v>4300</v>
+      </c>
+      <c r="L884" t="s">
+        <v>4301</v>
+      </c>
+    </row>
+    <row r="885" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A885">
+        <v>884</v>
+      </c>
+      <c r="B885" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C885" t="s">
+        <v>14</v>
+      </c>
+      <c r="D885" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E885" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F885" t="s">
+        <v>4302</v>
+      </c>
+      <c r="G885" t="s">
+        <v>4303</v>
+      </c>
+      <c r="H885" t="s">
+        <v>428</v>
+      </c>
+      <c r="I885" t="s">
+        <v>4304</v>
+      </c>
+      <c r="J885" t="s">
+        <v>366</v>
+      </c>
+      <c r="K885" t="s">
+        <v>4305</v>
+      </c>
+      <c r="L885" t="s">
+        <v>4306</v>
+      </c>
+    </row>
+    <row r="886" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A886">
+        <v>885</v>
+      </c>
+      <c r="B886" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C886" t="s">
+        <v>14</v>
+      </c>
+      <c r="D886" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E886" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F886" t="s">
+        <v>4307</v>
+      </c>
+      <c r="G886" t="s">
+        <v>4308</v>
+      </c>
+      <c r="H886" t="s">
+        <v>428</v>
+      </c>
+      <c r="I886" t="s">
+        <v>4309</v>
+      </c>
+      <c r="J886" t="s">
+        <v>366</v>
+      </c>
+      <c r="K886" t="s">
+        <v>4310</v>
+      </c>
+      <c r="L886" t="s">
+        <v>4311</v>
+      </c>
+    </row>
+    <row r="887" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A887">
+        <v>886</v>
+      </c>
+      <c r="B887" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C887" t="s">
+        <v>14</v>
+      </c>
+      <c r="D887" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E887" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F887" t="s">
+        <v>4312</v>
+      </c>
+      <c r="G887" t="s">
+        <v>4313</v>
+      </c>
+      <c r="H887" t="s">
+        <v>428</v>
+      </c>
+      <c r="I887" t="s">
+        <v>4314</v>
+      </c>
+      <c r="J887" t="s">
+        <v>366</v>
+      </c>
+      <c r="K887" t="s">
+        <v>4315</v>
+      </c>
+      <c r="L887" t="s">
+        <v>4316</v>
+      </c>
+    </row>
+    <row r="888" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A888">
+        <v>887</v>
+      </c>
+      <c r="B888" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C888" t="s">
+        <v>14</v>
+      </c>
+      <c r="D888" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E888" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F888" t="s">
+        <v>4317</v>
+      </c>
+      <c r="G888" t="s">
+        <v>4318</v>
+      </c>
+      <c r="H888" t="s">
+        <v>428</v>
+      </c>
+      <c r="I888" t="s">
+        <v>4319</v>
+      </c>
+      <c r="J888" t="s">
+        <v>366</v>
+      </c>
+      <c r="K888" t="s">
+        <v>4320</v>
+      </c>
+      <c r="L888" t="s">
+        <v>4321</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 39 WebKreatives OSM leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7794" uniqueCount="4322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8223" uniqueCount="4501">
   <si>
     <t>#</t>
   </si>
@@ -12977,6 +12977,543 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:2851803165 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.koopmankappers.nl</t>
+  </si>
+  <si>
+    <t>inf@kapsalonhairenmore.nl</t>
+  </si>
+  <si>
+    <t>Hair &amp; More</t>
+  </si>
+  <si>
+    <t>van Peltlaan 6533ZK</t>
+  </si>
+  <si>
+    <t>+31 24 355 7181</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2851861037 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: http://www.kapsalonhairenmore.nl</t>
+  </si>
+  <si>
+    <t>mirandavanstaveren@hotmail.com</t>
+  </si>
+  <si>
+    <t>Van Staveren Hairstylisten</t>
+  </si>
+  <si>
+    <t>Einsteinstraat 6533NL</t>
+  </si>
+  <si>
+    <t>+31 24 355 4658</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2851910874 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.hairstyling-vanstaveren.nl</t>
+  </si>
+  <si>
+    <t>info@salonesthernijmegen.nl</t>
+  </si>
+  <si>
+    <t>Salon Esther</t>
+  </si>
+  <si>
+    <t>St. Agnetenweg 6545AT</t>
+  </si>
+  <si>
+    <t>+31 24 378 7425</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2949294657 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://salonesthernijmegen.nl</t>
+  </si>
+  <si>
+    <t>info@anita-hair-beauty-fashion.nl</t>
+  </si>
+  <si>
+    <t>Anita Hair Beauty Fashion</t>
+  </si>
+  <si>
+    <t>St. Agnetenweg 6545AW</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2949344990 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://anita-hair-beauty-fashion.nl</t>
+  </si>
+  <si>
+    <t>salon@kapsalonhaarenzo.nl</t>
+  </si>
+  <si>
+    <t>Kapsalon Haar en Zo</t>
+  </si>
+  <si>
+    <t>Tweede Oude Heselaan 6542VJ</t>
+  </si>
+  <si>
+    <t>+31 24 378 5967</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2953405999 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://kapsalonhaarenzo.nl</t>
+  </si>
+  <si>
+    <t>nijmegen@amikappers.nl</t>
+  </si>
+  <si>
+    <t>AMI Kappers Nijmegen Centrum</t>
+  </si>
+  <si>
+    <t>Bisschop Hamerstraat 6511NB</t>
+  </si>
+  <si>
+    <t>+31 24 322 2284</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:3459867619 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.amikappers.nl/salons/nijmegen</t>
+  </si>
+  <si>
+    <t>info@sedashairdesign.nl</t>
+  </si>
+  <si>
+    <t>Seda's Hair Design</t>
+  </si>
+  <si>
+    <t>Cataloniëstraat 6663NJ</t>
+  </si>
+  <si>
+    <t>+31 6 41729752</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:4552185736 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://www.sedashairdesign.nl</t>
+  </si>
+  <si>
+    <t>info@goodfellas-barbershop.nl</t>
+  </si>
+  <si>
+    <t>Goodfellas</t>
+  </si>
+  <si>
+    <t>+31 24 234 0005</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:11394824776 | Source: OpenStreetMap | kapsalon | Nijmegen | Website: https://goodfellas-barbershop.nl</t>
+  </si>
+  <si>
+    <t>info@maudyvossen.nl</t>
+  </si>
+  <si>
+    <t>Maudy Vossen Huidverjongingsinstituut</t>
+  </si>
+  <si>
+    <t>St. Annastraat 6525GT</t>
+  </si>
+  <si>
+    <t>+31 6 53550803</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2826599046 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://www.maudyvossen.nl</t>
+  </si>
+  <si>
+    <t>info@pureclinics.nl</t>
+  </si>
+  <si>
+    <t>Pure Clinics</t>
+  </si>
+  <si>
+    <t>St. Annastraat 6524EA</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2828263434 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://www.pureclinics.nl</t>
+  </si>
+  <si>
+    <t>info@japandiheadspa.nl</t>
+  </si>
+  <si>
+    <t>Japandi</t>
+  </si>
+  <si>
+    <t>van Peltlaan 6533ZR</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2851755899 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://japandiheadspa.nl</t>
+  </si>
+  <si>
+    <t>info@sanjasteenhuidzorg.nl</t>
+  </si>
+  <si>
+    <t>Sanja Steen Huidzorg</t>
+  </si>
+  <si>
+    <t>Sint Jacobslaan 6533VP</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2851804217 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://www.sanjasteenhuidzorg.nl</t>
+  </si>
+  <si>
+    <t>win.nails@yahoo.com</t>
+  </si>
+  <si>
+    <t>Win Nails Spa</t>
+  </si>
+  <si>
+    <t>Zwanenveld 6538TC</t>
+  </si>
+  <si>
+    <t>+31 24 785 0232</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2890149636 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://www.winnails.nl</t>
+  </si>
+  <si>
+    <t>sunspecialdukenburg@hotmail.com</t>
+  </si>
+  <si>
+    <t>SunSpecial</t>
+  </si>
+  <si>
+    <t>Zwanenveld 6538SE</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2890186021 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://zonnestudiosunspecial.nl/vestiging/nijmegen-dukenburg</t>
+  </si>
+  <si>
+    <t>contact@petersbeauty.nl</t>
+  </si>
+  <si>
+    <t>Peters</t>
+  </si>
+  <si>
+    <t>Pastoor van Laakstraat 6663CC</t>
+  </si>
+  <si>
+    <t>+31 6 23672282</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2960034039 | Source: OpenStreetMap | schoonheidssalon | Nijmegen | Website: https://petersbeauty.nl</t>
+  </si>
+  <si>
+    <t>info@zoevers.nl</t>
+  </si>
+  <si>
+    <t>Zoevers</t>
+  </si>
+  <si>
+    <t>Griftdijk Zuid 6663BE</t>
+  </si>
+  <si>
+    <t>+31 24 820 0201</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:940714663 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://www.zoevers.nl</t>
+  </si>
+  <si>
+    <t>info@brouwerbikestore.nl</t>
+  </si>
+  <si>
+    <t>Brouwer Bike Store</t>
+  </si>
+  <si>
+    <t>Lentse Tuinstraat 6663BG</t>
+  </si>
+  <si>
+    <t>+31 24 324 3988</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:940714671 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://brouwerbikestore.nl</t>
+  </si>
+  <si>
+    <t>rijwielhandeldeconcurrent@hetnet.nl</t>
+  </si>
+  <si>
+    <t>Rijwielhandel de Concurrent</t>
+  </si>
+  <si>
+    <t>van Trieststraat 6512CW</t>
+  </si>
+  <si>
+    <t>+31 24 323 1819</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2847324648 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://www.rijwielhandeldeconcurrent.nl</t>
+  </si>
+  <si>
+    <t>trekstorenijmegen@trekbikes.com</t>
+  </si>
+  <si>
+    <t>Trek</t>
+  </si>
+  <si>
+    <t>Hatertseweg 6533GV</t>
+  </si>
+  <si>
+    <t>+31 24 355 3906</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2852063801 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://www.trekbikes.com/nl/nl_NL/retail/nijmegen</t>
+  </si>
+  <si>
+    <t>info@scheepersbiketotaal.nl</t>
+  </si>
+  <si>
+    <t>Rijwielhuis Janssen</t>
+  </si>
+  <si>
+    <t>Malvert 6538DP</t>
+  </si>
+  <si>
+    <t>+31 24 785 5951</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2853038850 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: http://www.scheepersbiketotaal.nl</t>
+  </si>
+  <si>
+    <t>info@fietsreparatiedukenburg.nl</t>
+  </si>
+  <si>
+    <t>Fietsreparatie Dukenburg</t>
+  </si>
+  <si>
+    <t>Zwanenveld 6538TA</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2890149630 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://fietsreparatiedukenburg.nl</t>
+  </si>
+  <si>
+    <t>info@re-cycled.nl</t>
+  </si>
+  <si>
+    <t>Re-Cycled</t>
+  </si>
+  <si>
+    <t>Zwanenveld 6538SB</t>
+  </si>
+  <si>
+    <t>+31 6 87990893</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2890186053 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://www.re-cycled.nl</t>
+  </si>
+  <si>
+    <t>info@wfsnijmegen.nl</t>
+  </si>
+  <si>
+    <t>Wouter Fiets Service Nijmegen</t>
+  </si>
+  <si>
+    <t>+31 6 24605897</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2949294659 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://wfsnijmegen.nl</t>
+  </si>
+  <si>
+    <t>info@jankooij.nl</t>
+  </si>
+  <si>
+    <t>Jan Kooij 2 Wielers</t>
+  </si>
+  <si>
+    <t>Nieuwe Dukenburgseweg 6534AD</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:11968405582 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://jankooij.nl</t>
+  </si>
+  <si>
+    <t>lschouten@cubestores.nl</t>
+  </si>
+  <si>
+    <t>CUBE store Nijmegen</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:11968405585 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://www.cubestores.nl/pages/cube-store-nijmegen</t>
+  </si>
+  <si>
+    <t>info@stip-kinderfietsen.nl</t>
+  </si>
+  <si>
+    <t>Stip kinderfietsen</t>
+  </si>
+  <si>
+    <t>+31 24 2340530</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:12265612813 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://stip-kinderfietsen.nl</t>
+  </si>
+  <si>
+    <t>info@fietshuis-nijmegen.nl</t>
+  </si>
+  <si>
+    <t>Fietshuis Nijmegen</t>
+  </si>
+  <si>
+    <t>Postweg 6523LD</t>
+  </si>
+  <si>
+    <t>+31 6 381 387 45</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:13039651862 | Source: OpenStreetMap | fietsenwinkel | Nijmegen | Website: https://www.fietshuis-nijmegen.nl</t>
+  </si>
+  <si>
+    <t>nijmegen@degroeneweg.nl</t>
+  </si>
+  <si>
+    <t>De Groene Weg</t>
+  </si>
+  <si>
+    <t>Groenestraat 6531HE</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2087601804 | Source: OpenStreetMap | slager | Nijmegen | Website: https://nijmegen.degroeneweg.nl</t>
+  </si>
+  <si>
+    <t>slagerijcorvandijk@planet.nl</t>
+  </si>
+  <si>
+    <t>Slagerij Van Dijk</t>
+  </si>
+  <si>
+    <t>Heidevenstraat 6533TP</t>
+  </si>
+  <si>
+    <t>+31 24 355 3755</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2851801485 | Source: OpenStreetMap | slager | Nijmegen | Website: https://www.slagerijcorvandijk.nl</t>
+  </si>
+  <si>
+    <t>info@stadsbakkerijdebie.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij De Bie</t>
+  </si>
+  <si>
+    <t>Krayenhofflaan 6541PZ</t>
+  </si>
+  <si>
+    <t>+31 24 377 5325</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:986657188 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://bakkerijdebie.nl</t>
+  </si>
+  <si>
+    <t>info@deknollentuin.nl</t>
+  </si>
+  <si>
+    <t>De Knollentuin</t>
+  </si>
+  <si>
+    <t>Fransestraat 6524HR</t>
+  </si>
+  <si>
+    <t>+31 24 322 5977</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2828266713 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.deknollentuin.nl</t>
+  </si>
+  <si>
+    <t>post@streekbakkerjorrit.nl</t>
+  </si>
+  <si>
+    <t>Streekbakker Jorrit</t>
+  </si>
+  <si>
+    <t>Thijmstraat 6531CP</t>
+  </si>
+  <si>
+    <t>+31 24 737 0483</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2848101682 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.streekbakkerjorrit.nl</t>
+  </si>
+  <si>
+    <t>info@artsbakkers.nl</t>
+  </si>
+  <si>
+    <t>Brood- en Banketbakkerij De Korenschoof</t>
+  </si>
+  <si>
+    <t>Steenbokstraat 6531TH</t>
+  </si>
+  <si>
+    <t>+31 24 350 3440</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2848317575 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.artsbakkers.nl</t>
+  </si>
+  <si>
+    <t>bakkerijholland@upcmail.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij Holland</t>
+  </si>
+  <si>
+    <t>Sint Jacobslaan 6533VC</t>
+  </si>
+  <si>
+    <t>+31 24 355 0708</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2851756482 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.bakkerij-holland.nl</t>
+  </si>
+  <si>
+    <t>info@vaneigendeeg.nl</t>
+  </si>
+  <si>
+    <t>Van Eigen Deeg</t>
+  </si>
+  <si>
+    <t>Roggeweg 6534AJ</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2852084572 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.vaneigendeeg.nl</t>
+  </si>
+  <si>
+    <t>info@kraayennest.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij 't Kraayennest</t>
+  </si>
+  <si>
+    <t>Fuchsiastraat 6542NX</t>
+  </si>
+  <si>
+    <t>+31 24 204 9625</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2953227594 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.kraayennest.nl/winkels</t>
+  </si>
+  <si>
+    <t>info@bakkerijkoekkoek.nl</t>
+  </si>
+  <si>
+    <t>Bakkerij KoekKoek</t>
+  </si>
+  <si>
+    <t>Passage Molenpoort 6511HS</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:3673024291 | Source: OpenStreetMap | bakkerij | Nijmegen | Website: https://www.bakkerijkoekkoek.nl</t>
+  </si>
+  <si>
+    <t>contact@bloemwerknijmegen.nl</t>
+  </si>
+  <si>
+    <t>Bellis Bloemwerk Nijmegen</t>
+  </si>
+  <si>
+    <t>+31 6 83 27 12 80</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2087626943 | Source: OpenStreetMap | bloemist | Nijmegen | Website: https://bloemwerknijmegen.nl</t>
+  </si>
+  <si>
+    <t>order@flowersinsight.nl</t>
+  </si>
+  <si>
+    <t>Flowers Insight</t>
+  </si>
+  <si>
+    <t>Stationsplein 6512AB</t>
+  </si>
+  <si>
+    <t>+31 24 322 5197</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:3530962649 | Source: OpenStreetMap | bloemist | Nijmegen | Website: https://flowersinsight.nl</t>
   </si>
 </sst>
 </file>
@@ -13353,7 +13890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L888"/>
+  <dimension ref="A1:L927"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -41178,6 +41715,1488 @@
         <v>4321</v>
       </c>
     </row>
+    <row r="889" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A889">
+        <v>888</v>
+      </c>
+      <c r="B889" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C889" t="s">
+        <v>14</v>
+      </c>
+      <c r="D889" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E889" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F889" t="s">
+        <v>4322</v>
+      </c>
+      <c r="G889" t="s">
+        <v>4323</v>
+      </c>
+      <c r="H889" t="s">
+        <v>428</v>
+      </c>
+      <c r="I889" t="s">
+        <v>4324</v>
+      </c>
+      <c r="J889" t="s">
+        <v>366</v>
+      </c>
+      <c r="K889" t="s">
+        <v>4325</v>
+      </c>
+      <c r="L889" t="s">
+        <v>4326</v>
+      </c>
+    </row>
+    <row r="890" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A890">
+        <v>889</v>
+      </c>
+      <c r="B890" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C890" t="s">
+        <v>14</v>
+      </c>
+      <c r="D890" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E890" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F890" t="s">
+        <v>4327</v>
+      </c>
+      <c r="G890" t="s">
+        <v>4328</v>
+      </c>
+      <c r="H890" t="s">
+        <v>428</v>
+      </c>
+      <c r="I890" t="s">
+        <v>4329</v>
+      </c>
+      <c r="J890" t="s">
+        <v>366</v>
+      </c>
+      <c r="K890" t="s">
+        <v>4330</v>
+      </c>
+      <c r="L890" t="s">
+        <v>4331</v>
+      </c>
+    </row>
+    <row r="891" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A891">
+        <v>890</v>
+      </c>
+      <c r="B891" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C891" t="s">
+        <v>14</v>
+      </c>
+      <c r="D891" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E891" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F891" t="s">
+        <v>4332</v>
+      </c>
+      <c r="G891" t="s">
+        <v>4333</v>
+      </c>
+      <c r="H891" t="s">
+        <v>428</v>
+      </c>
+      <c r="I891" t="s">
+        <v>4334</v>
+      </c>
+      <c r="J891" t="s">
+        <v>366</v>
+      </c>
+      <c r="K891" t="s">
+        <v>4335</v>
+      </c>
+      <c r="L891" t="s">
+        <v>4336</v>
+      </c>
+    </row>
+    <row r="892" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A892">
+        <v>891</v>
+      </c>
+      <c r="B892" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C892" t="s">
+        <v>14</v>
+      </c>
+      <c r="D892" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E892" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F892" t="s">
+        <v>4337</v>
+      </c>
+      <c r="G892" t="s">
+        <v>4338</v>
+      </c>
+      <c r="H892" t="s">
+        <v>428</v>
+      </c>
+      <c r="I892" t="s">
+        <v>4339</v>
+      </c>
+      <c r="J892" t="s">
+        <v>366</v>
+      </c>
+      <c r="K892" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L892" t="s">
+        <v>4340</v>
+      </c>
+    </row>
+    <row r="893" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A893">
+        <v>892</v>
+      </c>
+      <c r="B893" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C893" t="s">
+        <v>14</v>
+      </c>
+      <c r="D893" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E893" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F893" t="s">
+        <v>4341</v>
+      </c>
+      <c r="G893" t="s">
+        <v>4342</v>
+      </c>
+      <c r="H893" t="s">
+        <v>428</v>
+      </c>
+      <c r="I893" t="s">
+        <v>4343</v>
+      </c>
+      <c r="J893" t="s">
+        <v>366</v>
+      </c>
+      <c r="K893" t="s">
+        <v>4344</v>
+      </c>
+      <c r="L893" t="s">
+        <v>4345</v>
+      </c>
+    </row>
+    <row r="894" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A894">
+        <v>893</v>
+      </c>
+      <c r="B894" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C894" t="s">
+        <v>14</v>
+      </c>
+      <c r="D894" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E894" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F894" t="s">
+        <v>4346</v>
+      </c>
+      <c r="G894" t="s">
+        <v>4347</v>
+      </c>
+      <c r="H894" t="s">
+        <v>428</v>
+      </c>
+      <c r="I894" t="s">
+        <v>4348</v>
+      </c>
+      <c r="J894" t="s">
+        <v>366</v>
+      </c>
+      <c r="K894" t="s">
+        <v>4349</v>
+      </c>
+      <c r="L894" t="s">
+        <v>4350</v>
+      </c>
+    </row>
+    <row r="895" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A895">
+        <v>894</v>
+      </c>
+      <c r="B895" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C895" t="s">
+        <v>14</v>
+      </c>
+      <c r="D895" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E895" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F895" t="s">
+        <v>4351</v>
+      </c>
+      <c r="G895" t="s">
+        <v>4352</v>
+      </c>
+      <c r="H895" t="s">
+        <v>428</v>
+      </c>
+      <c r="I895" t="s">
+        <v>4353</v>
+      </c>
+      <c r="J895" t="s">
+        <v>4261</v>
+      </c>
+      <c r="K895" t="s">
+        <v>4354</v>
+      </c>
+      <c r="L895" t="s">
+        <v>4355</v>
+      </c>
+    </row>
+    <row r="896" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A896">
+        <v>895</v>
+      </c>
+      <c r="B896" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C896" t="s">
+        <v>14</v>
+      </c>
+      <c r="D896" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E896" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F896" t="s">
+        <v>4356</v>
+      </c>
+      <c r="G896" t="s">
+        <v>4357</v>
+      </c>
+      <c r="H896" t="s">
+        <v>428</v>
+      </c>
+      <c r="I896" t="s">
+        <v>3962</v>
+      </c>
+      <c r="J896" t="s">
+        <v>366</v>
+      </c>
+      <c r="K896" t="s">
+        <v>4358</v>
+      </c>
+      <c r="L896" t="s">
+        <v>4359</v>
+      </c>
+    </row>
+    <row r="897" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A897">
+        <v>896</v>
+      </c>
+      <c r="B897" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C897" t="s">
+        <v>14</v>
+      </c>
+      <c r="D897" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E897" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F897" t="s">
+        <v>4360</v>
+      </c>
+      <c r="G897" t="s">
+        <v>4361</v>
+      </c>
+      <c r="H897" t="s">
+        <v>343</v>
+      </c>
+      <c r="I897" t="s">
+        <v>4362</v>
+      </c>
+      <c r="J897" t="s">
+        <v>366</v>
+      </c>
+      <c r="K897" t="s">
+        <v>4363</v>
+      </c>
+      <c r="L897" t="s">
+        <v>4364</v>
+      </c>
+    </row>
+    <row r="898" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A898">
+        <v>897</v>
+      </c>
+      <c r="B898" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C898" t="s">
+        <v>14</v>
+      </c>
+      <c r="D898" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E898" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F898" t="s">
+        <v>4365</v>
+      </c>
+      <c r="G898" t="s">
+        <v>4366</v>
+      </c>
+      <c r="H898" t="s">
+        <v>343</v>
+      </c>
+      <c r="I898" t="s">
+        <v>4367</v>
+      </c>
+      <c r="J898" t="s">
+        <v>366</v>
+      </c>
+      <c r="K898" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L898" t="s">
+        <v>4368</v>
+      </c>
+    </row>
+    <row r="899" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A899">
+        <v>898</v>
+      </c>
+      <c r="B899" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C899" t="s">
+        <v>14</v>
+      </c>
+      <c r="D899" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E899" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F899" t="s">
+        <v>4369</v>
+      </c>
+      <c r="G899" t="s">
+        <v>4370</v>
+      </c>
+      <c r="H899" t="s">
+        <v>343</v>
+      </c>
+      <c r="I899" t="s">
+        <v>4371</v>
+      </c>
+      <c r="J899" t="s">
+        <v>366</v>
+      </c>
+      <c r="K899" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L899" t="s">
+        <v>4372</v>
+      </c>
+    </row>
+    <row r="900" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A900">
+        <v>899</v>
+      </c>
+      <c r="B900" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C900" t="s">
+        <v>14</v>
+      </c>
+      <c r="D900" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E900" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F900" t="s">
+        <v>4373</v>
+      </c>
+      <c r="G900" t="s">
+        <v>4374</v>
+      </c>
+      <c r="H900" t="s">
+        <v>343</v>
+      </c>
+      <c r="I900" t="s">
+        <v>4375</v>
+      </c>
+      <c r="J900" t="s">
+        <v>366</v>
+      </c>
+      <c r="K900" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L900" t="s">
+        <v>4376</v>
+      </c>
+    </row>
+    <row r="901" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A901">
+        <v>900</v>
+      </c>
+      <c r="B901" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C901" t="s">
+        <v>14</v>
+      </c>
+      <c r="D901" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E901" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F901" t="s">
+        <v>4377</v>
+      </c>
+      <c r="G901" t="s">
+        <v>4378</v>
+      </c>
+      <c r="H901" t="s">
+        <v>343</v>
+      </c>
+      <c r="I901" t="s">
+        <v>4379</v>
+      </c>
+      <c r="J901" t="s">
+        <v>366</v>
+      </c>
+      <c r="K901" t="s">
+        <v>4380</v>
+      </c>
+      <c r="L901" t="s">
+        <v>4381</v>
+      </c>
+    </row>
+    <row r="902" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A902">
+        <v>901</v>
+      </c>
+      <c r="B902" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C902" t="s">
+        <v>14</v>
+      </c>
+      <c r="D902" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E902" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F902" t="s">
+        <v>4382</v>
+      </c>
+      <c r="G902" t="s">
+        <v>4383</v>
+      </c>
+      <c r="H902" t="s">
+        <v>343</v>
+      </c>
+      <c r="I902" t="s">
+        <v>4384</v>
+      </c>
+      <c r="J902" t="s">
+        <v>366</v>
+      </c>
+      <c r="K902" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L902" t="s">
+        <v>4385</v>
+      </c>
+    </row>
+    <row r="903" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A903">
+        <v>902</v>
+      </c>
+      <c r="B903" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C903" t="s">
+        <v>14</v>
+      </c>
+      <c r="D903" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E903" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F903" t="s">
+        <v>4386</v>
+      </c>
+      <c r="G903" t="s">
+        <v>4387</v>
+      </c>
+      <c r="H903" t="s">
+        <v>343</v>
+      </c>
+      <c r="I903" t="s">
+        <v>4388</v>
+      </c>
+      <c r="J903" t="s">
+        <v>4261</v>
+      </c>
+      <c r="K903" t="s">
+        <v>4389</v>
+      </c>
+      <c r="L903" t="s">
+        <v>4390</v>
+      </c>
+    </row>
+    <row r="904" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A904">
+        <v>903</v>
+      </c>
+      <c r="B904" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C904" t="s">
+        <v>14</v>
+      </c>
+      <c r="D904" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E904" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F904" t="s">
+        <v>4391</v>
+      </c>
+      <c r="G904" t="s">
+        <v>4392</v>
+      </c>
+      <c r="H904" t="s">
+        <v>522</v>
+      </c>
+      <c r="I904" t="s">
+        <v>4393</v>
+      </c>
+      <c r="J904" t="s">
+        <v>4261</v>
+      </c>
+      <c r="K904" t="s">
+        <v>4394</v>
+      </c>
+      <c r="L904" t="s">
+        <v>4395</v>
+      </c>
+    </row>
+    <row r="905" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A905">
+        <v>904</v>
+      </c>
+      <c r="B905" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C905" t="s">
+        <v>14</v>
+      </c>
+      <c r="D905" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E905" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F905" t="s">
+        <v>4396</v>
+      </c>
+      <c r="G905" t="s">
+        <v>4397</v>
+      </c>
+      <c r="H905" t="s">
+        <v>522</v>
+      </c>
+      <c r="I905" t="s">
+        <v>4398</v>
+      </c>
+      <c r="J905" t="s">
+        <v>4261</v>
+      </c>
+      <c r="K905" t="s">
+        <v>4399</v>
+      </c>
+      <c r="L905" t="s">
+        <v>4400</v>
+      </c>
+    </row>
+    <row r="906" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A906">
+        <v>905</v>
+      </c>
+      <c r="B906" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C906" t="s">
+        <v>14</v>
+      </c>
+      <c r="D906" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E906" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F906" t="s">
+        <v>4401</v>
+      </c>
+      <c r="G906" t="s">
+        <v>4402</v>
+      </c>
+      <c r="H906" t="s">
+        <v>522</v>
+      </c>
+      <c r="I906" t="s">
+        <v>4403</v>
+      </c>
+      <c r="J906" t="s">
+        <v>366</v>
+      </c>
+      <c r="K906" t="s">
+        <v>4404</v>
+      </c>
+      <c r="L906" t="s">
+        <v>4405</v>
+      </c>
+    </row>
+    <row r="907" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A907">
+        <v>906</v>
+      </c>
+      <c r="B907" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C907" t="s">
+        <v>14</v>
+      </c>
+      <c r="D907" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E907" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F907" t="s">
+        <v>4406</v>
+      </c>
+      <c r="G907" t="s">
+        <v>4407</v>
+      </c>
+      <c r="H907" t="s">
+        <v>522</v>
+      </c>
+      <c r="I907" t="s">
+        <v>4408</v>
+      </c>
+      <c r="J907" t="s">
+        <v>366</v>
+      </c>
+      <c r="K907" t="s">
+        <v>4409</v>
+      </c>
+      <c r="L907" t="s">
+        <v>4410</v>
+      </c>
+    </row>
+    <row r="908" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A908">
+        <v>907</v>
+      </c>
+      <c r="B908" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C908" t="s">
+        <v>14</v>
+      </c>
+      <c r="D908" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E908" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F908" t="s">
+        <v>4411</v>
+      </c>
+      <c r="G908" t="s">
+        <v>4412</v>
+      </c>
+      <c r="H908" t="s">
+        <v>522</v>
+      </c>
+      <c r="I908" t="s">
+        <v>4413</v>
+      </c>
+      <c r="J908" t="s">
+        <v>366</v>
+      </c>
+      <c r="K908" t="s">
+        <v>4414</v>
+      </c>
+      <c r="L908" t="s">
+        <v>4415</v>
+      </c>
+    </row>
+    <row r="909" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A909">
+        <v>908</v>
+      </c>
+      <c r="B909" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C909" t="s">
+        <v>14</v>
+      </c>
+      <c r="D909" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E909" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F909" t="s">
+        <v>4416</v>
+      </c>
+      <c r="G909" t="s">
+        <v>4417</v>
+      </c>
+      <c r="H909" t="s">
+        <v>522</v>
+      </c>
+      <c r="I909" t="s">
+        <v>4418</v>
+      </c>
+      <c r="J909" t="s">
+        <v>366</v>
+      </c>
+      <c r="K909" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L909" t="s">
+        <v>4419</v>
+      </c>
+    </row>
+    <row r="910" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A910">
+        <v>909</v>
+      </c>
+      <c r="B910" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C910" t="s">
+        <v>14</v>
+      </c>
+      <c r="D910" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E910" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F910" t="s">
+        <v>4420</v>
+      </c>
+      <c r="G910" t="s">
+        <v>4421</v>
+      </c>
+      <c r="H910" t="s">
+        <v>522</v>
+      </c>
+      <c r="I910" t="s">
+        <v>4422</v>
+      </c>
+      <c r="J910" t="s">
+        <v>366</v>
+      </c>
+      <c r="K910" t="s">
+        <v>4423</v>
+      </c>
+      <c r="L910" t="s">
+        <v>4424</v>
+      </c>
+    </row>
+    <row r="911" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A911">
+        <v>910</v>
+      </c>
+      <c r="B911" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C911" t="s">
+        <v>14</v>
+      </c>
+      <c r="D911" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E911" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F911" t="s">
+        <v>4425</v>
+      </c>
+      <c r="G911" t="s">
+        <v>4426</v>
+      </c>
+      <c r="H911" t="s">
+        <v>522</v>
+      </c>
+      <c r="I911" t="s">
+        <v>4334</v>
+      </c>
+      <c r="J911" t="s">
+        <v>366</v>
+      </c>
+      <c r="K911" t="s">
+        <v>4427</v>
+      </c>
+      <c r="L911" t="s">
+        <v>4428</v>
+      </c>
+    </row>
+    <row r="912" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A912">
+        <v>911</v>
+      </c>
+      <c r="B912" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C912" t="s">
+        <v>14</v>
+      </c>
+      <c r="D912" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E912" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F912" t="s">
+        <v>4429</v>
+      </c>
+      <c r="G912" t="s">
+        <v>4430</v>
+      </c>
+      <c r="H912" t="s">
+        <v>522</v>
+      </c>
+      <c r="I912" t="s">
+        <v>4431</v>
+      </c>
+      <c r="J912" t="s">
+        <v>366</v>
+      </c>
+      <c r="K912" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L912" t="s">
+        <v>4432</v>
+      </c>
+    </row>
+    <row r="913" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A913">
+        <v>912</v>
+      </c>
+      <c r="B913" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C913" t="s">
+        <v>14</v>
+      </c>
+      <c r="D913" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E913" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F913" t="s">
+        <v>4433</v>
+      </c>
+      <c r="G913" t="s">
+        <v>4434</v>
+      </c>
+      <c r="H913" t="s">
+        <v>522</v>
+      </c>
+      <c r="I913" t="s">
+        <v>4431</v>
+      </c>
+      <c r="J913" t="s">
+        <v>366</v>
+      </c>
+      <c r="K913" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L913" t="s">
+        <v>4435</v>
+      </c>
+    </row>
+    <row r="914" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A914">
+        <v>913</v>
+      </c>
+      <c r="B914" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C914" t="s">
+        <v>14</v>
+      </c>
+      <c r="D914" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E914" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F914" t="s">
+        <v>4436</v>
+      </c>
+      <c r="G914" t="s">
+        <v>4437</v>
+      </c>
+      <c r="H914" t="s">
+        <v>522</v>
+      </c>
+      <c r="I914" t="s">
+        <v>3962</v>
+      </c>
+      <c r="J914" t="s">
+        <v>366</v>
+      </c>
+      <c r="K914" t="s">
+        <v>4438</v>
+      </c>
+      <c r="L914" t="s">
+        <v>4439</v>
+      </c>
+    </row>
+    <row r="915" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A915">
+        <v>914</v>
+      </c>
+      <c r="B915" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C915" t="s">
+        <v>14</v>
+      </c>
+      <c r="D915" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E915" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F915" t="s">
+        <v>4440</v>
+      </c>
+      <c r="G915" t="s">
+        <v>4441</v>
+      </c>
+      <c r="H915" t="s">
+        <v>522</v>
+      </c>
+      <c r="I915" t="s">
+        <v>4442</v>
+      </c>
+      <c r="J915" t="s">
+        <v>366</v>
+      </c>
+      <c r="K915" t="s">
+        <v>4443</v>
+      </c>
+      <c r="L915" t="s">
+        <v>4444</v>
+      </c>
+    </row>
+    <row r="916" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A916">
+        <v>915</v>
+      </c>
+      <c r="B916" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C916" t="s">
+        <v>14</v>
+      </c>
+      <c r="D916" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E916" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F916" t="s">
+        <v>4445</v>
+      </c>
+      <c r="G916" t="s">
+        <v>4446</v>
+      </c>
+      <c r="H916" t="s">
+        <v>1765</v>
+      </c>
+      <c r="I916" t="s">
+        <v>4447</v>
+      </c>
+      <c r="J916" t="s">
+        <v>366</v>
+      </c>
+      <c r="K916" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L916" t="s">
+        <v>4448</v>
+      </c>
+    </row>
+    <row r="917" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A917">
+        <v>916</v>
+      </c>
+      <c r="B917" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C917" t="s">
+        <v>14</v>
+      </c>
+      <c r="D917" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E917" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F917" t="s">
+        <v>4449</v>
+      </c>
+      <c r="G917" t="s">
+        <v>4450</v>
+      </c>
+      <c r="H917" t="s">
+        <v>1765</v>
+      </c>
+      <c r="I917" t="s">
+        <v>4451</v>
+      </c>
+      <c r="J917" t="s">
+        <v>366</v>
+      </c>
+      <c r="K917" t="s">
+        <v>4452</v>
+      </c>
+      <c r="L917" t="s">
+        <v>4453</v>
+      </c>
+    </row>
+    <row r="918" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A918">
+        <v>917</v>
+      </c>
+      <c r="B918" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C918" t="s">
+        <v>14</v>
+      </c>
+      <c r="D918" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E918" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F918" t="s">
+        <v>4454</v>
+      </c>
+      <c r="G918" t="s">
+        <v>4455</v>
+      </c>
+      <c r="H918" t="s">
+        <v>390</v>
+      </c>
+      <c r="I918" t="s">
+        <v>4456</v>
+      </c>
+      <c r="J918" t="s">
+        <v>366</v>
+      </c>
+      <c r="K918" t="s">
+        <v>4457</v>
+      </c>
+      <c r="L918" t="s">
+        <v>4458</v>
+      </c>
+    </row>
+    <row r="919" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A919">
+        <v>918</v>
+      </c>
+      <c r="B919" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C919" t="s">
+        <v>14</v>
+      </c>
+      <c r="D919" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E919" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F919" t="s">
+        <v>4459</v>
+      </c>
+      <c r="G919" t="s">
+        <v>4460</v>
+      </c>
+      <c r="H919" t="s">
+        <v>390</v>
+      </c>
+      <c r="I919" t="s">
+        <v>4461</v>
+      </c>
+      <c r="J919" t="s">
+        <v>366</v>
+      </c>
+      <c r="K919" t="s">
+        <v>4462</v>
+      </c>
+      <c r="L919" t="s">
+        <v>4463</v>
+      </c>
+    </row>
+    <row r="920" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A920">
+        <v>919</v>
+      </c>
+      <c r="B920" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C920" t="s">
+        <v>14</v>
+      </c>
+      <c r="D920" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E920" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F920" t="s">
+        <v>4464</v>
+      </c>
+      <c r="G920" t="s">
+        <v>4465</v>
+      </c>
+      <c r="H920" t="s">
+        <v>390</v>
+      </c>
+      <c r="I920" t="s">
+        <v>4466</v>
+      </c>
+      <c r="J920" t="s">
+        <v>366</v>
+      </c>
+      <c r="K920" t="s">
+        <v>4467</v>
+      </c>
+      <c r="L920" t="s">
+        <v>4468</v>
+      </c>
+    </row>
+    <row r="921" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A921">
+        <v>920</v>
+      </c>
+      <c r="B921" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C921" t="s">
+        <v>14</v>
+      </c>
+      <c r="D921" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E921" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F921" t="s">
+        <v>4469</v>
+      </c>
+      <c r="G921" t="s">
+        <v>4470</v>
+      </c>
+      <c r="H921" t="s">
+        <v>390</v>
+      </c>
+      <c r="I921" t="s">
+        <v>4471</v>
+      </c>
+      <c r="J921" t="s">
+        <v>366</v>
+      </c>
+      <c r="K921" t="s">
+        <v>4472</v>
+      </c>
+      <c r="L921" t="s">
+        <v>4473</v>
+      </c>
+    </row>
+    <row r="922" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A922">
+        <v>921</v>
+      </c>
+      <c r="B922" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C922" t="s">
+        <v>14</v>
+      </c>
+      <c r="D922" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E922" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F922" t="s">
+        <v>4474</v>
+      </c>
+      <c r="G922" t="s">
+        <v>4475</v>
+      </c>
+      <c r="H922" t="s">
+        <v>390</v>
+      </c>
+      <c r="I922" t="s">
+        <v>4476</v>
+      </c>
+      <c r="J922" t="s">
+        <v>366</v>
+      </c>
+      <c r="K922" t="s">
+        <v>4477</v>
+      </c>
+      <c r="L922" t="s">
+        <v>4478</v>
+      </c>
+    </row>
+    <row r="923" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A923">
+        <v>922</v>
+      </c>
+      <c r="B923" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C923" t="s">
+        <v>14</v>
+      </c>
+      <c r="D923" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E923" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F923" t="s">
+        <v>4479</v>
+      </c>
+      <c r="G923" t="s">
+        <v>4480</v>
+      </c>
+      <c r="H923" t="s">
+        <v>390</v>
+      </c>
+      <c r="I923" t="s">
+        <v>4481</v>
+      </c>
+      <c r="J923" t="s">
+        <v>366</v>
+      </c>
+      <c r="K923" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L923" t="s">
+        <v>4482</v>
+      </c>
+    </row>
+    <row r="924" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A924">
+        <v>923</v>
+      </c>
+      <c r="B924" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C924" t="s">
+        <v>14</v>
+      </c>
+      <c r="D924" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E924" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F924" t="s">
+        <v>4483</v>
+      </c>
+      <c r="G924" t="s">
+        <v>4484</v>
+      </c>
+      <c r="H924" t="s">
+        <v>390</v>
+      </c>
+      <c r="I924" t="s">
+        <v>4485</v>
+      </c>
+      <c r="J924" t="s">
+        <v>366</v>
+      </c>
+      <c r="K924" t="s">
+        <v>4486</v>
+      </c>
+      <c r="L924" t="s">
+        <v>4487</v>
+      </c>
+    </row>
+    <row r="925" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A925">
+        <v>924</v>
+      </c>
+      <c r="B925" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C925" t="s">
+        <v>14</v>
+      </c>
+      <c r="D925" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E925" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F925" t="s">
+        <v>4488</v>
+      </c>
+      <c r="G925" t="s">
+        <v>4489</v>
+      </c>
+      <c r="H925" t="s">
+        <v>390</v>
+      </c>
+      <c r="I925" t="s">
+        <v>4490</v>
+      </c>
+      <c r="J925" t="s">
+        <v>366</v>
+      </c>
+      <c r="K925" t="s">
+        <v>3962</v>
+      </c>
+      <c r="L925" t="s">
+        <v>4491</v>
+      </c>
+    </row>
+    <row r="926" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A926">
+        <v>925</v>
+      </c>
+      <c r="B926" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C926" t="s">
+        <v>14</v>
+      </c>
+      <c r="D926" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E926" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F926" t="s">
+        <v>4492</v>
+      </c>
+      <c r="G926" t="s">
+        <v>4493</v>
+      </c>
+      <c r="H926" t="s">
+        <v>300</v>
+      </c>
+      <c r="I926" t="s">
+        <v>3962</v>
+      </c>
+      <c r="J926" t="s">
+        <v>366</v>
+      </c>
+      <c r="K926" t="s">
+        <v>4494</v>
+      </c>
+      <c r="L926" t="s">
+        <v>4495</v>
+      </c>
+    </row>
+    <row r="927" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A927">
+        <v>926</v>
+      </c>
+      <c r="B927" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C927" t="s">
+        <v>14</v>
+      </c>
+      <c r="D927" t="s">
+        <v>3962</v>
+      </c>
+      <c r="E927" t="s">
+        <v>3962</v>
+      </c>
+      <c r="F927" t="s">
+        <v>4496</v>
+      </c>
+      <c r="G927" t="s">
+        <v>4497</v>
+      </c>
+      <c r="H927" t="s">
+        <v>300</v>
+      </c>
+      <c r="I927" t="s">
+        <v>4498</v>
+      </c>
+      <c r="J927" t="s">
+        <v>366</v>
+      </c>
+      <c r="K927" t="s">
+        <v>4499</v>
+      </c>
+      <c r="L927" t="s">
+        <v>4500</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 WebKreatives OSM leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8973" uniqueCount="5114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8995" uniqueCount="5122">
   <si>
     <t>#</t>
   </si>
@@ -15353,6 +15353,30 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:2725646428 | Source: OpenStreetMap | schoonheidssalon | Arnhem | Website: https://www.lumebeautystudio.nl</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>somluck.thida@gmail.com</t>
+  </si>
+  <si>
+    <t>Sommy Nails</t>
+  </si>
+  <si>
+    <t>+31 6 28295370</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2726500262 | Source: OpenStreetMap | schoonheidssalon | Arnhem | Website: https://sommynails.nl</t>
+  </si>
+  <si>
+    <t>info@nillyskinmaster.nl</t>
+  </si>
+  <si>
+    <t>Nilly Skin Master</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:13724282302 | Source: OpenStreetMap | schoonheidssalon | Arnhem | Website: https://nillyskinmaster.nl</t>
   </si>
 </sst>
 </file>
@@ -15729,8 +15753,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1044"/>
-  <sheetFormatPr customHeight="1"/>
+  <dimension ref="A1:L1046"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -18633,7 +18657,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -47871,6 +47895,82 @@
         <v>5113</v>
       </c>
     </row>
+    <row r="1045" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1045">
+        <v>1048</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>1862</v>
+      </c>
+      <c r="C1045" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1045" t="s">
+        <v>5114</v>
+      </c>
+      <c r="E1045" t="s">
+        <v>5114</v>
+      </c>
+      <c r="F1045" t="s">
+        <v>5115</v>
+      </c>
+      <c r="G1045" t="s">
+        <v>5116</v>
+      </c>
+      <c r="H1045" t="s">
+        <v>343</v>
+      </c>
+      <c r="I1045" t="s">
+        <v>5087</v>
+      </c>
+      <c r="J1045" t="s">
+        <v>2717</v>
+      </c>
+      <c r="K1045" t="s">
+        <v>5117</v>
+      </c>
+      <c r="L1045" t="s">
+        <v>5118</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1046">
+        <v>1049</v>
+      </c>
+      <c r="B1046" t="s">
+        <v>1862</v>
+      </c>
+      <c r="C1046" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1046" t="s">
+        <v>5114</v>
+      </c>
+      <c r="E1046" t="s">
+        <v>5114</v>
+      </c>
+      <c r="F1046" t="s">
+        <v>5119</v>
+      </c>
+      <c r="G1046" t="s">
+        <v>5120</v>
+      </c>
+      <c r="H1046" t="s">
+        <v>343</v>
+      </c>
+      <c r="I1046" t="s">
+        <v>5114</v>
+      </c>
+      <c r="J1046" t="s">
+        <v>2717</v>
+      </c>
+      <c r="K1046" t="s">
+        <v>5114</v>
+      </c>
+      <c r="L1046" t="s">
+        <v>5121</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record outreach batch 374-393
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -14616,7 +14616,7 @@
         <v>374</v>
       </c>
       <c r="B375" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C375" t="str">
         <v>No</v>
@@ -14646,7 +14646,7 @@
         <v/>
       </c>
       <c r="L375" t="str">
-        <v>Website available | Email from website | OSM id:2728925490 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://petsenco.nl/item/lobbes</v>
+        <v>Website available | Email from website | OSM id:2728925490 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://petsenco.nl/item/lobbes | Outreach sent 2026-05-25T14:01:18.953Z label-ok</v>
       </c>
     </row>
     <row r="376">
@@ -14654,7 +14654,7 @@
         <v>375</v>
       </c>
       <c r="B376" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C376" t="str">
         <v>No</v>
@@ -14684,7 +14684,7 @@
         <v>+31 76 520 7037</v>
       </c>
       <c r="L376" t="str">
-        <v>Website available | Email from website | OSM id:2737934129 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://dierspecialist.nl</v>
+        <v>Website available | Email from website | OSM id:2737934129 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://dierspecialist.nl | Outreach sent 2026-05-25T14:01:22.303Z label-ok</v>
       </c>
     </row>
     <row r="377">
@@ -14692,7 +14692,7 @@
         <v>376</v>
       </c>
       <c r="B377" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C377" t="str">
         <v>No</v>
@@ -14722,7 +14722,7 @@
         <v>+31 76 303 05 04</v>
       </c>
       <c r="L377" t="str">
-        <v>Website available | Email from OSM | OSM id:2738419997 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://www.maxizoo.nl/winkels/maxi-zoo-breda</v>
+        <v>Website available | Email from OSM | OSM id:2738419997 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://www.maxizoo.nl/winkels/maxi-zoo-breda | Outreach sent 2026-05-25T14:01:25.405Z label-ok</v>
       </c>
     </row>
     <row r="378">
@@ -14730,7 +14730,7 @@
         <v>377</v>
       </c>
       <c r="B378" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C378" t="str">
         <v>No</v>
@@ -14760,7 +14760,7 @@
         <v>+31 76 560 2217</v>
       </c>
       <c r="L378" t="str">
-        <v>Website available | Email from OSM | OSM id:5433182112 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://dierspecialist.nl</v>
+        <v>Website available | Email from OSM | OSM id:5433182112 | Source: OpenStreetMap | dierenwinkel | Breda | Website: https://dierspecialist.nl | Outreach sent 2026-05-25T14:01:28.860Z label-ok</v>
       </c>
     </row>
     <row r="379">
@@ -14768,7 +14768,7 @@
         <v>378</v>
       </c>
       <c r="B379" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C379" t="str">
         <v>No</v>
@@ -14798,7 +14798,7 @@
         <v>+31 55 599 4433</v>
       </c>
       <c r="L379" t="str">
-        <v>Website available | Email from OSM | OSM id:2685596310 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: https://p-c-a.nl</v>
+        <v>Website available | Email from OSM | OSM id:2685596310 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: https://p-c-a.nl | Outreach sent 2026-05-25T14:01:32.653Z label-ok</v>
       </c>
     </row>
     <row r="380">
@@ -14806,7 +14806,7 @@
         <v>379</v>
       </c>
       <c r="B380" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C380" t="str">
         <v>No</v>
@@ -14836,7 +14836,7 @@
         <v>+31 55 366 7160</v>
       </c>
       <c r="L380" t="str">
-        <v>Website available | Email from OSM | OSM id:2686214962 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: https://www.jonker-schilders.nl</v>
+        <v>Website available | Email from OSM | OSM id:2686214962 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: https://www.jonker-schilders.nl | Outreach sent 2026-05-25T14:01:39.014Z label-ok</v>
       </c>
     </row>
     <row r="381">
@@ -14844,7 +14844,7 @@
         <v>380</v>
       </c>
       <c r="B381" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C381" t="str">
         <v>No</v>
@@ -14874,7 +14874,7 @@
         <v>+31 55 541 5140</v>
       </c>
       <c r="L381" t="str">
-        <v>Website available | Email from OSM | OSM id:2686869292 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: http://www.kleverwal.nl</v>
+        <v>Website available | Email from OSM | OSM id:2686869292 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: http://www.kleverwal.nl | Outreach sent 2026-05-25T14:01:42.498Z label-ok</v>
       </c>
     </row>
     <row r="382">
@@ -14882,7 +14882,7 @@
         <v>381</v>
       </c>
       <c r="B382" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C382" t="str">
         <v>No</v>
@@ -14912,7 +14912,7 @@
         <v>+31 55 542 4079</v>
       </c>
       <c r="L382" t="str">
-        <v>Website available | Email from OSM | OSM id:4886443401 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: https://www.stevenjansen.nl</v>
+        <v>Website available | Email from OSM | OSM id:4886443401 | Source: OpenStreetMap | schildersbedrijf | Apeldoorn | Website: https://www.stevenjansen.nl | Outreach sent 2026-05-25T14:01:45.368Z label-ok</v>
       </c>
     </row>
     <row r="383">
@@ -14920,7 +14920,7 @@
         <v>382</v>
       </c>
       <c r="B383" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C383" t="str">
         <v>No</v>
@@ -14950,7 +14950,7 @@
         <v/>
       </c>
       <c r="L383" t="str">
-        <v>Website available | Email from website | OSM id:12441285873 | Source: OpenStreetMap | elektricien | Amsterdam | Website: https://www.bruens-electrotechniek.nl</v>
+        <v>Website available | Email from website | OSM id:12441285873 | Source: OpenStreetMap | elektricien | Amsterdam | Website: https://www.bruens-electrotechniek.nl | Outreach sent 2026-05-25T14:01:48.311Z label-ok</v>
       </c>
     </row>
     <row r="384">
@@ -14958,7 +14958,7 @@
         <v>383</v>
       </c>
       <c r="B384" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C384" t="str">
         <v>No</v>
@@ -14988,7 +14988,7 @@
         <v/>
       </c>
       <c r="L384" t="str">
-        <v>Website available | Email from website | OSM id:5216297293 | Source: OpenStreetMap | rijschool | Tilburg | Website: https://www.verkeersschooltilburg.nl</v>
+        <v>Website available | Email from website | OSM id:5216297293 | Source: OpenStreetMap | rijschool | Tilburg | Website: https://www.verkeersschooltilburg.nl | Outreach sent 2026-05-25T14:01:51.269Z label-ok</v>
       </c>
     </row>
     <row r="385">
@@ -14996,7 +14996,7 @@
         <v>384</v>
       </c>
       <c r="B385" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C385" t="str">
         <v>No</v>
@@ -15026,7 +15026,7 @@
         <v>+31 75 614 2561</v>
       </c>
       <c r="L385" t="str">
-        <v>Website available | Email from website | OSM id:2895411254 | Source: OpenStreetMap | kapsalon | Zaandam | Website: https://www.kapsalonloes.nl</v>
+        <v>Website available | Email from website | OSM id:2895411254 | Source: OpenStreetMap | kapsalon | Zaandam | Website: https://www.kapsalonloes.nl | Outreach sent 2026-05-25T14:01:54.176Z label-ok</v>
       </c>
     </row>
     <row r="386">
@@ -15034,7 +15034,7 @@
         <v>385</v>
       </c>
       <c r="B386" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C386" t="str">
         <v>No</v>
@@ -15064,7 +15064,7 @@
         <v/>
       </c>
       <c r="L386" t="str">
-        <v>Website available | Email from website | OSM id:2896081290 | Source: OpenStreetMap | kapsalon | Zaandam | Website: http://gulcetabu.com</v>
+        <v>Website available | Email from website | OSM id:2896081290 | Source: OpenStreetMap | kapsalon | Zaandam | Website: http://gulcetabu.com | Outreach sent 2026-05-25T14:01:57.139Z label-ok</v>
       </c>
     </row>
     <row r="387">
@@ -15072,7 +15072,7 @@
         <v>386</v>
       </c>
       <c r="B387" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C387" t="str">
         <v>No</v>
@@ -15102,7 +15102,7 @@
         <v>+31 75 6141420</v>
       </c>
       <c r="L387" t="str">
-        <v>Website available | Email from website | OSM id:2896128432 | Source: OpenStreetMap | kapsalon | Zaandam | Website: https://www.dekapperzaandam.nl</v>
+        <v>Website available | Email from website | OSM id:2896128432 | Source: OpenStreetMap | kapsalon | Zaandam | Website: https://www.dekapperzaandam.nl | Outreach sent 2026-05-25T14:02:00.144Z label-ok</v>
       </c>
     </row>
     <row r="388">
@@ -15110,7 +15110,7 @@
         <v>387</v>
       </c>
       <c r="B388" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C388" t="str">
         <v>No</v>
@@ -15140,7 +15140,7 @@
         <v/>
       </c>
       <c r="L388" t="str">
-        <v>Website available | Email from website | OSM id:2747586448 | Source: OpenStreetMap | schoonheidssalon | Enschede | Website: https://headspaenschede.nl</v>
+        <v>Website available | Email from website | OSM id:2747586448 | Source: OpenStreetMap | schoonheidssalon | Enschede | Website: https://headspaenschede.nl | Outreach sent 2026-05-25T14:02:03.077Z label-ok</v>
       </c>
     </row>
     <row r="389">
@@ -15148,7 +15148,7 @@
         <v>388</v>
       </c>
       <c r="B389" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C389" t="str">
         <v>No</v>
@@ -15178,7 +15178,7 @@
         <v>+31 6 12 02 4200</v>
       </c>
       <c r="L389" t="str">
-        <v>Website available | Email from OSM | OSM id:2775683614 | Source: OpenStreetMap | schoonheidssalon | Enschede | Website: https://moonsbeauty.nl</v>
+        <v>Website available | Email from OSM | OSM id:2775683614 | Source: OpenStreetMap | schoonheidssalon | Enschede | Website: https://moonsbeauty.nl | Outreach sent 2026-05-25T14:02:06.135Z label-ok</v>
       </c>
     </row>
     <row r="390">
@@ -15186,7 +15186,7 @@
         <v>389</v>
       </c>
       <c r="B390" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C390" t="str">
         <v>No</v>
@@ -15216,7 +15216,7 @@
         <v/>
       </c>
       <c r="L390" t="str">
-        <v>Website available | Email from website | OSM id:5810505906 | Source: OpenStreetMap | schoonheidssalon | Enschede | Website: https://my-glow.nl</v>
+        <v>Website available | Email from website | OSM id:5810505906 | Source: OpenStreetMap | schoonheidssalon | Enschede | Website: https://my-glow.nl | Outreach sent 2026-05-25T14:02:09.089Z label-ok</v>
       </c>
     </row>
     <row r="391">
@@ -15224,7 +15224,7 @@
         <v>390</v>
       </c>
       <c r="B391" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C391" t="str">
         <v>No</v>
@@ -15254,7 +15254,7 @@
         <v/>
       </c>
       <c r="L391" t="str">
-        <v>Website available | Email from website | OSM id:2610207121 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://bluehawaiitattoo.nl</v>
+        <v>Website available | Email from website | OSM id:2610207121 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://bluehawaiitattoo.nl | Outreach sent 2026-05-25T14:02:12.013Z label-ok</v>
       </c>
     </row>
     <row r="392">
@@ -15262,7 +15262,7 @@
         <v>391</v>
       </c>
       <c r="B392" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C392" t="str">
         <v>No</v>
@@ -15292,7 +15292,7 @@
         <v>+31 10 8452495</v>
       </c>
       <c r="L392" t="str">
-        <v>Website available | Email from website | OSM id:2610245941 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://www.wallsandskin.com/rotterdam</v>
+        <v>Website available | Email from website | OSM id:2610245941 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://www.wallsandskin.com/rotterdam | Outreach sent 2026-05-25T14:02:14.893Z label-ok</v>
       </c>
     </row>
     <row r="393">
@@ -15300,7 +15300,7 @@
         <v>392</v>
       </c>
       <c r="B393" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C393" t="str">
         <v>No</v>
@@ -15330,7 +15330,7 @@
         <v>+31 6 43589182</v>
       </c>
       <c r="L393" t="str">
-        <v>Website available | Email from website | OSM id:2798596721 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://vean-tattoo.nl</v>
+        <v>Website available | Email from website | OSM id:2798596721 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://vean-tattoo.nl | Outreach sent 2026-05-25T14:02:17.933Z label-ok</v>
       </c>
     </row>
     <row r="394">
@@ -15338,7 +15338,7 @@
         <v>393</v>
       </c>
       <c r="B394" t="str">
-        <v>Not Yet</v>
+        <v>Yes</v>
       </c>
       <c r="C394" t="str">
         <v>No</v>
@@ -15368,7 +15368,7 @@
         <v>+31 10 845 8173</v>
       </c>
       <c r="L394" t="str">
-        <v>Website available | Email from website | OSM id:2814019662 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://www.studionoorderzon.com</v>
+        <v>Website available | Email from website | OSM id:2814019662 | Source: OpenStreetMap | tattooshop | Rotterdam | Website: https://www.studionoorderzon.com | Outreach sent 2026-05-25T14:02:21.008Z label-ok</v>
       </c>
     </row>
     <row r="395">

</xml_diff>

<commit_message>
Add 36 WebKreatives OSM leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10263" uniqueCount="5750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10659" uniqueCount="5910">
   <si>
     <t>#</t>
   </si>
@@ -17261,6 +17261,486 @@
   </si>
   <si>
     <t>Website available | Email from OSM | OSM id:2737778688 | Source: OpenStreetMap | schoonheidssalon | Apeldoorn | Website: https://www.purewellnesshair.nl</t>
+  </si>
+  <si>
+    <t>info@weersel.nl</t>
+  </si>
+  <si>
+    <t>van Weersel</t>
+  </si>
+  <si>
+    <t>Oldenzaalsestraat 7514DS</t>
+  </si>
+  <si>
+    <t>+31 53 435 4628</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2760960078 | Source: OpenStreetMap | muziekwinkel | Enschede | Website: https://www.weersel.nl</t>
+  </si>
+  <si>
+    <t>webshop@zooveel.nl</t>
+  </si>
+  <si>
+    <t>Zooveel</t>
+  </si>
+  <si>
+    <t>Lage Bothofstraat 7533AS</t>
+  </si>
+  <si>
+    <t>+31 53 432 7353</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:4386456496 | Source: OpenStreetMap | dierenwinkel | Enschede | Website: https://www.zooveel.nl</t>
+  </si>
+  <si>
+    <t>klantenservice@toppets.nl</t>
+  </si>
+  <si>
+    <t>TopPets</t>
+  </si>
+  <si>
+    <t>+31 53 230 4794</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:4659344442 | Source: OpenStreetMap | dierenwinkel | Enschede | Website: https://www.toppets.nl</t>
+  </si>
+  <si>
+    <t>info@kuipersdthshop.nl</t>
+  </si>
+  <si>
+    <t>De Dierenwinkel</t>
+  </si>
+  <si>
+    <t>+31 53 476 7797</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:9930157871 | Source: OpenStreetMap | dierenwinkel | Enschede | Website: https://www.kuipersdthshop.nl</t>
+  </si>
+  <si>
+    <t>info@meerdanschilderwerk.nl</t>
+  </si>
+  <si>
+    <t>De Kooter Spuit- en Schilderwerk</t>
+  </si>
+  <si>
+    <t>Klaproosstraat 7514XR</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2760972494 | Source: OpenStreetMap | schildersbedrijf | Enschede | Website: https://www.meerdanschilderwerk.nl</t>
+  </si>
+  <si>
+    <t>info.enschede@kropman.nl</t>
+  </si>
+  <si>
+    <t>Kropman</t>
+  </si>
+  <si>
+    <t>Twekkeler Es 7547ST</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:8863267691 | Source: OpenStreetMap | elektricien | Enschede | Website: https://kropman.nl</t>
+  </si>
+  <si>
+    <t>info@polhuistotaal.nl</t>
+  </si>
+  <si>
+    <t>Polhuis Totaal Installatie</t>
+  </si>
+  <si>
+    <t>Lossersestraat</t>
+  </si>
+  <si>
+    <t>+31 53 536 1626</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:12165544887 | Source: OpenStreetMap | elektricien | Enschede | Website: https://polhuistotaal.nl</t>
+  </si>
+  <si>
+    <t>gering@houtenbeton.nl</t>
+  </si>
+  <si>
+    <t>Gering Hout &amp; Beton B.V.</t>
+  </si>
+  <si>
+    <t>Vosbultweg 7532AW</t>
+  </si>
+  <si>
+    <t>+31 53 461 1737</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2763487216 | Source: OpenStreetMap | klussenbedrijf | Enschede | Website: https://www.gering.nl</t>
+  </si>
+  <si>
+    <t>jamie@home.nl</t>
+  </si>
+  <si>
+    <t>Rijschool Homeijer</t>
+  </si>
+  <si>
+    <t>Jupiterstraat 7521JM</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2747582757 | Source: OpenStreetMap | rijschool | Enschede | Website: https://homeijer.nl</t>
+  </si>
+  <si>
+    <t>info@pinnadelicatessen.nl</t>
+  </si>
+  <si>
+    <t>Pinna</t>
+  </si>
+  <si>
+    <t>Chrysantstraat 7531KD</t>
+  </si>
+  <si>
+    <t>+31 53 785 2724</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:5483577530 | Source: OpenStreetMap | traiteur | Enschede | Website: https://pinnadelicatessen.nl</t>
+  </si>
+  <si>
+    <t>info@gastrovinovaneker.nl</t>
+  </si>
+  <si>
+    <t>Gastrovino Vaneker</t>
+  </si>
+  <si>
+    <t>+31 53 476 8300</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:9930157861 | Source: OpenStreetMap | traiteur | Enschede | Website: https://www.gastrovinovaneker.nl</t>
+  </si>
+  <si>
+    <t>info@eastsidetattoo.nl</t>
+  </si>
+  <si>
+    <t>Eastside Tattoo</t>
+  </si>
+  <si>
+    <t>Korte Haaksbergerstraat 7511JS</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2775263683 | Source: OpenStreetMap | tattooshop | Enschede | Website: https://eastsidetattoo.nl</t>
+  </si>
+  <si>
+    <t>info@damhuisbiketotaal.nl</t>
+  </si>
+  <si>
+    <t>Bike Totaal Damhuis</t>
+  </si>
+  <si>
+    <t>Gronausestraat 7534AR</t>
+  </si>
+  <si>
+    <t>+31 53 461 1807</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:243725566 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://biketotaaldamhuis.nl</t>
+  </si>
+  <si>
+    <t>info@koelemanrijwielen.nl</t>
+  </si>
+  <si>
+    <t>Koeleman Rijwielen</t>
+  </si>
+  <si>
+    <t>+31 53 431 5995</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:1242510301 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.koelemanrijwielen.nl</t>
+  </si>
+  <si>
+    <t>info@kroezetweewielers.nl</t>
+  </si>
+  <si>
+    <t>Kroeze tweewielers</t>
+  </si>
+  <si>
+    <t>Kerkstraat 7532AV</t>
+  </si>
+  <si>
+    <t>+31 53 461 1297</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:1989929672 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.kroezetweewielers.nl</t>
+  </si>
+  <si>
+    <t>info@go-fietsservice.nl</t>
+  </si>
+  <si>
+    <t>Go-fietsservice</t>
+  </si>
+  <si>
+    <t>G.J. van Heekstraat 7521EB</t>
+  </si>
+  <si>
+    <t>+31 6 12707522</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2747582043 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.go-fietsservice.nl</t>
+  </si>
+  <si>
+    <t>deversnelling@detwentsezorgcentra.nl</t>
+  </si>
+  <si>
+    <t>de Versnelling</t>
+  </si>
+  <si>
+    <t>Calslaan 7522MG</t>
+  </si>
+  <si>
+    <t>+31 88 430 63 15</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2749686732 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.deversnelling.nl</t>
+  </si>
+  <si>
+    <t>info@josharmelink.nl</t>
+  </si>
+  <si>
+    <t>Jos Harmelink</t>
+  </si>
+  <si>
+    <t>Deurningerstraat 7522CM</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2750224336 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: http://www.josharmelink.nl</t>
+  </si>
+  <si>
+    <t>budgetbikeshoeve@gmail.com</t>
+  </si>
+  <si>
+    <t>Budget Bikes Hoeve</t>
+  </si>
+  <si>
+    <t>Kanaalstraat 7547AR</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2755970659 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.budgetbikeshoeve.nl</t>
+  </si>
+  <si>
+    <t>info@oudeheuvel2wielers.nl</t>
+  </si>
+  <si>
+    <t>Oude Heuvel</t>
+  </si>
+  <si>
+    <t>Gronausestraat 7534AN</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2762184937 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.oudeheuvel2wielers.nl</t>
+  </si>
+  <si>
+    <t>info@biketotaallandewe.nl</t>
+  </si>
+  <si>
+    <t>Bike Totaal Landewé</t>
+  </si>
+  <si>
+    <t>Broekheurnerweg 7513ES</t>
+  </si>
+  <si>
+    <t>+31 53 431 5952</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2775689369 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.landewe.nl</t>
+  </si>
+  <si>
+    <t>info@freddystweewielers.nl</t>
+  </si>
+  <si>
+    <t>Freddy's Tweewielers</t>
+  </si>
+  <si>
+    <t>+31 53 431 2627</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2775690410 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: http://www.freddystweewielers.nl</t>
+  </si>
+  <si>
+    <t>info@snellersfietsen.nl</t>
+  </si>
+  <si>
+    <t>Snellers</t>
+  </si>
+  <si>
+    <t>Haaksbergerstraat 7513EA</t>
+  </si>
+  <si>
+    <t>+31 53 432 22 23</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:4414906528 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.snellersfietsen.nl/fietsenwinkel-enschede</t>
+  </si>
+  <si>
+    <t>info@falagro.nl</t>
+  </si>
+  <si>
+    <t>Falagro</t>
+  </si>
+  <si>
+    <t>+31 53 740 0530</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:9930157870 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.falagro.nl</t>
+  </si>
+  <si>
+    <t>info@piest.nl</t>
+  </si>
+  <si>
+    <t>Piest</t>
+  </si>
+  <si>
+    <t>Olieslagweg 7521HX</t>
+  </si>
+  <si>
+    <t>+31 53 435 9112</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:10556711960 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://www.piest.nl/fietsen-e-bikes</t>
+  </si>
+  <si>
+    <t>roel@wielerstudio.nl</t>
+  </si>
+  <si>
+    <t>Wielerstudio</t>
+  </si>
+  <si>
+    <t>Goolkatenweg 7521BE</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:11439966202 | Source: OpenStreetMap | fietsenwinkel | Enschede | Website: https://wielerstudio.nl</t>
+  </si>
+  <si>
+    <t>info@slagerijlohman.nl</t>
+  </si>
+  <si>
+    <t>Jos Lohman</t>
+  </si>
+  <si>
+    <t>+31 53 435 7349</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:819708867 | Source: OpenStreetMap | slager | Enschede | Website: https://www.slagerijlohman.nl</t>
+  </si>
+  <si>
+    <t>info@elzinga.keurslager.nl</t>
+  </si>
+  <si>
+    <t>Elzinga</t>
+  </si>
+  <si>
+    <t>+31 53 476 5685</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:9930157865 | Source: OpenStreetMap | slager | Enschede | Website: https://elzinga.keurslager.nl</t>
+  </si>
+  <si>
+    <t>info@poelier-mattemaker.nl</t>
+  </si>
+  <si>
+    <t>Poelier Mattemaker</t>
+  </si>
+  <si>
+    <t>Pijpenstraat 7511GM</t>
+  </si>
+  <si>
+    <t>+31 53 432 3906</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:10089437647 | Source: OpenStreetMap | slager | Enschede | Website: https://www.poelier-mattemaker.nl</t>
+  </si>
+  <si>
+    <t>deppenbroek@bakkerijnollen.nl</t>
+  </si>
+  <si>
+    <t>Nollen</t>
+  </si>
+  <si>
+    <t>+31 53 434 5958</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:819708969 | Source: OpenStreetMap | bakkerij | Enschede | Website: https://www.bakkerijnollen.nl/winkels/enschede-deppenbroek</t>
+  </si>
+  <si>
+    <t>enschede@hush.nl</t>
+  </si>
+  <si>
+    <t>Hush</t>
+  </si>
+  <si>
+    <t>+31 88 1344002</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:11435599457 | Source: OpenStreetMap | bakkerij | Enschede | Website: https://www.hush.nl/lunch-in-enschede</t>
+  </si>
+  <si>
+    <t>info@bloemenboetiek-stadsveld.nl</t>
+  </si>
+  <si>
+    <t>Bloemenboetiek Stadsveld</t>
+  </si>
+  <si>
+    <t>Zweringweg 7545DA</t>
+  </si>
+  <si>
+    <t>+31 53 478 5105</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2744509901 | Source: OpenStreetMap | bloemist | Enschede | Website: https://www.bloemenboetiek-stadsveld.nl</t>
+  </si>
+  <si>
+    <t>info@mekkelholt-bloemen.nl</t>
+  </si>
+  <si>
+    <t>Bloemsierkunst 't Mekkelholt</t>
+  </si>
+  <si>
+    <t>Brouwerijstraat 7523XE</t>
+  </si>
+  <si>
+    <t>+31 53 435 7482</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2750247474 | Source: OpenStreetMap | bloemist | Enschede | Website: https://www.mekkelholt-bloemen.nl/bloemwinkel-roombeek</t>
+  </si>
+  <si>
+    <t>info@bloemsierkunstflorade.nl</t>
+  </si>
+  <si>
+    <t>Florade</t>
+  </si>
+  <si>
+    <t>+31 53 785 7323</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2761327760 | Source: OpenStreetMap | bloemist | Enschede | Website: https://bloemsierkunstflorade.nl</t>
+  </si>
+  <si>
+    <t>info@tombloemen.nl</t>
+  </si>
+  <si>
+    <t>TOM bloemen &amp; wonen</t>
+  </si>
+  <si>
+    <t>Fresiastraat 7531VJ</t>
+  </si>
+  <si>
+    <t>+31 53 303 4599</t>
+  </si>
+  <si>
+    <t>Website available | Email from OSM | OSM id:2761336741 | Source: OpenStreetMap | bloemist | Enschede | Website: https://www.tombloemen.nl</t>
+  </si>
+  <si>
+    <t>info@bloemsierkunstmimosa.nl</t>
+  </si>
+  <si>
+    <t>Mimosa</t>
+  </si>
+  <si>
+    <t>Korte Hengelosestraat 7511JA</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:4959131889 | Source: OpenStreetMap | bloemist | Enschede | Website: https://www.bloemsierkunstmimosa.nl</t>
   </si>
 </sst>
 </file>
@@ -17637,8 +18117,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1181"/>
-  <sheetFormatPr customHeight="1"/>
+  <dimension ref="A1:L1217"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -54334,6 +54814,1374 @@
         <v>5749</v>
       </c>
     </row>
+    <row r="1182" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1182">
+        <v>1185</v>
+      </c>
+      <c r="B1182" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1182" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1182" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1182" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1182" t="s">
+        <v>5750</v>
+      </c>
+      <c r="G1182" t="s">
+        <v>5751</v>
+      </c>
+      <c r="H1182" t="s">
+        <v>716</v>
+      </c>
+      <c r="I1182" t="s">
+        <v>5752</v>
+      </c>
+      <c r="J1182" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1182" t="s">
+        <v>5753</v>
+      </c>
+      <c r="L1182" t="s">
+        <v>5754</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1183">
+        <v>1186</v>
+      </c>
+      <c r="B1183" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1183" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1183" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1183" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1183" t="s">
+        <v>5755</v>
+      </c>
+      <c r="G1183" t="s">
+        <v>5756</v>
+      </c>
+      <c r="H1183" t="s">
+        <v>2054</v>
+      </c>
+      <c r="I1183" t="s">
+        <v>5757</v>
+      </c>
+      <c r="J1183" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1183" t="s">
+        <v>5758</v>
+      </c>
+      <c r="L1183" t="s">
+        <v>5759</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1184">
+        <v>1187</v>
+      </c>
+      <c r="B1184" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1184" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1184" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1184" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1184" t="s">
+        <v>5760</v>
+      </c>
+      <c r="G1184" t="s">
+        <v>5761</v>
+      </c>
+      <c r="H1184" t="s">
+        <v>2054</v>
+      </c>
+      <c r="I1184" t="s">
+        <v>2117</v>
+      </c>
+      <c r="J1184" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1184" t="s">
+        <v>5762</v>
+      </c>
+      <c r="L1184" t="s">
+        <v>5763</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1185">
+        <v>1188</v>
+      </c>
+      <c r="B1185" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1185" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1185" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1185" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1185" t="s">
+        <v>5764</v>
+      </c>
+      <c r="G1185" t="s">
+        <v>5765</v>
+      </c>
+      <c r="H1185" t="s">
+        <v>2054</v>
+      </c>
+      <c r="I1185" t="s">
+        <v>1970</v>
+      </c>
+      <c r="J1185" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1185" t="s">
+        <v>5766</v>
+      </c>
+      <c r="L1185" t="s">
+        <v>5767</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1186">
+        <v>1189</v>
+      </c>
+      <c r="B1186" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1186" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1186" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1186" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1186" t="s">
+        <v>5768</v>
+      </c>
+      <c r="G1186" t="s">
+        <v>5769</v>
+      </c>
+      <c r="H1186" t="s">
+        <v>290</v>
+      </c>
+      <c r="I1186" t="s">
+        <v>5770</v>
+      </c>
+      <c r="J1186" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1186" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1186" t="s">
+        <v>5771</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1187">
+        <v>1190</v>
+      </c>
+      <c r="B1187" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1187" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1187" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1187" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1187" t="s">
+        <v>5772</v>
+      </c>
+      <c r="G1187" t="s">
+        <v>5773</v>
+      </c>
+      <c r="H1187" t="s">
+        <v>380</v>
+      </c>
+      <c r="I1187" t="s">
+        <v>5774</v>
+      </c>
+      <c r="J1187" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1187" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1187" t="s">
+        <v>5775</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1188">
+        <v>1191</v>
+      </c>
+      <c r="B1188" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1188" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1188" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1188" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1188" t="s">
+        <v>5776</v>
+      </c>
+      <c r="G1188" t="s">
+        <v>5777</v>
+      </c>
+      <c r="H1188" t="s">
+        <v>380</v>
+      </c>
+      <c r="I1188" t="s">
+        <v>5778</v>
+      </c>
+      <c r="J1188" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1188" t="s">
+        <v>5779</v>
+      </c>
+      <c r="L1188" t="s">
+        <v>5780</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1189">
+        <v>1192</v>
+      </c>
+      <c r="B1189" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1189" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1189" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1189" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1189" t="s">
+        <v>5781</v>
+      </c>
+      <c r="G1189" t="s">
+        <v>5782</v>
+      </c>
+      <c r="H1189" t="s">
+        <v>1907</v>
+      </c>
+      <c r="I1189" t="s">
+        <v>5783</v>
+      </c>
+      <c r="J1189" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1189" t="s">
+        <v>5784</v>
+      </c>
+      <c r="L1189" t="s">
+        <v>5785</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1190">
+        <v>1193</v>
+      </c>
+      <c r="B1190" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1190" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1190" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1190" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1190" t="s">
+        <v>5786</v>
+      </c>
+      <c r="G1190" t="s">
+        <v>5787</v>
+      </c>
+      <c r="H1190" t="s">
+        <v>370</v>
+      </c>
+      <c r="I1190" t="s">
+        <v>5788</v>
+      </c>
+      <c r="J1190" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1190" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1190" t="s">
+        <v>5789</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1191">
+        <v>1194</v>
+      </c>
+      <c r="B1191" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1191" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1191" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1191" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1191" t="s">
+        <v>5790</v>
+      </c>
+      <c r="G1191" t="s">
+        <v>5791</v>
+      </c>
+      <c r="H1191" t="s">
+        <v>2444</v>
+      </c>
+      <c r="I1191" t="s">
+        <v>5792</v>
+      </c>
+      <c r="J1191" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1191" t="s">
+        <v>5793</v>
+      </c>
+      <c r="L1191" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1192">
+        <v>1195</v>
+      </c>
+      <c r="B1192" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1192" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1192" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1192" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1192" t="s">
+        <v>5795</v>
+      </c>
+      <c r="G1192" t="s">
+        <v>5796</v>
+      </c>
+      <c r="H1192" t="s">
+        <v>2444</v>
+      </c>
+      <c r="I1192" t="s">
+        <v>1970</v>
+      </c>
+      <c r="J1192" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1192" t="s">
+        <v>5797</v>
+      </c>
+      <c r="L1192" t="s">
+        <v>5798</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1193">
+        <v>1196</v>
+      </c>
+      <c r="B1193" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1193" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1193" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1193" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1193" t="s">
+        <v>5799</v>
+      </c>
+      <c r="G1193" t="s">
+        <v>5800</v>
+      </c>
+      <c r="H1193" t="s">
+        <v>1975</v>
+      </c>
+      <c r="I1193" t="s">
+        <v>5801</v>
+      </c>
+      <c r="J1193" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1193" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1193" t="s">
+        <v>5802</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1194">
+        <v>1197</v>
+      </c>
+      <c r="B1194" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1194" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1194" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1194" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1194" t="s">
+        <v>5803</v>
+      </c>
+      <c r="G1194" t="s">
+        <v>5804</v>
+      </c>
+      <c r="H1194" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1194" t="s">
+        <v>5805</v>
+      </c>
+      <c r="J1194" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1194" t="s">
+        <v>5806</v>
+      </c>
+      <c r="L1194" t="s">
+        <v>5807</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1195">
+        <v>1198</v>
+      </c>
+      <c r="B1195" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1195" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1195" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1195" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1195" t="s">
+        <v>5808</v>
+      </c>
+      <c r="G1195" t="s">
+        <v>5809</v>
+      </c>
+      <c r="H1195" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1195" t="s">
+        <v>1916</v>
+      </c>
+      <c r="J1195" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1195" t="s">
+        <v>5810</v>
+      </c>
+      <c r="L1195" t="s">
+        <v>5811</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1196">
+        <v>1199</v>
+      </c>
+      <c r="B1196" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1196" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1196" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1196" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1196" t="s">
+        <v>5812</v>
+      </c>
+      <c r="G1196" t="s">
+        <v>5813</v>
+      </c>
+      <c r="H1196" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1196" t="s">
+        <v>5814</v>
+      </c>
+      <c r="J1196" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1196" t="s">
+        <v>5815</v>
+      </c>
+      <c r="L1196" t="s">
+        <v>5816</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1197">
+        <v>1200</v>
+      </c>
+      <c r="B1197" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1197" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1197" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1197" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1197" t="s">
+        <v>5817</v>
+      </c>
+      <c r="G1197" t="s">
+        <v>5818</v>
+      </c>
+      <c r="H1197" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1197" t="s">
+        <v>5819</v>
+      </c>
+      <c r="J1197" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1197" t="s">
+        <v>5820</v>
+      </c>
+      <c r="L1197" t="s">
+        <v>5821</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1198">
+        <v>1201</v>
+      </c>
+      <c r="B1198" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1198" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1198" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1198" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1198" t="s">
+        <v>5822</v>
+      </c>
+      <c r="G1198" t="s">
+        <v>5823</v>
+      </c>
+      <c r="H1198" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1198" t="s">
+        <v>5824</v>
+      </c>
+      <c r="J1198" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1198" t="s">
+        <v>5825</v>
+      </c>
+      <c r="L1198" t="s">
+        <v>5826</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1199">
+        <v>1202</v>
+      </c>
+      <c r="B1199" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1199" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1199" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1199" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1199" t="s">
+        <v>5827</v>
+      </c>
+      <c r="G1199" t="s">
+        <v>5828</v>
+      </c>
+      <c r="H1199" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1199" t="s">
+        <v>5829</v>
+      </c>
+      <c r="J1199" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1199" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1199" t="s">
+        <v>5830</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1200">
+        <v>1203</v>
+      </c>
+      <c r="B1200" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1200" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1200" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1200" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1200" t="s">
+        <v>5831</v>
+      </c>
+      <c r="G1200" t="s">
+        <v>5832</v>
+      </c>
+      <c r="H1200" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1200" t="s">
+        <v>5833</v>
+      </c>
+      <c r="J1200" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1200" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1200" t="s">
+        <v>5834</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1201">
+        <v>1204</v>
+      </c>
+      <c r="B1201" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1201" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1201" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1201" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1201" t="s">
+        <v>5835</v>
+      </c>
+      <c r="G1201" t="s">
+        <v>5836</v>
+      </c>
+      <c r="H1201" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1201" t="s">
+        <v>5837</v>
+      </c>
+      <c r="J1201" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1201" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1201" t="s">
+        <v>5838</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1202">
+        <v>1205</v>
+      </c>
+      <c r="B1202" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1202" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1202" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1202" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1202" t="s">
+        <v>5839</v>
+      </c>
+      <c r="G1202" t="s">
+        <v>5840</v>
+      </c>
+      <c r="H1202" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1202" t="s">
+        <v>5841</v>
+      </c>
+      <c r="J1202" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1202" t="s">
+        <v>5842</v>
+      </c>
+      <c r="L1202" t="s">
+        <v>5843</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1203">
+        <v>1206</v>
+      </c>
+      <c r="B1203" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1203" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1203" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1203" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1203" t="s">
+        <v>5844</v>
+      </c>
+      <c r="G1203" t="s">
+        <v>5845</v>
+      </c>
+      <c r="H1203" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1203" t="s">
+        <v>5841</v>
+      </c>
+      <c r="J1203" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1203" t="s">
+        <v>5846</v>
+      </c>
+      <c r="L1203" t="s">
+        <v>5847</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1204">
+        <v>1207</v>
+      </c>
+      <c r="B1204" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1204" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1204" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1204" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1204" t="s">
+        <v>5848</v>
+      </c>
+      <c r="G1204" t="s">
+        <v>5849</v>
+      </c>
+      <c r="H1204" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1204" t="s">
+        <v>5850</v>
+      </c>
+      <c r="J1204" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1204" t="s">
+        <v>5851</v>
+      </c>
+      <c r="L1204" t="s">
+        <v>5852</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1205">
+        <v>1208</v>
+      </c>
+      <c r="B1205" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1205" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1205" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1205" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1205" t="s">
+        <v>5853</v>
+      </c>
+      <c r="G1205" t="s">
+        <v>5854</v>
+      </c>
+      <c r="H1205" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1205" t="s">
+        <v>1970</v>
+      </c>
+      <c r="J1205" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1205" t="s">
+        <v>5855</v>
+      </c>
+      <c r="L1205" t="s">
+        <v>5856</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1206">
+        <v>1209</v>
+      </c>
+      <c r="B1206" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1206" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1206" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1206" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1206" t="s">
+        <v>5857</v>
+      </c>
+      <c r="G1206" t="s">
+        <v>5858</v>
+      </c>
+      <c r="H1206" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1206" t="s">
+        <v>5859</v>
+      </c>
+      <c r="J1206" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1206" t="s">
+        <v>5860</v>
+      </c>
+      <c r="L1206" t="s">
+        <v>5861</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1207">
+        <v>1210</v>
+      </c>
+      <c r="B1207" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1207" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1207" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1207" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1207" t="s">
+        <v>5862</v>
+      </c>
+      <c r="G1207" t="s">
+        <v>5863</v>
+      </c>
+      <c r="H1207" t="s">
+        <v>522</v>
+      </c>
+      <c r="I1207" t="s">
+        <v>5864</v>
+      </c>
+      <c r="J1207" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1207" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1207" t="s">
+        <v>5865</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1208">
+        <v>1211</v>
+      </c>
+      <c r="B1208" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1208" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1208" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1208" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1208" t="s">
+        <v>5866</v>
+      </c>
+      <c r="G1208" t="s">
+        <v>5867</v>
+      </c>
+      <c r="H1208" t="s">
+        <v>1764</v>
+      </c>
+      <c r="I1208" t="s">
+        <v>2401</v>
+      </c>
+      <c r="J1208" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1208" t="s">
+        <v>5868</v>
+      </c>
+      <c r="L1208" t="s">
+        <v>5869</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1209">
+        <v>1212</v>
+      </c>
+      <c r="B1209" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1209" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1209" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1209" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1209" t="s">
+        <v>5870</v>
+      </c>
+      <c r="G1209" t="s">
+        <v>5871</v>
+      </c>
+      <c r="H1209" t="s">
+        <v>1764</v>
+      </c>
+      <c r="I1209" t="s">
+        <v>1970</v>
+      </c>
+      <c r="J1209" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1209" t="s">
+        <v>5872</v>
+      </c>
+      <c r="L1209" t="s">
+        <v>5873</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1210">
+        <v>1213</v>
+      </c>
+      <c r="B1210" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1210" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1210" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1210" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1210" t="s">
+        <v>5874</v>
+      </c>
+      <c r="G1210" t="s">
+        <v>5875</v>
+      </c>
+      <c r="H1210" t="s">
+        <v>1764</v>
+      </c>
+      <c r="I1210" t="s">
+        <v>5876</v>
+      </c>
+      <c r="J1210" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1210" t="s">
+        <v>5877</v>
+      </c>
+      <c r="L1210" t="s">
+        <v>5878</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1211">
+        <v>1214</v>
+      </c>
+      <c r="B1211" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1211" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1211" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1211" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1211" t="s">
+        <v>5879</v>
+      </c>
+      <c r="G1211" t="s">
+        <v>5880</v>
+      </c>
+      <c r="H1211" t="s">
+        <v>390</v>
+      </c>
+      <c r="I1211" t="s">
+        <v>2401</v>
+      </c>
+      <c r="J1211" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1211" t="s">
+        <v>5881</v>
+      </c>
+      <c r="L1211" t="s">
+        <v>5882</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1212">
+        <v>1215</v>
+      </c>
+      <c r="B1212" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1212" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1212" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1212" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1212" t="s">
+        <v>5883</v>
+      </c>
+      <c r="G1212" t="s">
+        <v>5884</v>
+      </c>
+      <c r="H1212" t="s">
+        <v>390</v>
+      </c>
+      <c r="I1212" t="s">
+        <v>5774</v>
+      </c>
+      <c r="J1212" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1212" t="s">
+        <v>5885</v>
+      </c>
+      <c r="L1212" t="s">
+        <v>5886</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1213">
+        <v>1216</v>
+      </c>
+      <c r="B1213" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1213" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1213" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1213" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1213" t="s">
+        <v>5887</v>
+      </c>
+      <c r="G1213" t="s">
+        <v>5888</v>
+      </c>
+      <c r="H1213" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1213" t="s">
+        <v>5889</v>
+      </c>
+      <c r="J1213" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1213" t="s">
+        <v>5890</v>
+      </c>
+      <c r="L1213" t="s">
+        <v>5891</v>
+      </c>
+    </row>
+    <row r="1214" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1214">
+        <v>1217</v>
+      </c>
+      <c r="B1214" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1214" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1214" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1214" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1214" t="s">
+        <v>5892</v>
+      </c>
+      <c r="G1214" t="s">
+        <v>5893</v>
+      </c>
+      <c r="H1214" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1214" t="s">
+        <v>5894</v>
+      </c>
+      <c r="J1214" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1214" t="s">
+        <v>5895</v>
+      </c>
+      <c r="L1214" t="s">
+        <v>5896</v>
+      </c>
+    </row>
+    <row r="1215" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1215">
+        <v>1218</v>
+      </c>
+      <c r="B1215" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1215" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1215" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1215" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1215" t="s">
+        <v>5897</v>
+      </c>
+      <c r="G1215" t="s">
+        <v>5898</v>
+      </c>
+      <c r="H1215" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1215" t="s">
+        <v>1945</v>
+      </c>
+      <c r="J1215" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1215" t="s">
+        <v>5899</v>
+      </c>
+      <c r="L1215" t="s">
+        <v>5900</v>
+      </c>
+    </row>
+    <row r="1216" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1216">
+        <v>1219</v>
+      </c>
+      <c r="B1216" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1216" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1216" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1216" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1216" t="s">
+        <v>5901</v>
+      </c>
+      <c r="G1216" t="s">
+        <v>5902</v>
+      </c>
+      <c r="H1216" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1216" t="s">
+        <v>5903</v>
+      </c>
+      <c r="J1216" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1216" t="s">
+        <v>5904</v>
+      </c>
+      <c r="L1216" t="s">
+        <v>5905</v>
+      </c>
+    </row>
+    <row r="1217" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1217">
+        <v>1220</v>
+      </c>
+      <c r="B1217" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1217" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1217" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1217" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1217" t="s">
+        <v>5906</v>
+      </c>
+      <c r="G1217" t="s">
+        <v>5907</v>
+      </c>
+      <c r="H1217" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1217" t="s">
+        <v>5908</v>
+      </c>
+      <c r="J1217" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1217" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1217" t="s">
+        <v>5909</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 9 WebKreatives OSM leads
</commit_message>
<xml_diff>
--- a/leads/Leads.xlsx
+++ b/leads/Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10659" uniqueCount="5910">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10758" uniqueCount="5943">
   <si>
     <t>#</t>
   </si>
@@ -17741,6 +17741,105 @@
   </si>
   <si>
     <t>Website available | Email from website | OSM id:4959131889 | Source: OpenStreetMap | bloemist | Enschede | Website: https://www.bloemsierkunstmimosa.nl</t>
+  </si>
+  <si>
+    <t>dtbntilburg@gmail.com</t>
+  </si>
+  <si>
+    <t>De Tandenbleker</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2851160937 | Source: OpenStreetMap | schoonheidssalon | Tilburg | Website: https://detandenblekertilburg.nl</t>
+  </si>
+  <si>
+    <t>tattooshoponi@gmail.com</t>
+  </si>
+  <si>
+    <t>Oni Tattoo</t>
+  </si>
+  <si>
+    <t>Gondelstraat 5017CK</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2850735168 | Source: OpenStreetMap | tattooshop | Tilburg | Website: https://onitattoo.nl</t>
+  </si>
+  <si>
+    <t>info@almabroodlab.nl</t>
+  </si>
+  <si>
+    <t>Alma Broodlab</t>
+  </si>
+  <si>
+    <t>+31 13 542 4993</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2850736827 | Source: OpenStreetMap | bakkerij | Tilburg | Website: https://almabroodlab.nl</t>
+  </si>
+  <si>
+    <t>info@medinillabloemsierkunst.nl</t>
+  </si>
+  <si>
+    <t>Medinilla</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2847044895 | Source: OpenStreetMap | bloemist | Tilburg | Website: https://medinillabloemsierkunst.nl</t>
+  </si>
+  <si>
+    <t>info@allurebloemenenplanten.nl</t>
+  </si>
+  <si>
+    <t>Allure</t>
+  </si>
+  <si>
+    <t>Heyhoefpromenade 5043RB</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2848244488 | Source: OpenStreetMap | bloemist | Tilburg | Website: https://allurebloemenenplanten.nl</t>
+  </si>
+  <si>
+    <t>info@all-aboutflowers.nl</t>
+  </si>
+  <si>
+    <t>All About Flowers</t>
+  </si>
+  <si>
+    <t>Vredeman de Vriesstraat 5041GR</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2850123322 | Source: OpenStreetMap | bloemist | Tilburg | Website: https://www.all-aboutflowers.nl</t>
+  </si>
+  <si>
+    <t>winkel@cocoontilburg.nl</t>
+  </si>
+  <si>
+    <t>Cocoon</t>
+  </si>
+  <si>
+    <t>Wilhelminapark 5041EC</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2850941577 | Source: OpenStreetMap | bloemist | Tilburg | Website: https://cocoontilburg.nl</t>
+  </si>
+  <si>
+    <t>flowerwisestudio@gmail.com</t>
+  </si>
+  <si>
+    <t>Flowerwise</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:12878823503 | Source: OpenStreetMap | bloemist | Tilburg | Website: https://www.flowerwise.nl</t>
+  </si>
+  <si>
+    <t>info@wassjop.com</t>
+  </si>
+  <si>
+    <t>Wassjop</t>
+  </si>
+  <si>
+    <t>Molenstraat 5014NA</t>
+  </si>
+  <si>
+    <t>Website available | Email from website | OSM id:2848977068 | Source: OpenStreetMap | wasserette | Tilburg | Website: https://wassjop.com</t>
   </si>
 </sst>
 </file>
@@ -18117,7 +18216,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1217"/>
+  <dimension ref="A1:L1226"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -56182,6 +56281,348 @@
         <v>5909</v>
       </c>
     </row>
+    <row r="1218" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1218">
+        <v>1221</v>
+      </c>
+      <c r="B1218" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1218" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1218" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1218" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1218" t="s">
+        <v>5910</v>
+      </c>
+      <c r="G1218" t="s">
+        <v>5911</v>
+      </c>
+      <c r="H1218" t="s">
+        <v>343</v>
+      </c>
+      <c r="I1218" t="s">
+        <v>3480</v>
+      </c>
+      <c r="J1218" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1218" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1218" t="s">
+        <v>5912</v>
+      </c>
+    </row>
+    <row r="1219" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1219">
+        <v>1222</v>
+      </c>
+      <c r="B1219" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1219" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1219" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1219" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1219" t="s">
+        <v>5913</v>
+      </c>
+      <c r="G1219" t="s">
+        <v>5914</v>
+      </c>
+      <c r="H1219" t="s">
+        <v>1975</v>
+      </c>
+      <c r="I1219" t="s">
+        <v>5915</v>
+      </c>
+      <c r="J1219" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1219" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1219" t="s">
+        <v>5916</v>
+      </c>
+    </row>
+    <row r="1220" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1220">
+        <v>1223</v>
+      </c>
+      <c r="B1220" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1220" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1220" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1220" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1220" t="s">
+        <v>5917</v>
+      </c>
+      <c r="G1220" t="s">
+        <v>5918</v>
+      </c>
+      <c r="H1220" t="s">
+        <v>390</v>
+      </c>
+      <c r="I1220" t="s">
+        <v>3421</v>
+      </c>
+      <c r="J1220" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1220" t="s">
+        <v>5919</v>
+      </c>
+      <c r="L1220" t="s">
+        <v>5920</v>
+      </c>
+    </row>
+    <row r="1221" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1221">
+        <v>1224</v>
+      </c>
+      <c r="B1221" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1221" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1221" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1221" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1221" t="s">
+        <v>5921</v>
+      </c>
+      <c r="G1221" t="s">
+        <v>5922</v>
+      </c>
+      <c r="H1221" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1221" t="s">
+        <v>3599</v>
+      </c>
+      <c r="J1221" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1221" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1221" t="s">
+        <v>5923</v>
+      </c>
+    </row>
+    <row r="1222" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1222">
+        <v>1225</v>
+      </c>
+      <c r="B1222" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1222" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1222" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1222" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1222" t="s">
+        <v>5924</v>
+      </c>
+      <c r="G1222" t="s">
+        <v>5925</v>
+      </c>
+      <c r="H1222" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1222" t="s">
+        <v>5926</v>
+      </c>
+      <c r="J1222" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1222" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1222" t="s">
+        <v>5927</v>
+      </c>
+    </row>
+    <row r="1223" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1223">
+        <v>1226</v>
+      </c>
+      <c r="B1223" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1223" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1223" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1223" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1223" t="s">
+        <v>5928</v>
+      </c>
+      <c r="G1223" t="s">
+        <v>5929</v>
+      </c>
+      <c r="H1223" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1223" t="s">
+        <v>5930</v>
+      </c>
+      <c r="J1223" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1223" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1223" t="s">
+        <v>5931</v>
+      </c>
+    </row>
+    <row r="1224" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1224">
+        <v>1227</v>
+      </c>
+      <c r="B1224" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1224" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1224" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1224" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1224" t="s">
+        <v>5932</v>
+      </c>
+      <c r="G1224" t="s">
+        <v>5933</v>
+      </c>
+      <c r="H1224" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1224" t="s">
+        <v>5934</v>
+      </c>
+      <c r="J1224" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1224" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1224" t="s">
+        <v>5935</v>
+      </c>
+    </row>
+    <row r="1225" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1225">
+        <v>1228</v>
+      </c>
+      <c r="B1225" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1225" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1225" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1225" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1225" t="s">
+        <v>5936</v>
+      </c>
+      <c r="G1225" t="s">
+        <v>5937</v>
+      </c>
+      <c r="H1225" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1225" t="s">
+        <v>5559</v>
+      </c>
+      <c r="J1225" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1225" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1225" t="s">
+        <v>5938</v>
+      </c>
+    </row>
+    <row r="1226" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1226">
+        <v>1229</v>
+      </c>
+      <c r="B1226" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1226" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1226" t="s">
+        <v>5559</v>
+      </c>
+      <c r="E1226" t="s">
+        <v>5559</v>
+      </c>
+      <c r="F1226" t="s">
+        <v>5939</v>
+      </c>
+      <c r="G1226" t="s">
+        <v>5940</v>
+      </c>
+      <c r="H1226" t="s">
+        <v>1895</v>
+      </c>
+      <c r="I1226" t="s">
+        <v>5941</v>
+      </c>
+      <c r="J1226" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1226" t="s">
+        <v>5559</v>
+      </c>
+      <c r="L1226" t="s">
+        <v>5942</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>